<commit_message>
chore(data): update inventory data to 23:25
</commit_message>
<xml_diff>
--- a/BaoCao_TonKho.xlsx
+++ b/BaoCao_TonKho.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>04/06/2026 12:50:55</t>
+          <t>04/06/2026 23:36:16</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -579,25 +579,25 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4825</v>
+        <v>6197</v>
       </c>
       <c r="C7" t="n">
-        <v>182</v>
+        <v>114</v>
       </c>
       <c r="D7" t="n">
-        <v>144</v>
+        <v>30</v>
       </c>
       <c r="E7" t="n">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="F7" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G7" t="n">
         <v>6</v>
       </c>
       <c r="H7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -606,7 +606,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>5189</v>
+        <v>6391</v>
       </c>
     </row>
     <row r="8">
@@ -616,26 +616,28 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>490</v>
+        <v>1438</v>
       </c>
       <c r="C8" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="D8" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E8" t="n">
-        <v>6</v>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8" t="inlineStr"/>
+        <v>9</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="n">
+        <v>1</v>
+      </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="n">
-        <v>512</v>
+        <v>1479</v>
       </c>
     </row>
     <row r="9">
@@ -645,20 +647,18 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>599</v>
+        <v>848</v>
       </c>
       <c r="C9" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="D9" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="E9" t="n">
-        <v>2</v>
-      </c>
-      <c r="F9" t="n">
-        <v>6</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
         <v>2</v>
       </c>
@@ -666,7 +666,7 @@
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="n">
-        <v>634</v>
+        <v>883</v>
       </c>
     </row>
     <row r="10">
@@ -676,22 +676,24 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>846</v>
+        <v>774</v>
       </c>
       <c r="C10" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="D10" t="n">
-        <v>10</v>
-      </c>
-      <c r="E10" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="n">
-        <v>880</v>
+        <v>813</v>
       </c>
     </row>
     <row r="11">
@@ -701,16 +703,16 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>419</v>
+        <v>495</v>
       </c>
       <c r="C11" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
@@ -718,7 +720,7 @@
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="n">
-        <v>430</v>
+        <v>507</v>
       </c>
     </row>
     <row r="12">
@@ -728,16 +730,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>350</v>
+        <v>319</v>
       </c>
       <c r="C12" t="n">
-        <v>95</v>
+        <v>8</v>
       </c>
       <c r="D12" t="n">
-        <v>60</v>
+        <v>2</v>
       </c>
       <c r="E12" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
@@ -745,7 +747,7 @@
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="n">
-        <v>510</v>
+        <v>331</v>
       </c>
     </row>
     <row r="13">
@@ -755,22 +757,22 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2121</v>
+        <v>2323</v>
       </c>
       <c r="C13" t="n">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="D13" t="n">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="E13" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="F13" t="n">
         <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H13" t="n">
         <v>2</v>
@@ -778,7 +780,7 @@
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="n">
-        <v>2223</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="14">
@@ -788,16 +790,16 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>476</v>
+        <v>1340</v>
       </c>
       <c r="C14" t="n">
-        <v>21</v>
+        <v>177</v>
       </c>
       <c r="D14" t="n">
         <v>10</v>
       </c>
       <c r="E14" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F14" t="n">
         <v>1</v>
@@ -815,7 +817,7 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>524</v>
+        <v>1545</v>
       </c>
     </row>
     <row r="15">
@@ -825,10 +827,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>31</v>
+        <v>64</v>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="D15" t="n">
         <v>1</v>
@@ -840,7 +842,7 @@
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="n">
-        <v>33</v>
+        <v>79</v>
       </c>
     </row>
     <row r="16">
@@ -850,9 +852,11 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>38</v>
-      </c>
-      <c r="C16" t="inlineStr"/>
+        <v>123</v>
+      </c>
+      <c r="C16" t="n">
+        <v>8</v>
+      </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
         <v>1</v>
@@ -863,7 +867,7 @@
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="n">
-        <v>39</v>
+        <v>132</v>
       </c>
     </row>
     <row r="17">
@@ -873,9 +877,11 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>7</v>
-      </c>
-      <c r="C17" t="inlineStr"/>
+        <v>21</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
         <v>1</v>
@@ -886,7 +892,7 @@
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="n">
-        <v>8</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18">
@@ -896,10 +902,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="C18" t="n">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="D18" t="n">
         <v>1</v>
@@ -911,7 +917,7 @@
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="n">
-        <v>65</v>
+        <v>105</v>
       </c>
     </row>
     <row r="19">
@@ -921,13 +927,15 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>28</v>
-      </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" t="inlineStr"/>
+        <v>81</v>
+      </c>
+      <c r="C19" t="n">
+        <v>11</v>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
       <c r="F19" t="n">
         <v>1</v>
       </c>
@@ -938,7 +946,7 @@
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="n">
-        <v>31</v>
+        <v>95</v>
       </c>
     </row>
     <row r="20">
@@ -948,10 +956,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>44</v>
+        <v>101</v>
       </c>
       <c r="C20" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
@@ -963,7 +971,7 @@
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="n">
-        <v>46</v>
+        <v>117</v>
       </c>
     </row>
     <row r="21">
@@ -973,10 +981,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
@@ -988,7 +996,7 @@
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="n">
-        <v>25</v>
+        <v>63</v>
       </c>
     </row>
     <row r="22">
@@ -998,10 +1006,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>38</v>
+        <v>82</v>
       </c>
       <c r="C22" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="D22" t="n">
         <v>1</v>
@@ -1015,7 +1023,7 @@
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="n">
-        <v>49</v>
+        <v>108</v>
       </c>
     </row>
     <row r="23">
@@ -1025,9 +1033,11 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>15</v>
-      </c>
-      <c r="C23" t="inlineStr"/>
+        <v>56</v>
+      </c>
+      <c r="C23" t="n">
+        <v>6</v>
+      </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="n">
         <v>1</v>
@@ -1038,7 +1048,7 @@
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="n">
-        <v>16</v>
+        <v>63</v>
       </c>
     </row>
     <row r="24">
@@ -1048,9 +1058,11 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>48</v>
-      </c>
-      <c r="C24" t="inlineStr"/>
+        <v>143</v>
+      </c>
+      <c r="C24" t="n">
+        <v>9</v>
+      </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
@@ -1059,7 +1071,7 @@
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="n">
-        <v>48</v>
+        <v>152</v>
       </c>
     </row>
     <row r="25">
@@ -1069,9 +1081,11 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>33</v>
-      </c>
-      <c r="C25" t="inlineStr"/>
+        <v>97</v>
+      </c>
+      <c r="C25" t="n">
+        <v>3</v>
+      </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
@@ -1080,7 +1094,7 @@
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="n">
-        <v>33</v>
+        <v>100</v>
       </c>
     </row>
     <row r="26">
@@ -1090,12 +1104,14 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>70</v>
+        <v>179</v>
       </c>
       <c r="C26" t="n">
-        <v>2</v>
-      </c>
-      <c r="D26" t="inlineStr"/>
+        <v>17</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
       <c r="E26" t="n">
         <v>1</v>
       </c>
@@ -1105,7 +1121,7 @@
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="n">
-        <v>73</v>
+        <v>198</v>
       </c>
     </row>
     <row r="27">
@@ -1115,10 +1131,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>29</v>
+        <v>225</v>
       </c>
       <c r="C27" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D27" t="n">
         <v>6</v>
@@ -1134,7 +1150,7 @@
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="n">
-        <v>45</v>
+        <v>245</v>
       </c>
     </row>
     <row r="28">
@@ -1144,9 +1160,11 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>12</v>
-      </c>
-      <c r="C28" t="inlineStr"/>
+        <v>60</v>
+      </c>
+      <c r="C28" t="n">
+        <v>4</v>
+      </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="n">
         <v>1</v>
@@ -1157,7 +1175,7 @@
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="n">
-        <v>13</v>
+        <v>65</v>
       </c>
     </row>
     <row r="29">
@@ -1167,16 +1185,16 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>233</v>
+        <v>83</v>
       </c>
       <c r="C29" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="D29" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="E29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F29" t="n">
         <v>0</v>
@@ -1194,7 +1212,7 @@
         <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>255</v>
+        <v>109</v>
       </c>
     </row>
     <row r="30">
@@ -1204,16 +1222,16 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>233</v>
+        <v>83</v>
       </c>
       <c r="C30" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="D30" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="E30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr"/>
@@ -1223,7 +1241,7 @@
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="n">
-        <v>255</v>
+        <v>109</v>
       </c>
     </row>
     <row r="31">
@@ -1233,22 +1251,22 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>17668</v>
+        <v>25718</v>
       </c>
       <c r="C31" t="n">
-        <v>744</v>
+        <v>266</v>
       </c>
       <c r="D31" t="n">
-        <v>374</v>
+        <v>120</v>
       </c>
       <c r="E31" t="n">
-        <v>89</v>
+        <v>133</v>
       </c>
       <c r="F31" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G31" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="H31" t="n">
         <v>5</v>
@@ -1260,7 +1278,7 @@
         <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>18915</v>
+        <v>26279</v>
       </c>
     </row>
     <row r="32">
@@ -1270,16 +1288,16 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>569</v>
+        <v>1686</v>
       </c>
       <c r="C32" t="n">
-        <v>7</v>
+        <v>38</v>
       </c>
       <c r="D32" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E32" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F32" t="n">
         <v>1</v>
@@ -1291,7 +1309,7 @@
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="n">
-        <v>590</v>
+        <v>1738</v>
       </c>
     </row>
     <row r="33">
@@ -1301,26 +1319,28 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>349</v>
+        <v>509</v>
       </c>
       <c r="C33" t="n">
         <v>5</v>
       </c>
       <c r="D33" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E33" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="n">
-        <v>2</v>
-      </c>
-      <c r="H33" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H33" t="n">
+        <v>1</v>
+      </c>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="n">
-        <v>373</v>
+        <v>530</v>
       </c>
     </row>
     <row r="34">
@@ -1330,28 +1350,28 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>5408</v>
+        <v>3204</v>
       </c>
       <c r="C34" t="n">
-        <v>68</v>
+        <v>31</v>
       </c>
       <c r="D34" t="n">
-        <v>71</v>
+        <v>27</v>
       </c>
       <c r="E34" t="n">
         <v>24</v>
       </c>
-      <c r="F34" t="inlineStr"/>
+      <c r="F34" t="n">
+        <v>5</v>
+      </c>
       <c r="G34" t="n">
         <v>12</v>
       </c>
-      <c r="H34" t="n">
-        <v>1</v>
-      </c>
+      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="n">
-        <v>5584</v>
+        <v>3303</v>
       </c>
     </row>
     <row r="35">
@@ -1361,28 +1381,28 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>427</v>
+        <v>782</v>
       </c>
       <c r="C35" t="n">
+        <v>12</v>
+      </c>
+      <c r="D35" t="n">
+        <v>14</v>
+      </c>
+      <c r="E35" t="n">
         <v>15</v>
-      </c>
-      <c r="D35" t="n">
-        <v>19</v>
-      </c>
-      <c r="E35" t="n">
-        <v>7</v>
       </c>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="n">
         <v>2</v>
       </c>
       <c r="H35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="n">
-        <v>473</v>
+        <v>827</v>
       </c>
     </row>
     <row r="36">
@@ -1392,26 +1412,28 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1092</v>
+        <v>714</v>
       </c>
       <c r="C36" t="n">
-        <v>267</v>
+        <v>9</v>
       </c>
       <c r="D36" t="n">
-        <v>108</v>
+        <v>3</v>
       </c>
       <c r="E36" t="n">
         <v>8</v>
       </c>
       <c r="F36" t="n">
-        <v>2</v>
-      </c>
-      <c r="G36" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G36" t="n">
+        <v>1</v>
+      </c>
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="n">
-        <v>1477</v>
+        <v>736</v>
       </c>
     </row>
     <row r="37">
@@ -1421,16 +1443,16 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>2573</v>
+        <v>4346</v>
       </c>
       <c r="C37" t="n">
-        <v>94</v>
+        <v>19</v>
       </c>
       <c r="D37" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E37" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="n">
@@ -1442,7 +1464,7 @@
       </c>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="n">
-        <v>2691</v>
+        <v>4396</v>
       </c>
     </row>
     <row r="38">
@@ -1452,18 +1474,20 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>3043</v>
+        <v>6645</v>
       </c>
       <c r="C38" t="n">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="D38" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E38" t="n">
-        <v>13</v>
-      </c>
-      <c r="F38" t="inlineStr"/>
+        <v>17</v>
+      </c>
+      <c r="F38" t="n">
+        <v>3</v>
+      </c>
       <c r="G38" t="n">
         <v>2</v>
       </c>
@@ -1471,7 +1495,7 @@
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="n">
-        <v>3122</v>
+        <v>6734</v>
       </c>
     </row>
     <row r="39">
@@ -1481,28 +1505,30 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>762</v>
+        <v>1629</v>
       </c>
       <c r="C39" t="n">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="D39" t="n">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="E39" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F39" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G39" t="n">
-        <v>2</v>
-      </c>
-      <c r="H39" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H39" t="n">
+        <v>1</v>
+      </c>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="n">
-        <v>850</v>
+        <v>1698</v>
       </c>
     </row>
     <row r="40">
@@ -1512,16 +1538,16 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>783</v>
+        <v>2081</v>
       </c>
       <c r="C40" t="n">
+        <v>14</v>
+      </c>
+      <c r="D40" t="n">
         <v>7</v>
       </c>
-      <c r="D40" t="n">
-        <v>15</v>
-      </c>
       <c r="E40" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="n">
@@ -1531,7 +1557,7 @@
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="n">
-        <v>811</v>
+        <v>2113</v>
       </c>
     </row>
     <row r="41">
@@ -1541,13 +1567,13 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>780</v>
+        <v>645</v>
       </c>
       <c r="C41" t="n">
-        <v>137</v>
+        <v>6</v>
       </c>
       <c r="D41" t="n">
-        <v>55</v>
+        <v>5</v>
       </c>
       <c r="E41" t="n">
         <v>5</v>
@@ -1560,7 +1586,7 @@
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="n">
-        <v>978</v>
+        <v>662</v>
       </c>
     </row>
     <row r="42">
@@ -1570,16 +1596,16 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1208</v>
+        <v>2395</v>
       </c>
       <c r="C42" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D42" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="E42" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr"/>
@@ -1587,7 +1613,7 @@
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="n">
-        <v>1241</v>
+        <v>2421</v>
       </c>
     </row>
     <row r="43">
@@ -1597,28 +1623,26 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>674</v>
+        <v>1082</v>
       </c>
       <c r="C43" t="n">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="D43" t="n">
         <v>8</v>
       </c>
       <c r="E43" t="n">
-        <v>4</v>
-      </c>
-      <c r="F43" t="n">
-        <v>1</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="F43" t="inlineStr"/>
       <c r="G43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="n">
-        <v>725</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="44">
@@ -1628,25 +1652,25 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>2728</v>
+        <v>2645</v>
       </c>
       <c r="C44" t="n">
-        <v>1831</v>
+        <v>1903</v>
       </c>
       <c r="D44" t="n">
-        <v>279</v>
+        <v>901</v>
       </c>
       <c r="E44" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="F44" t="n">
         <v>2</v>
       </c>
       <c r="G44" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H44" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I44" t="n">
         <v>1</v>
@@ -1655,7 +1679,7 @@
         <v>0</v>
       </c>
       <c r="K44" t="n">
-        <v>4859</v>
+        <v>5477</v>
       </c>
     </row>
     <row r="45">
@@ -1665,30 +1689,32 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>2728</v>
+        <v>2645</v>
       </c>
       <c r="C45" t="n">
-        <v>1831</v>
+        <v>1903</v>
       </c>
       <c r="D45" t="n">
-        <v>279</v>
+        <v>901</v>
       </c>
       <c r="E45" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="F45" t="n">
         <v>2</v>
       </c>
       <c r="G45" t="n">
-        <v>7</v>
-      </c>
-      <c r="H45" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="H45" t="n">
+        <v>3</v>
+      </c>
       <c r="I45" t="n">
         <v>1</v>
       </c>
       <c r="J45" t="inlineStr"/>
       <c r="K45" t="n">
-        <v>4859</v>
+        <v>5477</v>
       </c>
     </row>
     <row r="46">
@@ -1698,25 +1724,25 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>11827</v>
+        <v>19217</v>
       </c>
       <c r="C46" t="n">
-        <v>303</v>
+        <v>2828</v>
       </c>
       <c r="D46" t="n">
-        <v>84</v>
+        <v>140</v>
       </c>
       <c r="E46" t="n">
-        <v>62</v>
+        <v>83</v>
       </c>
       <c r="F46" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="G46" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H46" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I46" t="n">
         <v>0</v>
@@ -1725,7 +1751,7 @@
         <v>0</v>
       </c>
       <c r="K46" t="n">
-        <v>12303</v>
+        <v>22296</v>
       </c>
     </row>
     <row r="47">
@@ -1735,28 +1761,28 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>3682</v>
+        <v>5375</v>
       </c>
       <c r="C47" t="n">
-        <v>71</v>
+        <v>808</v>
       </c>
       <c r="D47" t="n">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="E47" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F47" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G47" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="n">
-        <v>3790</v>
+        <v>6242</v>
       </c>
     </row>
     <row r="48">
@@ -1766,19 +1792,19 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1528</v>
+        <v>2530</v>
       </c>
       <c r="C48" t="n">
-        <v>31</v>
+        <v>451</v>
       </c>
       <c r="D48" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E48" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F48" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G48" t="n">
         <v>3</v>
@@ -1787,7 +1813,7 @@
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="n">
-        <v>1588</v>
+        <v>3022</v>
       </c>
     </row>
     <row r="49">
@@ -1797,22 +1823,22 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>2945</v>
+        <v>5067</v>
       </c>
       <c r="C49" t="n">
-        <v>75</v>
+        <v>637</v>
       </c>
       <c r="D49" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="E49" t="n">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="F49" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G49" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H49" t="n">
         <v>2</v>
@@ -1820,7 +1846,7 @@
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="n">
-        <v>3063</v>
+        <v>5763</v>
       </c>
     </row>
     <row r="50">
@@ -1830,28 +1856,30 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>1662</v>
+        <v>2945</v>
       </c>
       <c r="C50" t="n">
-        <v>90</v>
+        <v>416</v>
       </c>
       <c r="D50" t="n">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="E50" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G50" t="n">
-        <v>3</v>
-      </c>
-      <c r="H50" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="H50" t="n">
+        <v>2</v>
+      </c>
       <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr"/>
       <c r="K50" t="n">
-        <v>1796</v>
+        <v>3424</v>
       </c>
     </row>
     <row r="51">
@@ -1861,18 +1889,20 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>2010</v>
+        <v>3300</v>
       </c>
       <c r="C51" t="n">
-        <v>36</v>
+        <v>516</v>
       </c>
       <c r="D51" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="E51" t="n">
-        <v>13</v>
-      </c>
-      <c r="F51" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="F51" t="n">
+        <v>1</v>
+      </c>
       <c r="G51" t="n">
         <v>2</v>
       </c>
@@ -1880,7 +1910,7 @@
       <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr"/>
       <c r="K51" t="n">
-        <v>2066</v>
+        <v>3845</v>
       </c>
     </row>
     <row r="52">
@@ -1890,16 +1920,16 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>854</v>
+        <v>568</v>
       </c>
       <c r="C52" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="D52" t="n">
         <v>2</v>
       </c>
       <c r="E52" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F52" t="n">
         <v>1</v>
@@ -1917,7 +1947,7 @@
         <v>0</v>
       </c>
       <c r="K52" t="n">
-        <v>877</v>
+        <v>579</v>
       </c>
     </row>
     <row r="53">
@@ -1927,16 +1957,16 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>854</v>
+        <v>568</v>
       </c>
       <c r="C53" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="D53" t="n">
         <v>2</v>
       </c>
       <c r="E53" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F53" t="n">
         <v>1</v>
@@ -1948,7 +1978,7 @@
       <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr"/>
       <c r="K53" t="n">
-        <v>877</v>
+        <v>579</v>
       </c>
     </row>
     <row r="54">
@@ -1958,25 +1988,25 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>38611</v>
+        <v>55768</v>
       </c>
       <c r="C54" t="n">
-        <v>3104</v>
+        <v>5310</v>
       </c>
       <c r="D54" t="n">
-        <v>906</v>
+        <v>1207</v>
       </c>
       <c r="E54" t="n">
-        <v>203</v>
+        <v>295</v>
       </c>
       <c r="F54" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="G54" t="n">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="H54" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="I54" t="n">
         <v>2</v>
@@ -1985,7 +2015,7 @@
         <v>0</v>
       </c>
       <c r="K54" t="n">
-        <v>42922</v>
+        <v>62676</v>
       </c>
     </row>
   </sheetData>
@@ -2061,19 +2091,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1523</v>
+        <v>895</v>
       </c>
       <c r="C2" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D2" t="n">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="E2" t="n">
         <v>5</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G2" t="n">
         <v>2</v>
@@ -2085,7 +2115,7 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>1569</v>
+        <v>920</v>
       </c>
     </row>
     <row r="3">
@@ -2095,22 +2125,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>616</v>
+        <v>574</v>
       </c>
       <c r="C3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D3" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="E3" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F3" t="n">
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -2119,7 +2149,7 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>638</v>
+        <v>592</v>
       </c>
     </row>
     <row r="4">
@@ -2129,22 +2159,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3881</v>
+        <v>5846</v>
       </c>
       <c r="C4" t="n">
-        <v>72</v>
+        <v>824</v>
       </c>
       <c r="D4" t="n">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="E4" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="F4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
@@ -2153,7 +2183,7 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>3994</v>
+        <v>6733</v>
       </c>
     </row>
     <row r="5">
@@ -2163,19 +2193,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>721</v>
+        <v>1282</v>
       </c>
       <c r="C5" t="n">
-        <v>12</v>
+        <v>59</v>
       </c>
       <c r="D5" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
         <v>2</v>
@@ -2187,7 +2217,7 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>758</v>
+        <v>1352</v>
       </c>
     </row>
     <row r="6">
@@ -2197,16 +2227,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>828</v>
+        <v>765</v>
       </c>
       <c r="C6" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="D6" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
@@ -2221,7 +2251,7 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>861</v>
+        <v>803</v>
       </c>
     </row>
     <row r="7">
@@ -2231,31 +2261,31 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>223</v>
+        <v>328</v>
       </c>
       <c r="C7" t="n">
         <v>6</v>
       </c>
       <c r="D7" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>239</v>
+        <v>342</v>
       </c>
     </row>
     <row r="8">
@@ -2265,19 +2295,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>690</v>
+        <v>428</v>
       </c>
       <c r="C8" t="n">
         <v>5</v>
       </c>
       <c r="D8" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" t="n">
         <v>2</v>
@@ -2289,7 +2319,7 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>707</v>
+        <v>439</v>
       </c>
     </row>
     <row r="9">
@@ -2299,10 +2329,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>292</v>
+        <v>376</v>
       </c>
       <c r="C9" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="D9" t="n">
         <v>3</v>
@@ -2323,7 +2353,7 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>298</v>
+        <v>395</v>
       </c>
     </row>
     <row r="10">
@@ -2333,13 +2363,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="C10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -2357,7 +2387,7 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>33</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11">
@@ -2367,16 +2397,16 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>329</v>
+        <v>467</v>
       </c>
       <c r="C11" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
@@ -2391,7 +2421,7 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>338</v>
+        <v>475</v>
       </c>
     </row>
     <row r="12">
@@ -2401,19 +2431,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1539</v>
+        <v>2790</v>
       </c>
       <c r="C12" t="n">
-        <v>30</v>
+        <v>457</v>
       </c>
       <c r="D12" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E12" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F12" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G12" t="n">
         <v>4</v>
@@ -2425,7 +2455,7 @@
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>1601</v>
+        <v>3291</v>
       </c>
     </row>
     <row r="13">
@@ -2435,13 +2465,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>71</v>
+        <v>120</v>
       </c>
       <c r="C13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
@@ -2459,7 +2489,7 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>74</v>
+        <v>126</v>
       </c>
     </row>
     <row r="14">
@@ -2469,31 +2499,31 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>70</v>
+        <v>120</v>
       </c>
       <c r="C14" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>84</v>
+        <v>131</v>
       </c>
     </row>
     <row r="15">
@@ -2503,16 +2533,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="C15" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D15" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F15" t="n">
         <v>0</v>
@@ -2527,7 +2557,7 @@
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="16">
@@ -2537,19 +2567,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>783</v>
+        <v>541</v>
       </c>
       <c r="C16" t="n">
-        <v>198</v>
+        <v>9</v>
       </c>
       <c r="D16" t="n">
-        <v>76</v>
+        <v>3</v>
       </c>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
@@ -2561,7 +2591,7 @@
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>1061</v>
+        <v>557</v>
       </c>
     </row>
     <row r="17">
@@ -2571,10 +2601,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>80</v>
+        <v>141</v>
       </c>
       <c r="C17" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D17" t="n">
         <v>1</v>
@@ -2595,7 +2625,7 @@
         <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>86</v>
+        <v>144</v>
       </c>
     </row>
     <row r="18">
@@ -2605,10 +2635,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>127</v>
+        <v>336</v>
       </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
@@ -2629,7 +2659,7 @@
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>129</v>
+        <v>343</v>
       </c>
     </row>
     <row r="19">
@@ -2639,16 +2669,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1625</v>
+        <v>2723</v>
       </c>
       <c r="C19" t="n">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="D19" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E19" t="n">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
@@ -2657,13 +2687,13 @@
         <v>2</v>
       </c>
       <c r="H19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I19" t="n">
         <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>1710</v>
+        <v>2788</v>
       </c>
     </row>
     <row r="20">
@@ -2673,16 +2703,16 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>183</v>
+        <v>585</v>
       </c>
       <c r="C20" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D20" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F20" t="n">
         <v>1</v>
@@ -2697,7 +2727,7 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>191</v>
+        <v>600</v>
       </c>
     </row>
     <row r="21">
@@ -2707,16 +2737,16 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>124</v>
+        <v>179</v>
       </c>
       <c r="C21" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D21" t="n">
         <v>2</v>
       </c>
       <c r="E21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
@@ -2731,7 +2761,7 @@
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>132</v>
+        <v>183</v>
       </c>
     </row>
     <row r="22">
@@ -2741,13 +2771,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>232</v>
+        <v>483</v>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D22" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E22" t="n">
         <v>1</v>
@@ -2765,7 +2795,7 @@
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>239</v>
+        <v>500</v>
       </c>
     </row>
     <row r="23">
@@ -2775,14 +2805,14 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>246</v>
+        <v>649</v>
       </c>
       <c r="C23" t="n">
+        <v>9</v>
+      </c>
+      <c r="D23" t="n">
         <v>3</v>
       </c>
-      <c r="D23" t="n">
-        <v>2</v>
-      </c>
       <c r="E23" t="n">
         <v>0</v>
       </c>
@@ -2799,7 +2829,7 @@
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>251</v>
+        <v>661</v>
       </c>
     </row>
     <row r="24">
@@ -2809,19 +2839,19 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>462</v>
+        <v>811</v>
       </c>
       <c r="C24" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="D24" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
@@ -2833,7 +2863,7 @@
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>484</v>
+        <v>844</v>
       </c>
     </row>
     <row r="25">
@@ -2843,19 +2873,19 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="C25" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D25" t="n">
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G25" t="n">
         <v>0</v>
@@ -2867,7 +2897,7 @@
         <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>97</v>
+        <v>85</v>
       </c>
     </row>
     <row r="26">
@@ -2877,31 +2907,31 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>3409</v>
+        <v>4030</v>
       </c>
       <c r="C26" t="n">
-        <v>1829</v>
+        <v>1909</v>
       </c>
       <c r="D26" t="n">
-        <v>271</v>
+        <v>861</v>
       </c>
       <c r="E26" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="F26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" t="n">
         <v>3</v>
       </c>
-      <c r="G26" t="n">
-        <v>7</v>
-      </c>
       <c r="H26" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I26" t="n">
         <v>1</v>
       </c>
       <c r="J26" t="n">
-        <v>5540</v>
+        <v>6835</v>
       </c>
     </row>
     <row r="27">
@@ -2911,16 +2941,16 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>582</v>
+        <v>1603</v>
       </c>
       <c r="C27" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="D27" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="E27" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
@@ -2935,7 +2965,7 @@
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>611</v>
+        <v>1634</v>
       </c>
     </row>
     <row r="28">
@@ -2945,16 +2975,16 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1098</v>
+        <v>933</v>
       </c>
       <c r="C28" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D28" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E28" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F28" t="n">
         <v>2</v>
@@ -2969,7 +2999,7 @@
         <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>1150</v>
+        <v>979</v>
       </c>
     </row>
     <row r="29">
@@ -2979,22 +3009,22 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>301</v>
+        <v>177</v>
       </c>
       <c r="C29" t="n">
-        <v>77</v>
+        <v>5</v>
       </c>
       <c r="D29" t="n">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="E29" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F29" t="n">
         <v>1</v>
       </c>
       <c r="G29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H29" t="n">
         <v>0</v>
@@ -3003,7 +3033,7 @@
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>412</v>
+        <v>190</v>
       </c>
     </row>
     <row r="30">
@@ -3013,10 +3043,10 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>96</v>
+        <v>132</v>
       </c>
       <c r="C30" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D30" t="n">
         <v>0</v>
@@ -3037,7 +3067,7 @@
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>99</v>
+        <v>132</v>
       </c>
     </row>
     <row r="31">
@@ -3047,22 +3077,22 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>2831</v>
+        <v>4923</v>
       </c>
       <c r="C31" t="n">
-        <v>43</v>
+        <v>566</v>
       </c>
       <c r="D31" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E31" t="n">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="F31" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G31" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H31" t="n">
         <v>2</v>
@@ -3071,7 +3101,7 @@
         <v>0</v>
       </c>
       <c r="J31" t="n">
-        <v>2918</v>
+        <v>5546</v>
       </c>
     </row>
     <row r="32">
@@ -3081,16 +3111,16 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>134</v>
+        <v>169</v>
       </c>
       <c r="C32" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D32" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E32" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F32" t="n">
         <v>0</v>
@@ -3105,7 +3135,7 @@
         <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>143</v>
+        <v>175</v>
       </c>
     </row>
     <row r="33">
@@ -3115,13 +3145,13 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>54</v>
+        <v>111</v>
       </c>
       <c r="C33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E33" t="n">
         <v>0</v>
@@ -3139,7 +3169,7 @@
         <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>59</v>
+        <v>116</v>
       </c>
     </row>
     <row r="34">
@@ -3149,16 +3179,16 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>85</v>
+        <v>196</v>
       </c>
       <c r="C34" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F34" t="n">
         <v>0</v>
@@ -3173,7 +3203,7 @@
         <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>89</v>
+        <v>200</v>
       </c>
     </row>
     <row r="35">
@@ -3183,13 +3213,13 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>233</v>
+        <v>566</v>
       </c>
       <c r="C35" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E35" t="n">
         <v>2</v>
@@ -3207,7 +3237,7 @@
         <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>240</v>
+        <v>579</v>
       </c>
     </row>
     <row r="36">
@@ -3217,17 +3247,17 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>389</v>
+        <v>1108</v>
       </c>
       <c r="C36" t="n">
+        <v>31</v>
+      </c>
+      <c r="D36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" t="n">
         <v>6</v>
       </c>
-      <c r="D36" t="n">
-        <v>3</v>
-      </c>
-      <c r="E36" t="n">
-        <v>5</v>
-      </c>
       <c r="F36" t="n">
         <v>0</v>
       </c>
@@ -3241,7 +3271,7 @@
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>405</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="37">
@@ -3251,13 +3281,13 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>128</v>
+        <v>362</v>
       </c>
       <c r="C37" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E37" t="n">
         <v>0</v>
@@ -3275,7 +3305,7 @@
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>132</v>
+        <v>367</v>
       </c>
     </row>
     <row r="38">
@@ -3285,16 +3315,16 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>222</v>
+        <v>490</v>
       </c>
       <c r="C38" t="n">
         <v>1</v>
       </c>
       <c r="D38" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F38" t="n">
         <v>0</v>
@@ -3309,7 +3339,7 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>227</v>
+        <v>495</v>
       </c>
     </row>
     <row r="39">
@@ -3319,19 +3349,19 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>194</v>
+        <v>367</v>
       </c>
       <c r="C39" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D39" t="n">
         <v>2</v>
       </c>
       <c r="E39" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G39" t="n">
         <v>0</v>
@@ -3343,7 +3373,7 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>206</v>
+        <v>383</v>
       </c>
     </row>
     <row r="40">
@@ -3353,16 +3383,16 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>127</v>
+        <v>174</v>
       </c>
       <c r="C40" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D40" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E40" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F40" t="n">
         <v>0</v>
@@ -3377,7 +3407,7 @@
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>141</v>
+        <v>185</v>
       </c>
     </row>
     <row r="41">
@@ -3387,13 +3417,13 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>438</v>
+        <v>374</v>
       </c>
       <c r="C41" t="n">
-        <v>78</v>
+        <v>4</v>
       </c>
       <c r="D41" t="n">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="E41" t="n">
         <v>3</v>
@@ -3411,7 +3441,7 @@
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>547</v>
+        <v>386</v>
       </c>
     </row>
     <row r="42">
@@ -3421,17 +3451,17 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>324</v>
+        <v>579</v>
       </c>
       <c r="C42" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" t="n">
         <v>3</v>
       </c>
-      <c r="E42" t="n">
-        <v>2</v>
-      </c>
       <c r="F42" t="n">
         <v>0</v>
       </c>
@@ -3445,7 +3475,7 @@
         <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>335</v>
+        <v>588</v>
       </c>
     </row>
     <row r="43">
@@ -3455,16 +3485,16 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>419</v>
+        <v>510</v>
       </c>
       <c r="C43" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D43" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E43" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F43" t="n">
         <v>0</v>
@@ -3479,7 +3509,7 @@
         <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>430</v>
+        <v>522</v>
       </c>
     </row>
     <row r="44">
@@ -3489,16 +3519,16 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>379</v>
+        <v>592</v>
       </c>
       <c r="C44" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="D44" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E44" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F44" t="n">
         <v>0</v>
@@ -3513,7 +3543,7 @@
         <v>1</v>
       </c>
       <c r="J44" t="n">
-        <v>399</v>
+        <v>623</v>
       </c>
     </row>
     <row r="45">
@@ -3523,13 +3553,13 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>326</v>
+        <v>271</v>
       </c>
       <c r="C45" t="n">
-        <v>57</v>
+        <v>1</v>
       </c>
       <c r="D45" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="E45" t="n">
         <v>2</v>
@@ -3547,7 +3577,7 @@
         <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>410</v>
+        <v>276</v>
       </c>
     </row>
     <row r="46">
@@ -3557,31 +3587,31 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>883</v>
+        <v>520</v>
       </c>
       <c r="C46" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D46" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E46" t="n">
         <v>8</v>
       </c>
       <c r="F46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G46" t="n">
         <v>3</v>
       </c>
       <c r="H46" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I46" t="n">
         <v>0</v>
       </c>
       <c r="J46" t="n">
-        <v>911</v>
+        <v>537</v>
       </c>
     </row>
     <row r="47">
@@ -3591,16 +3621,16 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>140</v>
+        <v>203</v>
       </c>
       <c r="C47" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="D47" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F47" t="n">
         <v>0</v>
@@ -3615,7 +3645,7 @@
         <v>0</v>
       </c>
       <c r="J47" t="n">
-        <v>156</v>
+        <v>208</v>
       </c>
     </row>
     <row r="48">
@@ -3625,31 +3655,31 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>494</v>
+        <v>1447</v>
       </c>
       <c r="C48" t="n">
+        <v>26</v>
+      </c>
+      <c r="D48" t="n">
         <v>10</v>
       </c>
-      <c r="D48" t="n">
-        <v>12</v>
-      </c>
       <c r="E48" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I48" t="n">
         <v>0</v>
       </c>
       <c r="J48" t="n">
-        <v>524</v>
+        <v>1495</v>
       </c>
     </row>
     <row r="49">
@@ -3659,16 +3689,16 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>205</v>
+        <v>452</v>
       </c>
       <c r="C49" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F49" t="n">
         <v>0</v>
@@ -3683,7 +3713,7 @@
         <v>0</v>
       </c>
       <c r="J49" t="n">
-        <v>209</v>
+        <v>464</v>
       </c>
     </row>
     <row r="50">
@@ -3693,13 +3723,13 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>169</v>
+        <v>187</v>
       </c>
       <c r="C50" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D50" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E50" t="n">
         <v>0</v>
@@ -3717,7 +3747,7 @@
         <v>0</v>
       </c>
       <c r="J50" t="n">
-        <v>175</v>
+        <v>193</v>
       </c>
     </row>
     <row r="51">
@@ -3727,16 +3757,16 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>335</v>
+        <v>824</v>
       </c>
       <c r="C51" t="n">
+        <v>2</v>
+      </c>
+      <c r="D51" t="n">
         <v>3</v>
       </c>
-      <c r="D51" t="n">
-        <v>6</v>
-      </c>
       <c r="E51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F51" t="n">
         <v>0</v>
@@ -3751,7 +3781,7 @@
         <v>0</v>
       </c>
       <c r="J51" t="n">
-        <v>344</v>
+        <v>830</v>
       </c>
     </row>
     <row r="52">
@@ -3761,31 +3791,31 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>1869</v>
+        <v>3725</v>
       </c>
       <c r="C52" t="n">
-        <v>127</v>
+        <v>474</v>
       </c>
       <c r="D52" t="n">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="E52" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="F52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G52" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H52" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I52" t="n">
         <v>0</v>
       </c>
       <c r="J52" t="n">
-        <v>2042</v>
+        <v>4268</v>
       </c>
     </row>
     <row r="53">
@@ -3795,14 +3825,14 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>761</v>
+        <v>424</v>
       </c>
       <c r="C53" t="n">
+        <v>3</v>
+      </c>
+      <c r="D53" t="n">
         <v>5</v>
       </c>
-      <c r="D53" t="n">
-        <v>12</v>
-      </c>
       <c r="E53" t="n">
         <v>0</v>
       </c>
@@ -3819,7 +3849,7 @@
         <v>0</v>
       </c>
       <c r="J53" t="n">
-        <v>778</v>
+        <v>432</v>
       </c>
     </row>
     <row r="54">
@@ -3829,13 +3859,13 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>77</v>
+        <v>139</v>
       </c>
       <c r="C54" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E54" t="n">
         <v>0</v>
@@ -3853,7 +3883,7 @@
         <v>0</v>
       </c>
       <c r="J54" t="n">
-        <v>78</v>
+        <v>141</v>
       </c>
     </row>
     <row r="55">
@@ -3863,19 +3893,19 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>1922</v>
+        <v>3446</v>
       </c>
       <c r="C55" t="n">
-        <v>41</v>
+        <v>515</v>
       </c>
       <c r="D55" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="E55" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G55" t="n">
         <v>2</v>
@@ -3887,7 +3917,7 @@
         <v>0</v>
       </c>
       <c r="J55" t="n">
-        <v>1985</v>
+        <v>3991</v>
       </c>
     </row>
     <row r="56">
@@ -3897,7 +3927,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>129</v>
+        <v>97</v>
       </c>
       <c r="C56" t="n">
         <v>6</v>
@@ -3906,7 +3936,7 @@
         <v>1</v>
       </c>
       <c r="E56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F56" t="n">
         <v>0</v>
@@ -3921,7 +3951,7 @@
         <v>0</v>
       </c>
       <c r="J56" t="n">
-        <v>138</v>
+        <v>107</v>
       </c>
     </row>
     <row r="57">
@@ -3931,13 +3961,13 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>174</v>
+        <v>329</v>
       </c>
       <c r="C57" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D57" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E57" t="n">
         <v>1</v>
@@ -3955,7 +3985,7 @@
         <v>0</v>
       </c>
       <c r="J57" t="n">
-        <v>183</v>
+        <v>342</v>
       </c>
     </row>
     <row r="58">
@@ -3965,14 +3995,14 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>124</v>
+        <v>165</v>
       </c>
       <c r="C58" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" t="n">
         <v>4</v>
       </c>
-      <c r="D58" t="n">
-        <v>3</v>
-      </c>
       <c r="E58" t="n">
         <v>1</v>
       </c>
@@ -3989,7 +4019,7 @@
         <v>0</v>
       </c>
       <c r="J58" t="n">
-        <v>132</v>
+        <v>171</v>
       </c>
     </row>
     <row r="59">
@@ -3999,17 +4029,17 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>94</v>
+        <v>117</v>
       </c>
       <c r="C59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D59" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" t="n">
         <v>3</v>
       </c>
-      <c r="E59" t="n">
-        <v>0</v>
-      </c>
       <c r="F59" t="n">
         <v>0</v>
       </c>
@@ -4023,7 +4053,7 @@
         <v>0</v>
       </c>
       <c r="J59" t="n">
-        <v>98</v>
+        <v>122</v>
       </c>
     </row>
     <row r="60">
@@ -4033,16 +4063,16 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>538</v>
+        <v>1037</v>
       </c>
       <c r="C60" t="n">
         <v>7</v>
       </c>
       <c r="D60" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E60" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F60" t="n">
         <v>0</v>
@@ -4057,7 +4087,7 @@
         <v>0</v>
       </c>
       <c r="J60" t="n">
-        <v>554</v>
+        <v>1052</v>
       </c>
     </row>
     <row r="61">
@@ -4067,22 +4097,22 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>656</v>
+        <v>1030</v>
       </c>
       <c r="C61" t="n">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="D61" t="n">
         <v>8</v>
       </c>
       <c r="E61" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F61" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H61" t="n">
         <v>0</v>
@@ -4091,7 +4121,7 @@
         <v>0</v>
       </c>
       <c r="J61" t="n">
-        <v>718</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="62">
@@ -4101,16 +4131,16 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>370</v>
+        <v>334</v>
       </c>
       <c r="C62" t="n">
-        <v>99</v>
+        <v>8</v>
       </c>
       <c r="D62" t="n">
-        <v>60</v>
+        <v>2</v>
       </c>
       <c r="E62" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F62" t="n">
         <v>0</v>
@@ -4125,7 +4155,7 @@
         <v>0</v>
       </c>
       <c r="J62" t="n">
-        <v>534</v>
+        <v>346</v>
       </c>
     </row>
     <row r="63">
@@ -4135,16 +4165,16 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>1520</v>
+        <v>1808</v>
       </c>
       <c r="C63" t="n">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="D63" t="n">
-        <v>41</v>
+        <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="F63" t="n">
         <v>0</v>
@@ -4159,7 +4189,7 @@
         <v>0</v>
       </c>
       <c r="J63" t="n">
-        <v>1604</v>
+        <v>1849</v>
       </c>
     </row>
     <row r="64">
@@ -4169,19 +4199,19 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>1389</v>
+        <v>1010</v>
       </c>
       <c r="C64" t="n">
-        <v>35</v>
+        <v>62</v>
       </c>
       <c r="D64" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="E64" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G64" t="n">
         <v>3</v>
@@ -4193,7 +4223,7 @@
         <v>0</v>
       </c>
       <c r="J64" t="n">
-        <v>1451</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="65">
@@ -4203,31 +4233,31 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>38611</v>
+        <v>55768</v>
       </c>
       <c r="C65" t="n">
-        <v>3104</v>
+        <v>5310</v>
       </c>
       <c r="D65" t="n">
-        <v>906</v>
+        <v>1207</v>
       </c>
       <c r="E65" t="n">
-        <v>203</v>
+        <v>295</v>
       </c>
       <c r="F65" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="G65" t="n">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="H65" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="I65" t="n">
         <v>2</v>
       </c>
       <c r="J65" t="n">
-        <v>42922</v>
+        <v>62676</v>
       </c>
     </row>
   </sheetData>
@@ -4303,22 +4333,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3682</v>
+        <v>5375</v>
       </c>
       <c r="C2" t="n">
-        <v>71</v>
+        <v>808</v>
       </c>
       <c r="D2" t="n">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="E2" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -4327,7 +4357,7 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>3790</v>
+        <v>6242</v>
       </c>
     </row>
     <row r="3">
@@ -4337,19 +4367,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1528</v>
+        <v>2530</v>
       </c>
       <c r="C3" t="n">
-        <v>31</v>
+        <v>451</v>
       </c>
       <c r="D3" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E3" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G3" t="n">
         <v>3</v>
@@ -4361,7 +4391,7 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>1588</v>
+        <v>3022</v>
       </c>
     </row>
     <row r="4">
@@ -4371,31 +4401,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2728</v>
+        <v>2645</v>
       </c>
       <c r="C4" t="n">
-        <v>1831</v>
+        <v>1903</v>
       </c>
       <c r="D4" t="n">
-        <v>279</v>
+        <v>901</v>
       </c>
       <c r="E4" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="F4" t="n">
         <v>2</v>
       </c>
       <c r="G4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I4" t="n">
         <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>4859</v>
+        <v>5477</v>
       </c>
     </row>
     <row r="5">
@@ -4405,16 +4435,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>233</v>
+        <v>83</v>
       </c>
       <c r="C5" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="D5" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -4429,7 +4459,7 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>255</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6">
@@ -4439,31 +4469,31 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>490</v>
+        <v>1438</v>
       </c>
       <c r="C6" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="D6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E6" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>512</v>
+        <v>1479</v>
       </c>
     </row>
     <row r="7">
@@ -4473,19 +4503,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>599</v>
+        <v>848</v>
       </c>
       <c r="C7" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="D7" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F7" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
         <v>2</v>
@@ -4497,7 +4527,7 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>634</v>
+        <v>883</v>
       </c>
     </row>
     <row r="8">
@@ -4507,16 +4537,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>846</v>
+        <v>774</v>
       </c>
       <c r="C8" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="D8" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
@@ -4531,7 +4561,7 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>880</v>
+        <v>813</v>
       </c>
     </row>
     <row r="9">
@@ -4541,16 +4571,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>419</v>
+        <v>495</v>
       </c>
       <c r="C9" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
@@ -4565,7 +4595,7 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>430</v>
+        <v>507</v>
       </c>
     </row>
     <row r="10">
@@ -4575,16 +4605,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>350</v>
+        <v>319</v>
       </c>
       <c r="C10" t="n">
-        <v>95</v>
+        <v>8</v>
       </c>
       <c r="D10" t="n">
-        <v>60</v>
+        <v>2</v>
       </c>
       <c r="E10" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
@@ -4599,7 +4629,7 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>510</v>
+        <v>331</v>
       </c>
     </row>
     <row r="11">
@@ -4609,22 +4639,22 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2121</v>
+        <v>2323</v>
       </c>
       <c r="C11" t="n">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="D11" t="n">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="E11" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="F11" t="n">
         <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H11" t="n">
         <v>2</v>
@@ -4633,7 +4663,7 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>2223</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="12">
@@ -4643,10 +4673,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>31</v>
+        <v>64</v>
       </c>
       <c r="C12" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="D12" t="n">
         <v>1</v>
@@ -4667,7 +4697,7 @@
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>33</v>
+        <v>79</v>
       </c>
     </row>
     <row r="13">
@@ -4677,10 +4707,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>38</v>
+        <v>123</v>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
@@ -4701,7 +4731,7 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>39</v>
+        <v>132</v>
       </c>
     </row>
     <row r="14">
@@ -4711,10 +4741,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
@@ -4735,7 +4765,7 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>8</v>
+        <v>23</v>
       </c>
     </row>
     <row r="15">
@@ -4745,10 +4775,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="C15" t="n">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="D15" t="n">
         <v>1</v>
@@ -4769,7 +4799,7 @@
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>65</v>
+        <v>105</v>
       </c>
     </row>
     <row r="16">
@@ -4779,16 +4809,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>28</v>
+        <v>81</v>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16" t="n">
         <v>1</v>
@@ -4803,7 +4833,7 @@
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>31</v>
+        <v>95</v>
       </c>
     </row>
     <row r="17">
@@ -4813,10 +4843,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>44</v>
+        <v>101</v>
       </c>
       <c r="C17" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
@@ -4837,7 +4867,7 @@
         <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>46</v>
+        <v>117</v>
       </c>
     </row>
     <row r="18">
@@ -4847,10 +4877,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
@@ -4871,7 +4901,7 @@
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>25</v>
+        <v>63</v>
       </c>
     </row>
     <row r="19">
@@ -4881,10 +4911,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>38</v>
+        <v>82</v>
       </c>
       <c r="C19" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="D19" t="n">
         <v>1</v>
@@ -4905,7 +4935,7 @@
         <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>49</v>
+        <v>108</v>
       </c>
     </row>
     <row r="20">
@@ -4915,10 +4945,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>15</v>
+        <v>56</v>
       </c>
       <c r="C20" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
@@ -4939,7 +4969,7 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>16</v>
+        <v>63</v>
       </c>
     </row>
     <row r="21">
@@ -4949,10 +4979,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>48</v>
+        <v>143</v>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
@@ -4973,7 +5003,7 @@
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>48</v>
+        <v>152</v>
       </c>
     </row>
     <row r="22">
@@ -4983,10 +5013,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>33</v>
+        <v>97</v>
       </c>
       <c r="C22" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
@@ -5007,7 +5037,7 @@
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>33</v>
+        <v>100</v>
       </c>
     </row>
     <row r="23">
@@ -5017,13 +5047,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>70</v>
+        <v>179</v>
       </c>
       <c r="C23" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="D23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
@@ -5041,7 +5071,7 @@
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>73</v>
+        <v>198</v>
       </c>
     </row>
     <row r="24">
@@ -5051,10 +5081,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>29</v>
+        <v>225</v>
       </c>
       <c r="C24" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D24" t="n">
         <v>6</v>
@@ -5075,7 +5105,7 @@
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>45</v>
+        <v>245</v>
       </c>
     </row>
     <row r="25">
@@ -5085,10 +5115,10 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>12</v>
+        <v>60</v>
       </c>
       <c r="C25" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
@@ -5109,7 +5139,7 @@
         <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>13</v>
+        <v>65</v>
       </c>
     </row>
     <row r="26">
@@ -5119,16 +5149,16 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>569</v>
+        <v>1686</v>
       </c>
       <c r="C26" t="n">
-        <v>7</v>
+        <v>38</v>
       </c>
       <c r="D26" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E26" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F26" t="n">
         <v>1</v>
@@ -5143,7 +5173,7 @@
         <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>590</v>
+        <v>1738</v>
       </c>
     </row>
     <row r="27">
@@ -5153,31 +5183,31 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>349</v>
+        <v>509</v>
       </c>
       <c r="C27" t="n">
         <v>5</v>
       </c>
       <c r="D27" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E27" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I27" t="n">
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>373</v>
+        <v>530</v>
       </c>
     </row>
     <row r="28">
@@ -5187,31 +5217,31 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>5408</v>
+        <v>3204</v>
       </c>
       <c r="C28" t="n">
-        <v>68</v>
+        <v>31</v>
       </c>
       <c r="D28" t="n">
-        <v>71</v>
+        <v>27</v>
       </c>
       <c r="E28" t="n">
         <v>24</v>
       </c>
       <c r="F28" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G28" t="n">
         <v>12</v>
       </c>
       <c r="H28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I28" t="n">
         <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>5584</v>
+        <v>3303</v>
       </c>
     </row>
     <row r="29">
@@ -5221,17 +5251,17 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>427</v>
+        <v>782</v>
       </c>
       <c r="C29" t="n">
+        <v>12</v>
+      </c>
+      <c r="D29" t="n">
+        <v>14</v>
+      </c>
+      <c r="E29" t="n">
         <v>15</v>
       </c>
-      <c r="D29" t="n">
-        <v>19</v>
-      </c>
-      <c r="E29" t="n">
-        <v>7</v>
-      </c>
       <c r="F29" t="n">
         <v>0</v>
       </c>
@@ -5239,13 +5269,13 @@
         <v>2</v>
       </c>
       <c r="H29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I29" t="n">
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>473</v>
+        <v>827</v>
       </c>
     </row>
     <row r="30">
@@ -5255,22 +5285,22 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1092</v>
+        <v>714</v>
       </c>
       <c r="C30" t="n">
-        <v>267</v>
+        <v>9</v>
       </c>
       <c r="D30" t="n">
-        <v>108</v>
+        <v>3</v>
       </c>
       <c r="E30" t="n">
         <v>8</v>
       </c>
       <c r="F30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H30" t="n">
         <v>0</v>
@@ -5279,7 +5309,7 @@
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>1477</v>
+        <v>736</v>
       </c>
     </row>
     <row r="31">
@@ -5289,16 +5319,16 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>2573</v>
+        <v>4346</v>
       </c>
       <c r="C31" t="n">
-        <v>94</v>
+        <v>19</v>
       </c>
       <c r="D31" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E31" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="F31" t="n">
         <v>0</v>
@@ -5313,7 +5343,7 @@
         <v>1</v>
       </c>
       <c r="J31" t="n">
-        <v>2691</v>
+        <v>4396</v>
       </c>
     </row>
     <row r="32">
@@ -5323,19 +5353,19 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>3043</v>
+        <v>6645</v>
       </c>
       <c r="C32" t="n">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="D32" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E32" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G32" t="n">
         <v>2</v>
@@ -5347,7 +5377,7 @@
         <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>3122</v>
+        <v>6734</v>
       </c>
     </row>
     <row r="33">
@@ -5357,31 +5387,31 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>762</v>
+        <v>1629</v>
       </c>
       <c r="C33" t="n">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="D33" t="n">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="E33" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F33" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I33" t="n">
         <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>850</v>
+        <v>1698</v>
       </c>
     </row>
     <row r="34">
@@ -5391,16 +5421,16 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>783</v>
+        <v>2081</v>
       </c>
       <c r="C34" t="n">
+        <v>14</v>
+      </c>
+      <c r="D34" t="n">
         <v>7</v>
       </c>
-      <c r="D34" t="n">
-        <v>15</v>
-      </c>
       <c r="E34" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F34" t="n">
         <v>0</v>
@@ -5415,7 +5445,7 @@
         <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>811</v>
+        <v>2113</v>
       </c>
     </row>
     <row r="35">
@@ -5425,13 +5455,13 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>780</v>
+        <v>645</v>
       </c>
       <c r="C35" t="n">
-        <v>137</v>
+        <v>6</v>
       </c>
       <c r="D35" t="n">
-        <v>55</v>
+        <v>5</v>
       </c>
       <c r="E35" t="n">
         <v>5</v>
@@ -5449,7 +5479,7 @@
         <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>978</v>
+        <v>662</v>
       </c>
     </row>
     <row r="36">
@@ -5459,16 +5489,16 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1208</v>
+        <v>2395</v>
       </c>
       <c r="C36" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D36" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="E36" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F36" t="n">
         <v>0</v>
@@ -5483,7 +5513,7 @@
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>1241</v>
+        <v>2421</v>
       </c>
     </row>
     <row r="37">
@@ -5493,22 +5523,22 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>674</v>
+        <v>1082</v>
       </c>
       <c r="C37" t="n">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="D37" t="n">
         <v>8</v>
       </c>
       <c r="E37" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H37" t="n">
         <v>0</v>
@@ -5517,7 +5547,7 @@
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>725</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="38">
@@ -5527,22 +5557,22 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>2945</v>
+        <v>5067</v>
       </c>
       <c r="C38" t="n">
-        <v>75</v>
+        <v>637</v>
       </c>
       <c r="D38" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="E38" t="n">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="F38" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G38" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H38" t="n">
         <v>2</v>
@@ -5551,7 +5581,7 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>3063</v>
+        <v>5763</v>
       </c>
     </row>
     <row r="39">
@@ -5561,16 +5591,16 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>854</v>
+        <v>568</v>
       </c>
       <c r="C39" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="D39" t="n">
         <v>2</v>
       </c>
       <c r="E39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F39" t="n">
         <v>1</v>
@@ -5585,7 +5615,7 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>877</v>
+        <v>579</v>
       </c>
     </row>
     <row r="40">
@@ -5595,31 +5625,31 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1662</v>
+        <v>2945</v>
       </c>
       <c r="C40" t="n">
-        <v>90</v>
+        <v>416</v>
       </c>
       <c r="D40" t="n">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="E40" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H40" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I40" t="n">
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>1796</v>
+        <v>3424</v>
       </c>
     </row>
     <row r="41">
@@ -5629,19 +5659,19 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>2010</v>
+        <v>3300</v>
       </c>
       <c r="C41" t="n">
-        <v>36</v>
+        <v>516</v>
       </c>
       <c r="D41" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="E41" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G41" t="n">
         <v>2</v>
@@ -5653,7 +5683,7 @@
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>2066</v>
+        <v>3845</v>
       </c>
     </row>
     <row r="42">
@@ -5663,31 +5693,31 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>38611</v>
+        <v>55768</v>
       </c>
       <c r="C42" t="n">
-        <v>3104</v>
+        <v>5310</v>
       </c>
       <c r="D42" t="n">
-        <v>906</v>
+        <v>1207</v>
       </c>
       <c r="E42" t="n">
-        <v>203</v>
+        <v>295</v>
       </c>
       <c r="F42" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="G42" t="n">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="H42" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="I42" t="n">
         <v>2</v>
       </c>
       <c r="J42" t="n">
-        <v>42922</v>
+        <v>62676</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(metabase): filter metabase query on server-side to prevent excel truncation and match dashboard numbers
</commit_message>
<xml_diff>
--- a/BaoCao_TonKho.xlsx
+++ b/BaoCao_TonKho.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>04/06/2026 17:01:23</t>
+          <t>05/06/2026 00:38:37</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -579,19 +579,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>6893</v>
+        <v>10724</v>
       </c>
       <c r="C7" t="n">
-        <v>118</v>
+        <v>161</v>
       </c>
       <c r="D7" t="n">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="E7" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="F7" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="G7" t="n">
         <v>6</v>
@@ -606,7 +606,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>7092</v>
+        <v>10985</v>
       </c>
     </row>
     <row r="8">
@@ -616,19 +616,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1525</v>
+        <v>2863</v>
       </c>
       <c r="C8" t="n">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="D8" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
@@ -637,7 +637,7 @@
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="n">
-        <v>1566</v>
+        <v>2925</v>
       </c>
     </row>
     <row r="9">
@@ -647,18 +647,20 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>939</v>
+        <v>1918</v>
       </c>
       <c r="C9" t="n">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E9" t="n">
         <v>4</v>
       </c>
-      <c r="F9" t="inlineStr"/>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
       <c r="G9" t="n">
         <v>2</v>
       </c>
@@ -666,7 +668,7 @@
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="n">
-        <v>980</v>
+        <v>1967</v>
       </c>
     </row>
     <row r="10">
@@ -676,16 +678,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>872</v>
+        <v>1595</v>
       </c>
       <c r="C10" t="n">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="D10" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
@@ -693,7 +695,7 @@
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="n">
-        <v>911</v>
+        <v>1647</v>
       </c>
     </row>
     <row r="11">
@@ -703,24 +705,26 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>521</v>
+        <v>960</v>
       </c>
       <c r="C11" t="n">
         <v>8</v>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E11" t="n">
-        <v>3</v>
-      </c>
-      <c r="F11" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="n">
-        <v>533</v>
+        <v>974</v>
       </c>
     </row>
     <row r="12">
@@ -730,24 +734,26 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>347</v>
+        <v>694</v>
       </c>
       <c r="C12" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="D12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
-      </c>
-      <c r="F12" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="n">
-        <v>359</v>
+        <v>716</v>
       </c>
     </row>
     <row r="13">
@@ -757,19 +763,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2689</v>
+        <v>2694</v>
       </c>
       <c r="C13" t="n">
+        <v>18</v>
+      </c>
+      <c r="D13" t="n">
+        <v>16</v>
+      </c>
+      <c r="E13" t="n">
         <v>15</v>
       </c>
-      <c r="D13" t="n">
-        <v>12</v>
-      </c>
-      <c r="E13" t="n">
-        <v>18</v>
-      </c>
       <c r="F13" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G13" t="n">
         <v>4</v>
@@ -780,7 +786,7 @@
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="n">
-        <v>2743</v>
+        <v>2756</v>
       </c>
     </row>
     <row r="14">
@@ -790,25 +796,25 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1348</v>
+        <v>1514</v>
       </c>
       <c r="C14" t="n">
-        <v>202</v>
+        <v>266</v>
       </c>
       <c r="D14" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E14" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F14" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G14" t="n">
         <v>2</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -817,7 +823,7 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>1579</v>
+        <v>1812</v>
       </c>
     </row>
     <row r="15">
@@ -827,10 +833,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="C15" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D15" t="n">
         <v>1</v>
@@ -842,7 +848,7 @@
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="n">
-        <v>80</v>
+        <v>94</v>
       </c>
     </row>
     <row r="16">
@@ -852,10 +858,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C16" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
@@ -867,7 +873,7 @@
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="n">
-        <v>134</v>
+        <v>144</v>
       </c>
     </row>
     <row r="17">
@@ -877,7 +883,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="C17" t="n">
         <v>1</v>
@@ -892,7 +898,7 @@
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="18">
@@ -902,12 +908,14 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="C18" t="n">
-        <v>49</v>
-      </c>
-      <c r="D18" t="inlineStr"/>
+        <v>52</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
       <c r="E18" t="n">
         <v>1</v>
       </c>
@@ -917,7 +925,7 @@
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="n">
-        <v>107</v>
+        <v>121</v>
       </c>
     </row>
     <row r="19">
@@ -927,26 +935,26 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="C19" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="n">
         <v>1</v>
       </c>
-      <c r="F19" t="n">
-        <v>1</v>
-      </c>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="n">
         <v>1</v>
       </c>
-      <c r="H19" t="inlineStr"/>
+      <c r="H19" t="n">
+        <v>1</v>
+      </c>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="n">
-        <v>97</v>
+        <v>109</v>
       </c>
     </row>
     <row r="20">
@@ -956,10 +964,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="C20" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
@@ -971,7 +979,7 @@
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="n">
-        <v>123</v>
+        <v>137</v>
       </c>
     </row>
     <row r="21">
@@ -981,10 +989,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C21" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
@@ -998,7 +1006,7 @@
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="22">
@@ -1008,24 +1016,24 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="C22" t="n">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="D22" t="n">
         <v>2</v>
       </c>
-      <c r="E22" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="n">
+        <v>1</v>
+      </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="n">
-        <v>113</v>
+        <v>127</v>
       </c>
     </row>
     <row r="23">
@@ -1035,10 +1043,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="C23" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
@@ -1050,7 +1058,7 @@
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="n">
-        <v>65</v>
+        <v>72</v>
       </c>
     </row>
     <row r="24">
@@ -1060,10 +1068,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="C24" t="n">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr"/>
@@ -1073,7 +1081,7 @@
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="n">
-        <v>154</v>
+        <v>171</v>
       </c>
     </row>
     <row r="25">
@@ -1083,10 +1091,10 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="C25" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr"/>
@@ -1096,7 +1104,7 @@
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="n">
-        <v>103</v>
+        <v>123</v>
       </c>
     </row>
     <row r="26">
@@ -1106,13 +1114,13 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>180</v>
+        <v>202</v>
       </c>
       <c r="C26" t="n">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="D26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="n">
@@ -1123,7 +1131,7 @@
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="n">
-        <v>205</v>
+        <v>238</v>
       </c>
     </row>
     <row r="27">
@@ -1133,7 +1141,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>235</v>
+        <v>292</v>
       </c>
       <c r="C27" t="n">
         <v>9</v>
@@ -1142,10 +1150,10 @@
         <v>6</v>
       </c>
       <c r="E27" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G27" t="n">
         <v>1</v>
@@ -1154,7 +1162,7 @@
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="n">
-        <v>256</v>
+        <v>314</v>
       </c>
     </row>
     <row r="28">
@@ -1164,22 +1172,22 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C28" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D28" t="inlineStr"/>
-      <c r="E28" t="n">
-        <v>1</v>
-      </c>
-      <c r="F28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="n">
+        <v>1</v>
+      </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="n">
-        <v>66</v>
+        <v>77</v>
       </c>
     </row>
     <row r="29">
@@ -1189,10 +1197,10 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>117</v>
+        <v>195</v>
       </c>
       <c r="C29" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="D29" t="n">
         <v>4</v>
@@ -1216,7 +1224,7 @@
         <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>145</v>
+        <v>229</v>
       </c>
     </row>
     <row r="30">
@@ -1226,10 +1234,10 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>117</v>
+        <v>195</v>
       </c>
       <c r="C30" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="D30" t="n">
         <v>4</v>
@@ -1247,7 +1255,7 @@
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="n">
-        <v>145</v>
+        <v>229</v>
       </c>
     </row>
     <row r="31">
@@ -1257,19 +1265,19 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>25272</v>
+        <v>26662</v>
       </c>
       <c r="C31" t="n">
-        <v>301</v>
+        <v>436</v>
       </c>
       <c r="D31" t="n">
-        <v>120</v>
+        <v>174</v>
       </c>
       <c r="E31" t="n">
-        <v>132</v>
+        <v>119</v>
       </c>
       <c r="F31" t="n">
-        <v>18</v>
+        <v>48</v>
       </c>
       <c r="G31" t="n">
         <v>25</v>
@@ -1284,7 +1292,7 @@
         <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>25874</v>
+        <v>27470</v>
       </c>
     </row>
     <row r="32">
@@ -1294,19 +1302,19 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1782</v>
+        <v>3608</v>
       </c>
       <c r="C32" t="n">
-        <v>46</v>
+        <v>110</v>
       </c>
       <c r="D32" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E32" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F32" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G32" t="n">
         <v>2</v>
@@ -1315,7 +1323,7 @@
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="n">
-        <v>1841</v>
+        <v>3737</v>
       </c>
     </row>
     <row r="33">
@@ -1325,18 +1333,20 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>614</v>
+        <v>1273</v>
       </c>
       <c r="C33" t="n">
         <v>4</v>
       </c>
       <c r="D33" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E33" t="n">
-        <v>10</v>
-      </c>
-      <c r="F33" t="inlineStr"/>
+        <v>9</v>
+      </c>
+      <c r="F33" t="n">
+        <v>2</v>
+      </c>
       <c r="G33" t="n">
         <v>1</v>
       </c>
@@ -1346,7 +1356,7 @@
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="n">
-        <v>633</v>
+        <v>1295</v>
       </c>
     </row>
     <row r="34">
@@ -1356,19 +1366,19 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>3201</v>
+        <v>3263</v>
       </c>
       <c r="C34" t="n">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="D34" t="n">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="E34" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F34" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="G34" t="n">
         <v>12</v>
@@ -1377,7 +1387,7 @@
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="n">
-        <v>3301</v>
+        <v>3405</v>
       </c>
     </row>
     <row r="35">
@@ -1387,19 +1397,19 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>808</v>
+        <v>374</v>
       </c>
       <c r="C35" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D35" t="n">
         <v>12</v>
       </c>
       <c r="E35" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G35" t="n">
         <v>2</v>
@@ -1410,7 +1420,7 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="n">
-        <v>854</v>
+        <v>414</v>
       </c>
     </row>
     <row r="36">
@@ -1420,19 +1430,19 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>774</v>
+        <v>1470</v>
       </c>
       <c r="C36" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D36" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E36" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F36" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G36" t="n">
         <v>1</v>
@@ -1441,7 +1451,7 @@
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="n">
-        <v>797</v>
+        <v>1499</v>
       </c>
     </row>
     <row r="37">
@@ -1451,13 +1461,13 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>4551</v>
+        <v>935</v>
       </c>
       <c r="C37" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D37" t="n">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="E37" t="n">
         <v>15</v>
@@ -1472,7 +1482,7 @@
       </c>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="n">
-        <v>4604</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="38">
@@ -1482,19 +1492,19 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>6929</v>
+        <v>8965</v>
       </c>
       <c r="C38" t="n">
-        <v>71</v>
+        <v>92</v>
       </c>
       <c r="D38" t="n">
+        <v>13</v>
+      </c>
+      <c r="E38" t="n">
         <v>14</v>
       </c>
-      <c r="E38" t="n">
-        <v>15</v>
-      </c>
       <c r="F38" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G38" t="n">
         <v>2</v>
@@ -1503,7 +1513,7 @@
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="n">
-        <v>7036</v>
+        <v>9093</v>
       </c>
     </row>
     <row r="39">
@@ -1513,19 +1523,19 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1701</v>
+        <v>791</v>
       </c>
       <c r="C39" t="n">
-        <v>50</v>
+        <v>108</v>
       </c>
       <c r="D39" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="E39" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G39" t="n">
         <v>1</v>
@@ -1536,7 +1546,7 @@
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="n">
-        <v>1781</v>
+        <v>937</v>
       </c>
     </row>
     <row r="40">
@@ -1546,18 +1556,20 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>2186</v>
+        <v>1433</v>
       </c>
       <c r="C40" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="D40" t="n">
+        <v>9</v>
+      </c>
+      <c r="E40" t="n">
         <v>8</v>
       </c>
-      <c r="E40" t="n">
-        <v>9</v>
-      </c>
-      <c r="F40" t="inlineStr"/>
+      <c r="F40" t="n">
+        <v>3</v>
+      </c>
       <c r="G40" t="n">
         <v>2</v>
       </c>
@@ -1565,7 +1577,7 @@
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="n">
-        <v>2219</v>
+        <v>1461</v>
       </c>
     </row>
     <row r="41">
@@ -1575,18 +1587,20 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>709</v>
+        <v>1215</v>
       </c>
       <c r="C41" t="n">
+        <v>8</v>
+      </c>
+      <c r="D41" t="n">
+        <v>3</v>
+      </c>
+      <c r="E41" t="n">
         <v>6</v>
       </c>
-      <c r="D41" t="n">
-        <v>5</v>
-      </c>
-      <c r="E41" t="n">
-        <v>5</v>
-      </c>
-      <c r="F41" t="inlineStr"/>
+      <c r="F41" t="n">
+        <v>2</v>
+      </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="n">
         <v>1</v>
@@ -1594,7 +1608,7 @@
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="n">
-        <v>726</v>
+        <v>1235</v>
       </c>
     </row>
     <row r="42">
@@ -1604,24 +1618,26 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>855</v>
+        <v>2262</v>
       </c>
       <c r="C42" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D42" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E42" t="n">
-        <v>7</v>
-      </c>
-      <c r="F42" t="inlineStr"/>
+        <v>11</v>
+      </c>
+      <c r="F42" t="n">
+        <v>1</v>
+      </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="n">
-        <v>878</v>
+        <v>2285</v>
       </c>
     </row>
     <row r="43">
@@ -1631,18 +1647,20 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>1162</v>
+        <v>1073</v>
       </c>
       <c r="C43" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="D43" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E43" t="n">
         <v>5</v>
       </c>
-      <c r="F43" t="inlineStr"/>
+      <c r="F43" t="n">
+        <v>1</v>
+      </c>
       <c r="G43" t="n">
         <v>1</v>
       </c>
@@ -1650,7 +1668,7 @@
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="n">
-        <v>1204</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="44">
@@ -1660,16 +1678,16 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>2593</v>
+        <v>3409</v>
       </c>
       <c r="C44" t="n">
-        <v>1796</v>
+        <v>2245</v>
       </c>
       <c r="D44" t="n">
-        <v>1241</v>
+        <v>1905</v>
       </c>
       <c r="E44" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="F44" t="n">
         <v>2</v>
@@ -1687,7 +1705,7 @@
         <v>0</v>
       </c>
       <c r="K44" t="n">
-        <v>5659</v>
+        <v>7592</v>
       </c>
     </row>
     <row r="45">
@@ -1697,16 +1715,16 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>2593</v>
+        <v>3409</v>
       </c>
       <c r="C45" t="n">
-        <v>1796</v>
+        <v>2245</v>
       </c>
       <c r="D45" t="n">
-        <v>1241</v>
+        <v>1905</v>
       </c>
       <c r="E45" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="F45" t="n">
         <v>2</v>
@@ -1722,7 +1740,7 @@
       </c>
       <c r="J45" t="inlineStr"/>
       <c r="K45" t="n">
-        <v>5659</v>
+        <v>7592</v>
       </c>
     </row>
     <row r="46">
@@ -1732,19 +1750,19 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>19304</v>
+        <v>32375</v>
       </c>
       <c r="C46" t="n">
-        <v>3750</v>
+        <v>8101</v>
       </c>
       <c r="D46" t="n">
-        <v>153</v>
+        <v>272</v>
       </c>
       <c r="E46" t="n">
-        <v>77</v>
+        <v>59</v>
       </c>
       <c r="F46" t="n">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="G46" t="n">
         <v>16</v>
@@ -1759,7 +1777,7 @@
         <v>0</v>
       </c>
       <c r="K46" t="n">
-        <v>23317</v>
+        <v>40860</v>
       </c>
     </row>
     <row r="47">
@@ -1769,19 +1787,19 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>5420</v>
+        <v>9748</v>
       </c>
       <c r="C47" t="n">
-        <v>1099</v>
+        <v>2516</v>
       </c>
       <c r="D47" t="n">
-        <v>40</v>
+        <v>61</v>
       </c>
       <c r="E47" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F47" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G47" t="n">
         <v>4</v>
@@ -1792,7 +1810,7 @@
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="n">
-        <v>6582</v>
+        <v>12348</v>
       </c>
     </row>
     <row r="48">
@@ -1802,19 +1820,19 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>2569</v>
+        <v>3913</v>
       </c>
       <c r="C48" t="n">
-        <v>573</v>
+        <v>1098</v>
       </c>
       <c r="D48" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E48" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F48" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="G48" t="n">
         <v>3</v>
@@ -1823,7 +1841,7 @@
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="n">
-        <v>3183</v>
+        <v>5058</v>
       </c>
     </row>
     <row r="49">
@@ -1833,19 +1851,19 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>5063</v>
+        <v>8501</v>
       </c>
       <c r="C49" t="n">
-        <v>877</v>
+        <v>1947</v>
       </c>
       <c r="D49" t="n">
-        <v>27</v>
+        <v>67</v>
       </c>
       <c r="E49" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="F49" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G49" t="n">
         <v>5</v>
@@ -1856,7 +1874,7 @@
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="n">
-        <v>6000</v>
+        <v>10549</v>
       </c>
     </row>
     <row r="50">
@@ -1866,19 +1884,19 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>2964</v>
+        <v>4746</v>
       </c>
       <c r="C50" t="n">
-        <v>539</v>
+        <v>1106</v>
       </c>
       <c r="D50" t="n">
-        <v>53</v>
+        <v>93</v>
       </c>
       <c r="E50" t="n">
         <v>9</v>
       </c>
       <c r="F50" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G50" t="n">
         <v>2</v>
@@ -1889,7 +1907,7 @@
       <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr"/>
       <c r="K50" t="n">
-        <v>3571</v>
+        <v>5961</v>
       </c>
     </row>
     <row r="51">
@@ -1899,19 +1917,19 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>3288</v>
+        <v>5467</v>
       </c>
       <c r="C51" t="n">
-        <v>662</v>
+        <v>1434</v>
       </c>
       <c r="D51" t="n">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="E51" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F51" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G51" t="n">
         <v>2</v>
@@ -1920,7 +1938,7 @@
       <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr"/>
       <c r="K51" t="n">
-        <v>3981</v>
+        <v>6944</v>
       </c>
     </row>
     <row r="52">
@@ -1930,19 +1948,19 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>615</v>
+        <v>1110</v>
       </c>
       <c r="C52" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="D52" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F52" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G52" t="n">
         <v>1</v>
@@ -1957,7 +1975,7 @@
         <v>0</v>
       </c>
       <c r="K52" t="n">
-        <v>627</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="53">
@@ -1967,19 +1985,19 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>615</v>
+        <v>1110</v>
       </c>
       <c r="C53" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="D53" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F53" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G53" t="n">
         <v>1</v>
@@ -1988,7 +2006,7 @@
       <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr"/>
       <c r="K53" t="n">
-        <v>627</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="54">
@@ -1998,25 +2016,25 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>56142</v>
+        <v>75989</v>
       </c>
       <c r="C54" t="n">
-        <v>6192</v>
+        <v>11248</v>
       </c>
       <c r="D54" t="n">
-        <v>1561</v>
+        <v>2416</v>
       </c>
       <c r="E54" t="n">
-        <v>279</v>
+        <v>242</v>
       </c>
       <c r="F54" t="n">
-        <v>46</v>
+        <v>110</v>
       </c>
       <c r="G54" t="n">
         <v>54</v>
       </c>
       <c r="H54" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I54" t="n">
         <v>2</v>
@@ -2025,7 +2043,7 @@
         <v>0</v>
       </c>
       <c r="K54" t="n">
-        <v>64293</v>
+        <v>90079</v>
       </c>
     </row>
   </sheetData>
@@ -2101,20 +2119,20 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>932</v>
+        <v>883</v>
       </c>
       <c r="C2" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="D2" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="E2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F2" t="n">
         <v>5</v>
       </c>
-      <c r="F2" t="n">
-        <v>4</v>
-      </c>
       <c r="G2" t="n">
         <v>2</v>
       </c>
@@ -2125,7 +2143,7 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>957</v>
+        <v>919</v>
       </c>
     </row>
     <row r="3">
@@ -2135,19 +2153,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>673</v>
+        <v>652</v>
       </c>
       <c r="C3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3" t="n">
         <v>7</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3" t="n">
         <v>2</v>
@@ -2159,7 +2177,7 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>690</v>
+        <v>670</v>
       </c>
     </row>
     <row r="4">
@@ -2169,19 +2187,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5928</v>
+        <v>10033</v>
       </c>
       <c r="C4" t="n">
-        <v>1121</v>
+        <v>2529</v>
       </c>
       <c r="D4" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="E4" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G4" t="n">
         <v>4</v>
@@ -2193,7 +2211,7 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>7115</v>
+        <v>12648</v>
       </c>
     </row>
     <row r="5">
@@ -2203,19 +2221,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1373</v>
+        <v>2426</v>
       </c>
       <c r="C5" t="n">
-        <v>72</v>
+        <v>127</v>
       </c>
       <c r="D5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E5" t="n">
         <v>4</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" t="n">
         <v>2</v>
@@ -2227,7 +2245,7 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>1457</v>
+        <v>2567</v>
       </c>
     </row>
     <row r="6">
@@ -2237,16 +2255,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>860</v>
+        <v>1586</v>
       </c>
       <c r="C6" t="n">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="D6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
@@ -2261,7 +2279,7 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>898</v>
+        <v>1637</v>
       </c>
     </row>
     <row r="7">
@@ -2271,19 +2289,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>396</v>
+        <v>816</v>
       </c>
       <c r="C7" t="n">
         <v>4</v>
       </c>
       <c r="D7" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E7" t="n">
         <v>4</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -2295,7 +2313,7 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>410</v>
+        <v>833</v>
       </c>
     </row>
     <row r="8">
@@ -2305,19 +2323,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>432</v>
+        <v>635</v>
       </c>
       <c r="C8" t="n">
+        <v>8</v>
+      </c>
+      <c r="D8" t="n">
         <v>6</v>
       </c>
-      <c r="D8" t="n">
-        <v>1</v>
-      </c>
       <c r="E8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G8" t="n">
         <v>2</v>
@@ -2329,7 +2347,7 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>444</v>
+        <v>654</v>
       </c>
     </row>
     <row r="9">
@@ -2339,16 +2357,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>391</v>
+        <v>604</v>
       </c>
       <c r="C9" t="n">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="D9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
@@ -2363,7 +2381,7 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>410</v>
+        <v>632</v>
       </c>
     </row>
     <row r="10">
@@ -2373,7 +2391,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>59</v>
+        <v>84</v>
       </c>
       <c r="C10" t="n">
         <v>1</v>
@@ -2397,7 +2415,7 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>61</v>
+        <v>86</v>
       </c>
     </row>
     <row r="11">
@@ -2407,13 +2425,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>486</v>
+        <v>125</v>
       </c>
       <c r="C11" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E11" t="n">
         <v>2</v>
@@ -2431,7 +2449,7 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>496</v>
+        <v>141</v>
       </c>
     </row>
     <row r="12">
@@ -2441,31 +2459,31 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2845</v>
+        <v>4101</v>
       </c>
       <c r="C12" t="n">
-        <v>579</v>
+        <v>1095</v>
       </c>
       <c r="D12" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E12" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="F12" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="G12" t="n">
         <v>4</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>3468</v>
+        <v>5246</v>
       </c>
     </row>
     <row r="13">
@@ -2475,7 +2493,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>127</v>
+        <v>160</v>
       </c>
       <c r="C13" t="n">
         <v>4</v>
@@ -2499,7 +2517,7 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>133</v>
+        <v>166</v>
       </c>
     </row>
     <row r="14">
@@ -2509,13 +2527,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>129</v>
+        <v>52</v>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D14" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E14" t="n">
         <v>1</v>
@@ -2533,7 +2551,7 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>141</v>
+        <v>65</v>
       </c>
     </row>
     <row r="15">
@@ -2543,19 +2561,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>168</v>
+        <v>201</v>
       </c>
       <c r="C15" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D15" t="n">
         <v>2</v>
       </c>
       <c r="E15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
@@ -2567,7 +2585,7 @@
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>176</v>
+        <v>214</v>
       </c>
     </row>
     <row r="16">
@@ -2577,19 +2595,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>584</v>
+        <v>1063</v>
       </c>
       <c r="C16" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D16" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
@@ -2601,7 +2619,7 @@
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>601</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="17">
@@ -2611,10 +2629,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>156</v>
+        <v>176</v>
       </c>
       <c r="C17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D17" t="n">
         <v>1</v>
@@ -2635,7 +2653,7 @@
         <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>159</v>
+        <v>180</v>
       </c>
     </row>
     <row r="18">
@@ -2645,13 +2663,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>343</v>
+        <v>452</v>
       </c>
       <c r="C18" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
@@ -2669,7 +2687,7 @@
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>353</v>
+        <v>464</v>
       </c>
     </row>
     <row r="19">
@@ -2679,19 +2697,19 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2795</v>
+        <v>721</v>
       </c>
       <c r="C19" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D19" t="n">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="E19" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G19" t="n">
         <v>2</v>
@@ -2703,7 +2721,7 @@
         <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>2871</v>
+        <v>813</v>
       </c>
     </row>
     <row r="20">
@@ -2713,10 +2731,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>617</v>
+        <v>1126</v>
       </c>
       <c r="C20" t="n">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="D20" t="n">
         <v>2</v>
@@ -2725,7 +2743,7 @@
         <v>3</v>
       </c>
       <c r="F20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G20" t="n">
         <v>1</v>
@@ -2737,7 +2755,7 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>634</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="21">
@@ -2747,13 +2765,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>187</v>
+        <v>40</v>
       </c>
       <c r="C21" t="n">
         <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E21" t="n">
         <v>2</v>
@@ -2771,7 +2789,7 @@
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>191</v>
+        <v>46</v>
       </c>
     </row>
     <row r="22">
@@ -2781,10 +2799,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>502</v>
+        <v>617</v>
       </c>
       <c r="C22" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="D22" t="n">
         <v>5</v>
@@ -2805,7 +2823,7 @@
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>521</v>
+        <v>640</v>
       </c>
     </row>
     <row r="23">
@@ -2815,10 +2833,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>674</v>
+        <v>937</v>
       </c>
       <c r="C23" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="D23" t="n">
         <v>3</v>
@@ -2839,7 +2857,7 @@
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>689</v>
+        <v>956</v>
       </c>
     </row>
     <row r="24">
@@ -2849,13 +2867,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>844</v>
+        <v>919</v>
       </c>
       <c r="C24" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D24" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E24" t="n">
         <v>3</v>
@@ -2873,7 +2891,7 @@
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>877</v>
+        <v>954</v>
       </c>
     </row>
     <row r="25">
@@ -2883,19 +2901,19 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>73</v>
+        <v>178</v>
       </c>
       <c r="C25" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D25" t="n">
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G25" t="n">
         <v>0</v>
@@ -2907,7 +2925,7 @@
         <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>76</v>
+        <v>184</v>
       </c>
     </row>
     <row r="26">
@@ -2917,19 +2935,19 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>4045</v>
+        <v>4089</v>
       </c>
       <c r="C26" t="n">
-        <v>1823</v>
+        <v>2326</v>
       </c>
       <c r="D26" t="n">
-        <v>1185</v>
+        <v>1839</v>
       </c>
       <c r="E26" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F26" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G26" t="n">
         <v>4</v>
@@ -2941,7 +2959,7 @@
         <v>1</v>
       </c>
       <c r="J26" t="n">
-        <v>7089</v>
+        <v>8296</v>
       </c>
     </row>
     <row r="27">
@@ -2951,19 +2969,19 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1683</v>
+        <v>1121</v>
       </c>
       <c r="C27" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="D27" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E27" t="n">
         <v>7</v>
       </c>
       <c r="F27" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G27" t="n">
         <v>2</v>
@@ -2975,7 +2993,7 @@
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>1715</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="28">
@@ -2985,19 +3003,19 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>976</v>
+        <v>1377</v>
       </c>
       <c r="C28" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D28" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E28" t="n">
         <v>8</v>
       </c>
       <c r="F28" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G28" t="n">
         <v>1</v>
@@ -3009,7 +3027,7 @@
         <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>1026</v>
+        <v>1435</v>
       </c>
     </row>
     <row r="29">
@@ -3019,19 +3037,19 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>194</v>
+        <v>405</v>
       </c>
       <c r="C29" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E29" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F29" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G29" t="n">
         <v>1</v>
@@ -3043,7 +3061,7 @@
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>207</v>
+        <v>420</v>
       </c>
     </row>
     <row r="30">
@@ -3053,10 +3071,10 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>139</v>
+        <v>33</v>
       </c>
       <c r="C30" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D30" t="n">
         <v>0</v>
@@ -3077,7 +3095,7 @@
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>139</v>
+        <v>40</v>
       </c>
     </row>
     <row r="31">
@@ -3087,19 +3105,19 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>4902</v>
+        <v>7937</v>
       </c>
       <c r="C31" t="n">
-        <v>786</v>
+        <v>1781</v>
       </c>
       <c r="D31" t="n">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="E31" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F31" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G31" t="n">
         <v>5</v>
@@ -3111,7 +3129,7 @@
         <v>0</v>
       </c>
       <c r="J31" t="n">
-        <v>5746</v>
+        <v>9789</v>
       </c>
     </row>
     <row r="32">
@@ -3121,13 +3139,13 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>181</v>
+        <v>45</v>
       </c>
       <c r="C32" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D32" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E32" t="n">
         <v>2</v>
@@ -3145,7 +3163,7 @@
         <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>187</v>
+        <v>52</v>
       </c>
     </row>
     <row r="33">
@@ -3155,10 +3173,10 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>115</v>
+        <v>44</v>
       </c>
       <c r="C33" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D33" t="n">
         <v>2</v>
@@ -3179,7 +3197,7 @@
         <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>119</v>
+        <v>51</v>
       </c>
     </row>
     <row r="34">
@@ -3189,7 +3207,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>210</v>
+        <v>260</v>
       </c>
       <c r="C34" t="n">
         <v>1</v>
@@ -3213,7 +3231,7 @@
         <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>214</v>
+        <v>264</v>
       </c>
     </row>
     <row r="35">
@@ -3223,19 +3241,19 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>593</v>
+        <v>775</v>
       </c>
       <c r="C35" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D35" t="n">
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G35" t="n">
         <v>0</v>
@@ -3247,7 +3265,7 @@
         <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>608</v>
+        <v>791</v>
       </c>
     </row>
     <row r="36">
@@ -3257,19 +3275,19 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1172</v>
+        <v>2488</v>
       </c>
       <c r="C36" t="n">
-        <v>37</v>
+        <v>84</v>
       </c>
       <c r="D36" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E36" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F36" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G36" t="n">
         <v>2</v>
@@ -3281,7 +3299,7 @@
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>1217</v>
+        <v>2585</v>
       </c>
     </row>
     <row r="37">
@@ -3291,7 +3309,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>373</v>
+        <v>452</v>
       </c>
       <c r="C37" t="n">
         <v>5</v>
@@ -3315,7 +3333,7 @@
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>379</v>
+        <v>458</v>
       </c>
     </row>
     <row r="38">
@@ -3325,19 +3343,19 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>518</v>
+        <v>332</v>
       </c>
       <c r="C38" t="n">
         <v>1</v>
       </c>
       <c r="D38" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G38" t="n">
         <v>0</v>
@@ -3349,7 +3367,7 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>523</v>
+        <v>338</v>
       </c>
     </row>
     <row r="39">
@@ -3359,7 +3377,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>377</v>
+        <v>422</v>
       </c>
       <c r="C39" t="n">
         <v>8</v>
@@ -3383,7 +3401,7 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>393</v>
+        <v>438</v>
       </c>
     </row>
     <row r="40">
@@ -3393,19 +3411,19 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>210</v>
+        <v>442</v>
       </c>
       <c r="C40" t="n">
         <v>0</v>
       </c>
       <c r="D40" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E40" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G40" t="n">
         <v>1</v>
@@ -3417,7 +3435,7 @@
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>219</v>
+        <v>453</v>
       </c>
     </row>
     <row r="41">
@@ -3427,19 +3445,19 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>415</v>
+        <v>710</v>
       </c>
       <c r="C41" t="n">
+        <v>5</v>
+      </c>
+      <c r="D41" t="n">
+        <v>3</v>
+      </c>
+      <c r="E41" t="n">
         <v>4</v>
       </c>
-      <c r="D41" t="n">
-        <v>4</v>
-      </c>
-      <c r="E41" t="n">
-        <v>3</v>
-      </c>
       <c r="F41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G41" t="n">
         <v>0</v>
@@ -3451,7 +3469,7 @@
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>427</v>
+        <v>724</v>
       </c>
     </row>
     <row r="42">
@@ -3461,10 +3479,10 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>238</v>
+        <v>628</v>
       </c>
       <c r="C42" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D42" t="n">
         <v>1</v>
@@ -3473,7 +3491,7 @@
         <v>3</v>
       </c>
       <c r="F42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G42" t="n">
         <v>0</v>
@@ -3485,7 +3503,7 @@
         <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>247</v>
+        <v>637</v>
       </c>
     </row>
     <row r="43">
@@ -3495,19 +3513,19 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>535</v>
+        <v>981</v>
       </c>
       <c r="C43" t="n">
         <v>8</v>
       </c>
       <c r="D43" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E43" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G43" t="n">
         <v>0</v>
@@ -3519,7 +3537,7 @@
         <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>547</v>
+        <v>995</v>
       </c>
     </row>
     <row r="44">
@@ -3529,19 +3547,19 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>618</v>
+        <v>912</v>
       </c>
       <c r="C44" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D44" t="n">
         <v>6</v>
       </c>
       <c r="E44" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G44" t="n">
         <v>0</v>
@@ -3553,7 +3571,7 @@
         <v>1</v>
       </c>
       <c r="J44" t="n">
-        <v>649</v>
+        <v>946</v>
       </c>
     </row>
     <row r="45">
@@ -3563,19 +3581,19 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>295</v>
+        <v>510</v>
       </c>
       <c r="C45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E45" t="n">
         <v>2</v>
       </c>
       <c r="F45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G45" t="n">
         <v>0</v>
@@ -3587,7 +3605,7 @@
         <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>300</v>
+        <v>516</v>
       </c>
     </row>
     <row r="46">
@@ -3597,19 +3615,19 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="C46" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D46" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E46" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F46" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G46" t="n">
         <v>3</v>
@@ -3621,7 +3639,7 @@
         <v>0</v>
       </c>
       <c r="J46" t="n">
-        <v>578</v>
+        <v>591</v>
       </c>
     </row>
     <row r="47">
@@ -3631,13 +3649,13 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>222</v>
+        <v>85</v>
       </c>
       <c r="C47" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D47" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E47" t="n">
         <v>2</v>
@@ -3655,7 +3673,7 @@
         <v>0</v>
       </c>
       <c r="J47" t="n">
-        <v>227</v>
+        <v>95</v>
       </c>
     </row>
     <row r="48">
@@ -3665,19 +3683,19 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1537</v>
+        <v>2897</v>
       </c>
       <c r="C48" t="n">
-        <v>26</v>
+        <v>43</v>
       </c>
       <c r="D48" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E48" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F48" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G48" t="n">
         <v>1</v>
@@ -3689,7 +3707,7 @@
         <v>0</v>
       </c>
       <c r="J48" t="n">
-        <v>1585</v>
+        <v>2968</v>
       </c>
     </row>
     <row r="49">
@@ -3699,10 +3717,10 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>460</v>
+        <v>611</v>
       </c>
       <c r="C49" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D49" t="n">
         <v>2</v>
@@ -3723,7 +3741,7 @@
         <v>0</v>
       </c>
       <c r="J49" t="n">
-        <v>477</v>
+        <v>632</v>
       </c>
     </row>
     <row r="50">
@@ -3733,10 +3751,10 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>197</v>
+        <v>348</v>
       </c>
       <c r="C50" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="D50" t="n">
         <v>3</v>
@@ -3757,7 +3775,7 @@
         <v>0</v>
       </c>
       <c r="J50" t="n">
-        <v>204</v>
+        <v>362</v>
       </c>
     </row>
     <row r="51">
@@ -3767,16 +3785,16 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>329</v>
+        <v>790</v>
       </c>
       <c r="C51" t="n">
         <v>1</v>
       </c>
       <c r="D51" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E51" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F51" t="n">
         <v>0</v>
@@ -3791,7 +3809,7 @@
         <v>0</v>
       </c>
       <c r="J51" t="n">
-        <v>333</v>
+        <v>794</v>
       </c>
     </row>
     <row r="52">
@@ -3801,19 +3819,19 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>3791</v>
+        <v>5741</v>
       </c>
       <c r="C52" t="n">
-        <v>616</v>
+        <v>1244</v>
       </c>
       <c r="D52" t="n">
-        <v>56</v>
+        <v>124</v>
       </c>
       <c r="E52" t="n">
         <v>10</v>
       </c>
       <c r="F52" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G52" t="n">
         <v>2</v>
@@ -3825,7 +3843,7 @@
         <v>0</v>
       </c>
       <c r="J52" t="n">
-        <v>4480</v>
+        <v>7127</v>
       </c>
     </row>
     <row r="53">
@@ -3835,13 +3853,13 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>418</v>
+        <v>395</v>
       </c>
       <c r="C53" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D53" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E53" t="n">
         <v>0</v>
@@ -3859,7 +3877,7 @@
         <v>0</v>
       </c>
       <c r="J53" t="n">
-        <v>427</v>
+        <v>412</v>
       </c>
     </row>
     <row r="54">
@@ -3869,10 +3887,10 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>144</v>
+        <v>211</v>
       </c>
       <c r="C54" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D54" t="n">
         <v>0</v>
@@ -3893,7 +3911,7 @@
         <v>0</v>
       </c>
       <c r="J54" t="n">
-        <v>147</v>
+        <v>216</v>
       </c>
     </row>
     <row r="55">
@@ -3903,19 +3921,19 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>3431</v>
+        <v>5242</v>
       </c>
       <c r="C55" t="n">
-        <v>653</v>
+        <v>1373</v>
       </c>
       <c r="D55" t="n">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="E55" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F55" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G55" t="n">
         <v>2</v>
@@ -3927,7 +3945,7 @@
         <v>0</v>
       </c>
       <c r="J55" t="n">
-        <v>4117</v>
+        <v>6658</v>
       </c>
     </row>
     <row r="56">
@@ -3937,19 +3955,19 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>76</v>
+        <v>104</v>
       </c>
       <c r="C56" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D56" t="n">
         <v>1</v>
       </c>
       <c r="E56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F56" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G56" t="n">
         <v>1</v>
@@ -3961,7 +3979,7 @@
         <v>0</v>
       </c>
       <c r="J56" t="n">
-        <v>87</v>
+        <v>118</v>
       </c>
     </row>
     <row r="57">
@@ -3971,13 +3989,13 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>345</v>
+        <v>410</v>
       </c>
       <c r="C57" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="D57" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E57" t="n">
         <v>1</v>
@@ -3995,7 +4013,7 @@
         <v>0</v>
       </c>
       <c r="J57" t="n">
-        <v>361</v>
+        <v>433</v>
       </c>
     </row>
     <row r="58">
@@ -4005,13 +4023,13 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>183</v>
+        <v>35</v>
       </c>
       <c r="C58" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D58" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E58" t="n">
         <v>1</v>
@@ -4029,7 +4047,7 @@
         <v>0</v>
       </c>
       <c r="J58" t="n">
-        <v>189</v>
+        <v>45</v>
       </c>
     </row>
     <row r="59">
@@ -4039,10 +4057,10 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>128</v>
+        <v>42</v>
       </c>
       <c r="C59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D59" t="n">
         <v>0</v>
@@ -4063,7 +4081,7 @@
         <v>0</v>
       </c>
       <c r="J59" t="n">
-        <v>133</v>
+        <v>46</v>
       </c>
     </row>
     <row r="60">
@@ -4073,17 +4091,17 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>360</v>
+        <v>906</v>
       </c>
       <c r="C60" t="n">
+        <v>4</v>
+      </c>
+      <c r="D60" t="n">
+        <v>5</v>
+      </c>
+      <c r="E60" t="n">
         <v>6</v>
       </c>
-      <c r="D60" t="n">
-        <v>4</v>
-      </c>
-      <c r="E60" t="n">
-        <v>4</v>
-      </c>
       <c r="F60" t="n">
         <v>0</v>
       </c>
@@ -4097,7 +4115,7 @@
         <v>0</v>
       </c>
       <c r="J60" t="n">
-        <v>374</v>
+        <v>921</v>
       </c>
     </row>
     <row r="61">
@@ -4107,19 +4125,19 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>1106</v>
+        <v>1021</v>
       </c>
       <c r="C61" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="D61" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E61" t="n">
         <v>5</v>
       </c>
       <c r="F61" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G61" t="n">
         <v>1</v>
@@ -4131,7 +4149,7 @@
         <v>0</v>
       </c>
       <c r="J61" t="n">
-        <v>1159</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="62">
@@ -4141,19 +4159,19 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>365</v>
+        <v>702</v>
       </c>
       <c r="C62" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D62" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F62" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G62" t="n">
         <v>0</v>
@@ -4165,7 +4183,7 @@
         <v>0</v>
       </c>
       <c r="J62" t="n">
-        <v>377</v>
+        <v>725</v>
       </c>
     </row>
     <row r="63">
@@ -4175,19 +4193,19 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>2090</v>
+        <v>2164</v>
       </c>
       <c r="C63" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D63" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E63" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F63" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G63" t="n">
         <v>2</v>
@@ -4199,7 +4217,7 @@
         <v>0</v>
       </c>
       <c r="J63" t="n">
-        <v>2131</v>
+        <v>2211</v>
       </c>
     </row>
     <row r="64">
@@ -4209,19 +4227,19 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>1036</v>
+        <v>1168</v>
       </c>
       <c r="C64" t="n">
-        <v>73</v>
+        <v>138</v>
       </c>
       <c r="D64" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E64" t="n">
         <v>3</v>
       </c>
       <c r="F64" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G64" t="n">
         <v>3</v>
@@ -4233,7 +4251,7 @@
         <v>0</v>
       </c>
       <c r="J64" t="n">
-        <v>1128</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="65">
@@ -4243,31 +4261,31 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>56142</v>
+        <v>75989</v>
       </c>
       <c r="C65" t="n">
-        <v>6192</v>
+        <v>11248</v>
       </c>
       <c r="D65" t="n">
-        <v>1561</v>
+        <v>2416</v>
       </c>
       <c r="E65" t="n">
-        <v>279</v>
+        <v>242</v>
       </c>
       <c r="F65" t="n">
-        <v>46</v>
+        <v>110</v>
       </c>
       <c r="G65" t="n">
         <v>54</v>
       </c>
       <c r="H65" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I65" t="n">
         <v>2</v>
       </c>
       <c r="J65" t="n">
-        <v>64293</v>
+        <v>90079</v>
       </c>
     </row>
   </sheetData>
@@ -4343,19 +4361,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5420</v>
+        <v>9748</v>
       </c>
       <c r="C2" t="n">
-        <v>1099</v>
+        <v>2516</v>
       </c>
       <c r="D2" t="n">
-        <v>40</v>
+        <v>61</v>
       </c>
       <c r="E2" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G2" t="n">
         <v>4</v>
@@ -4367,7 +4385,7 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>6582</v>
+        <v>12348</v>
       </c>
     </row>
     <row r="3">
@@ -4377,19 +4395,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2569</v>
+        <v>3913</v>
       </c>
       <c r="C3" t="n">
-        <v>573</v>
+        <v>1098</v>
       </c>
       <c r="D3" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E3" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F3" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="G3" t="n">
         <v>3</v>
@@ -4401,7 +4419,7 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>3183</v>
+        <v>5058</v>
       </c>
     </row>
     <row r="4">
@@ -4411,16 +4429,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2593</v>
+        <v>3409</v>
       </c>
       <c r="C4" t="n">
-        <v>1796</v>
+        <v>2245</v>
       </c>
       <c r="D4" t="n">
-        <v>1241</v>
+        <v>1905</v>
       </c>
       <c r="E4" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="F4" t="n">
         <v>2</v>
@@ -4435,7 +4453,7 @@
         <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>5659</v>
+        <v>7592</v>
       </c>
     </row>
     <row r="5">
@@ -4445,10 +4463,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>117</v>
+        <v>195</v>
       </c>
       <c r="C5" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="D5" t="n">
         <v>4</v>
@@ -4469,7 +4487,7 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>145</v>
+        <v>229</v>
       </c>
     </row>
     <row r="6">
@@ -4479,19 +4497,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1525</v>
+        <v>2863</v>
       </c>
       <c r="C6" t="n">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -4503,7 +4521,7 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>1566</v>
+        <v>2925</v>
       </c>
     </row>
     <row r="7">
@@ -4513,19 +4531,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>939</v>
+        <v>1918</v>
       </c>
       <c r="C7" t="n">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E7" t="n">
         <v>4</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" t="n">
         <v>2</v>
@@ -4537,7 +4555,7 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>980</v>
+        <v>1967</v>
       </c>
     </row>
     <row r="8">
@@ -4547,16 +4565,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>872</v>
+        <v>1595</v>
       </c>
       <c r="C8" t="n">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="D8" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
@@ -4571,7 +4589,7 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>911</v>
+        <v>1647</v>
       </c>
     </row>
     <row r="9">
@@ -4581,19 +4599,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>521</v>
+        <v>960</v>
       </c>
       <c r="C9" t="n">
         <v>8</v>
       </c>
       <c r="D9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -4605,7 +4623,7 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>533</v>
+        <v>974</v>
       </c>
     </row>
     <row r="10">
@@ -4615,19 +4633,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>347</v>
+        <v>694</v>
       </c>
       <c r="C10" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -4639,7 +4657,7 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>359</v>
+        <v>716</v>
       </c>
     </row>
     <row r="11">
@@ -4649,19 +4667,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2689</v>
+        <v>2694</v>
       </c>
       <c r="C11" t="n">
+        <v>18</v>
+      </c>
+      <c r="D11" t="n">
+        <v>16</v>
+      </c>
+      <c r="E11" t="n">
         <v>15</v>
       </c>
-      <c r="D11" t="n">
-        <v>12</v>
-      </c>
-      <c r="E11" t="n">
-        <v>18</v>
-      </c>
       <c r="F11" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G11" t="n">
         <v>4</v>
@@ -4673,7 +4691,7 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>2743</v>
+        <v>2756</v>
       </c>
     </row>
     <row r="12">
@@ -4683,10 +4701,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="C12" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D12" t="n">
         <v>1</v>
@@ -4707,7 +4725,7 @@
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>80</v>
+        <v>94</v>
       </c>
     </row>
     <row r="13">
@@ -4717,10 +4735,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C13" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
@@ -4741,7 +4759,7 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>134</v>
+        <v>144</v>
       </c>
     </row>
     <row r="14">
@@ -4751,7 +4769,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="C14" t="n">
         <v>1</v>
@@ -4775,7 +4793,7 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15">
@@ -4785,13 +4803,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="C15" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
         <v>1</v>
@@ -4809,7 +4827,7 @@
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>107</v>
+        <v>121</v>
       </c>
     </row>
     <row r="16">
@@ -4819,10 +4837,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="C16" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
@@ -4831,19 +4849,19 @@
         <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G16" t="n">
         <v>1</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I16" t="n">
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>97</v>
+        <v>109</v>
       </c>
     </row>
     <row r="17">
@@ -4853,10 +4871,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="C17" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
@@ -4877,7 +4895,7 @@
         <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>123</v>
+        <v>137</v>
       </c>
     </row>
     <row r="18">
@@ -4887,10 +4905,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C18" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
@@ -4911,7 +4929,7 @@
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="19">
@@ -4921,19 +4939,19 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="C19" t="n">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="D19" t="n">
         <v>2</v>
       </c>
       <c r="E19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
@@ -4945,7 +4963,7 @@
         <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>113</v>
+        <v>127</v>
       </c>
     </row>
     <row r="20">
@@ -4955,10 +4973,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="C20" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
@@ -4979,7 +4997,7 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>65</v>
+        <v>72</v>
       </c>
     </row>
     <row r="21">
@@ -4989,10 +5007,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="C21" t="n">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
@@ -5013,7 +5031,7 @@
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>154</v>
+        <v>171</v>
       </c>
     </row>
     <row r="22">
@@ -5023,10 +5041,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="C22" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
@@ -5047,7 +5065,7 @@
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>103</v>
+        <v>123</v>
       </c>
     </row>
     <row r="23">
@@ -5057,13 +5075,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>180</v>
+        <v>202</v>
       </c>
       <c r="C23" t="n">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="D23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -5081,7 +5099,7 @@
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>205</v>
+        <v>238</v>
       </c>
     </row>
     <row r="24">
@@ -5091,7 +5109,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>235</v>
+        <v>292</v>
       </c>
       <c r="C24" t="n">
         <v>9</v>
@@ -5100,10 +5118,10 @@
         <v>6</v>
       </c>
       <c r="E24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G24" t="n">
         <v>1</v>
@@ -5115,7 +5133,7 @@
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>256</v>
+        <v>314</v>
       </c>
     </row>
     <row r="25">
@@ -5125,19 +5143,19 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C25" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G25" t="n">
         <v>0</v>
@@ -5149,7 +5167,7 @@
         <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>66</v>
+        <v>77</v>
       </c>
     </row>
     <row r="26">
@@ -5159,19 +5177,19 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1782</v>
+        <v>3608</v>
       </c>
       <c r="C26" t="n">
-        <v>46</v>
+        <v>110</v>
       </c>
       <c r="D26" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E26" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F26" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G26" t="n">
         <v>2</v>
@@ -5183,7 +5201,7 @@
         <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>1841</v>
+        <v>3737</v>
       </c>
     </row>
     <row r="27">
@@ -5193,19 +5211,19 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>614</v>
+        <v>1273</v>
       </c>
       <c r="C27" t="n">
         <v>4</v>
       </c>
       <c r="D27" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E27" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F27" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G27" t="n">
         <v>1</v>
@@ -5217,7 +5235,7 @@
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>633</v>
+        <v>1295</v>
       </c>
     </row>
     <row r="28">
@@ -5227,19 +5245,19 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>3201</v>
+        <v>3263</v>
       </c>
       <c r="C28" t="n">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="D28" t="n">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="E28" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F28" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="G28" t="n">
         <v>12</v>
@@ -5251,7 +5269,7 @@
         <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>3301</v>
+        <v>3405</v>
       </c>
     </row>
     <row r="29">
@@ -5261,19 +5279,19 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>808</v>
+        <v>374</v>
       </c>
       <c r="C29" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D29" t="n">
         <v>12</v>
       </c>
       <c r="E29" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G29" t="n">
         <v>2</v>
@@ -5285,7 +5303,7 @@
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>854</v>
+        <v>414</v>
       </c>
     </row>
     <row r="30">
@@ -5295,19 +5313,19 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>774</v>
+        <v>1470</v>
       </c>
       <c r="C30" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D30" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E30" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F30" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G30" t="n">
         <v>1</v>
@@ -5319,7 +5337,7 @@
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>797</v>
+        <v>1499</v>
       </c>
     </row>
     <row r="31">
@@ -5329,13 +5347,13 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>4551</v>
+        <v>935</v>
       </c>
       <c r="C31" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D31" t="n">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="E31" t="n">
         <v>15</v>
@@ -5353,7 +5371,7 @@
         <v>1</v>
       </c>
       <c r="J31" t="n">
-        <v>4604</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="32">
@@ -5363,19 +5381,19 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>6929</v>
+        <v>8965</v>
       </c>
       <c r="C32" t="n">
-        <v>71</v>
+        <v>92</v>
       </c>
       <c r="D32" t="n">
+        <v>13</v>
+      </c>
+      <c r="E32" t="n">
         <v>14</v>
       </c>
-      <c r="E32" t="n">
-        <v>15</v>
-      </c>
       <c r="F32" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G32" t="n">
         <v>2</v>
@@ -5387,7 +5405,7 @@
         <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>7036</v>
+        <v>9093</v>
       </c>
     </row>
     <row r="33">
@@ -5397,19 +5415,19 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1701</v>
+        <v>791</v>
       </c>
       <c r="C33" t="n">
-        <v>50</v>
+        <v>108</v>
       </c>
       <c r="D33" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="E33" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G33" t="n">
         <v>1</v>
@@ -5421,7 +5439,7 @@
         <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>1781</v>
+        <v>937</v>
       </c>
     </row>
     <row r="34">
@@ -5431,19 +5449,19 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>2186</v>
+        <v>1433</v>
       </c>
       <c r="C34" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="D34" t="n">
+        <v>9</v>
+      </c>
+      <c r="E34" t="n">
         <v>8</v>
       </c>
-      <c r="E34" t="n">
-        <v>9</v>
-      </c>
       <c r="F34" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G34" t="n">
         <v>2</v>
@@ -5455,7 +5473,7 @@
         <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>2219</v>
+        <v>1461</v>
       </c>
     </row>
     <row r="35">
@@ -5465,19 +5483,19 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>709</v>
+        <v>1215</v>
       </c>
       <c r="C35" t="n">
+        <v>8</v>
+      </c>
+      <c r="D35" t="n">
+        <v>3</v>
+      </c>
+      <c r="E35" t="n">
         <v>6</v>
       </c>
-      <c r="D35" t="n">
-        <v>5</v>
-      </c>
-      <c r="E35" t="n">
-        <v>5</v>
-      </c>
       <c r="F35" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G35" t="n">
         <v>0</v>
@@ -5489,7 +5507,7 @@
         <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>726</v>
+        <v>1235</v>
       </c>
     </row>
     <row r="36">
@@ -5499,19 +5517,19 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>855</v>
+        <v>2262</v>
       </c>
       <c r="C36" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D36" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E36" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G36" t="n">
         <v>0</v>
@@ -5523,7 +5541,7 @@
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>878</v>
+        <v>2285</v>
       </c>
     </row>
     <row r="37">
@@ -5533,19 +5551,19 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1162</v>
+        <v>1073</v>
       </c>
       <c r="C37" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="D37" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E37" t="n">
         <v>5</v>
       </c>
       <c r="F37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G37" t="n">
         <v>1</v>
@@ -5557,7 +5575,7 @@
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>1204</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="38">
@@ -5567,19 +5585,19 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>5063</v>
+        <v>8501</v>
       </c>
       <c r="C38" t="n">
-        <v>877</v>
+        <v>1947</v>
       </c>
       <c r="D38" t="n">
-        <v>27</v>
+        <v>67</v>
       </c>
       <c r="E38" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="F38" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G38" t="n">
         <v>5</v>
@@ -5591,7 +5609,7 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>6000</v>
+        <v>10549</v>
       </c>
     </row>
     <row r="39">
@@ -5601,19 +5619,19 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>615</v>
+        <v>1110</v>
       </c>
       <c r="C39" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="D39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G39" t="n">
         <v>1</v>
@@ -5625,7 +5643,7 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>627</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="40">
@@ -5635,19 +5653,19 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>2964</v>
+        <v>4746</v>
       </c>
       <c r="C40" t="n">
-        <v>539</v>
+        <v>1106</v>
       </c>
       <c r="D40" t="n">
-        <v>53</v>
+        <v>93</v>
       </c>
       <c r="E40" t="n">
         <v>9</v>
       </c>
       <c r="F40" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G40" t="n">
         <v>2</v>
@@ -5659,7 +5677,7 @@
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>3571</v>
+        <v>5961</v>
       </c>
     </row>
     <row r="41">
@@ -5669,19 +5687,19 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>3288</v>
+        <v>5467</v>
       </c>
       <c r="C41" t="n">
-        <v>662</v>
+        <v>1434</v>
       </c>
       <c r="D41" t="n">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="E41" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F41" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G41" t="n">
         <v>2</v>
@@ -5693,7 +5711,7 @@
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>3981</v>
+        <v>6944</v>
       </c>
     </row>
     <row r="42">
@@ -5703,31 +5721,31 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>56142</v>
+        <v>75989</v>
       </c>
       <c r="C42" t="n">
-        <v>6192</v>
+        <v>11248</v>
       </c>
       <c r="D42" t="n">
-        <v>1561</v>
+        <v>2416</v>
       </c>
       <c r="E42" t="n">
-        <v>279</v>
+        <v>242</v>
       </c>
       <c r="F42" t="n">
-        <v>46</v>
+        <v>110</v>
       </c>
       <c r="G42" t="n">
         <v>54</v>
       </c>
       <c r="H42" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I42" t="n">
         <v>2</v>
       </c>
       <c r="J42" t="n">
-        <v>64293</v>
+        <v>90079</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add metabase session token expiration notification and dashboard warnings
</commit_message>
<xml_diff>
--- a/BaoCao_TonKho.xlsx
+++ b/BaoCao_TonKho.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>05/06/2026 00:38:37</t>
+          <t>05/06/2026 00:52:34</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -579,25 +579,25 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>10724</v>
+        <v>10229</v>
       </c>
       <c r="C7" t="n">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="D7" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E7" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F7" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -606,7 +606,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>10985</v>
+        <v>10482</v>
       </c>
     </row>
     <row r="8">
@@ -616,19 +616,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2863</v>
+        <v>3010</v>
       </c>
       <c r="C8" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D8" t="n">
         <v>8</v>
       </c>
       <c r="E8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
@@ -637,7 +637,7 @@
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="n">
-        <v>2925</v>
+        <v>3074</v>
       </c>
     </row>
     <row r="9">
@@ -647,16 +647,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1918</v>
+        <v>588</v>
       </c>
       <c r="C9" t="n">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="D9" t="n">
         <v>5</v>
       </c>
       <c r="E9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
         <v>1</v>
@@ -668,7 +668,7 @@
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="n">
-        <v>1967</v>
+        <v>617</v>
       </c>
     </row>
     <row r="10">
@@ -678,10 +678,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1595</v>
+        <v>1712</v>
       </c>
       <c r="C10" t="n">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="D10" t="n">
         <v>11</v>
@@ -695,7 +695,7 @@
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="n">
-        <v>1647</v>
+        <v>1771</v>
       </c>
     </row>
     <row r="11">
@@ -705,10 +705,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>960</v>
+        <v>1021</v>
       </c>
       <c r="C11" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D11" t="n">
         <v>3</v>
@@ -724,7 +724,7 @@
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="n">
-        <v>974</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="12">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>694</v>
+        <v>743</v>
       </c>
       <c r="C12" t="n">
         <v>17</v>
@@ -742,18 +742,16 @@
       <c r="D12" t="n">
         <v>3</v>
       </c>
-      <c r="E12" t="n">
-        <v>1</v>
-      </c>
+      <c r="E12" t="inlineStr"/>
       <c r="F12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="n">
-        <v>716</v>
+        <v>765</v>
       </c>
     </row>
     <row r="13">
@@ -763,30 +761,30 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2694</v>
+        <v>3155</v>
       </c>
       <c r="C13" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D13" t="n">
+        <v>15</v>
+      </c>
+      <c r="E13" t="n">
         <v>16</v>
-      </c>
-      <c r="E13" t="n">
-        <v>15</v>
       </c>
       <c r="F13" t="n">
         <v>7</v>
       </c>
       <c r="G13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="n">
-        <v>2756</v>
+        <v>3218</v>
       </c>
     </row>
     <row r="14">
@@ -796,13 +794,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1514</v>
+        <v>1500</v>
       </c>
       <c r="C14" t="n">
-        <v>266</v>
+        <v>307</v>
       </c>
       <c r="D14" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E14" t="n">
         <v>6</v>
@@ -823,7 +821,7 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>1812</v>
+        <v>1840</v>
       </c>
     </row>
     <row r="15">
@@ -833,10 +831,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C15" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D15" t="n">
         <v>1</v>
@@ -858,10 +856,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C16" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
@@ -883,7 +881,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C17" t="n">
         <v>1</v>
@@ -898,7 +896,7 @@
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="18">
@@ -908,10 +906,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C18" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D18" t="n">
         <v>1</v>
@@ -925,7 +923,7 @@
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="n">
-        <v>121</v>
+        <v>125</v>
       </c>
     </row>
     <row r="19">
@@ -935,10 +933,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C19" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="n">
@@ -964,10 +962,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="C20" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
@@ -989,10 +987,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C21" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
@@ -1016,13 +1014,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C22" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="n">
@@ -1033,7 +1031,7 @@
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="n">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="23">
@@ -1043,10 +1041,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C23" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
@@ -1058,7 +1056,7 @@
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="24">
@@ -1068,10 +1066,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="C24" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr"/>
@@ -1081,7 +1079,7 @@
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="n">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="25">
@@ -1091,10 +1089,10 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="C25" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr"/>
@@ -1104,7 +1102,7 @@
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="26">
@@ -1114,10 +1112,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="C26" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="D26" t="n">
         <v>2</v>
@@ -1131,7 +1129,7 @@
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="n">
-        <v>238</v>
+        <v>243</v>
       </c>
     </row>
     <row r="27">
@@ -1141,7 +1139,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>292</v>
+        <v>302</v>
       </c>
       <c r="C27" t="n">
         <v>9</v>
@@ -1162,7 +1160,7 @@
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="n">
-        <v>314</v>
+        <v>324</v>
       </c>
     </row>
     <row r="28">
@@ -1197,10 +1195,10 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>195</v>
+        <v>225</v>
       </c>
       <c r="C29" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D29" t="n">
         <v>4</v>
@@ -1224,7 +1222,7 @@
         <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>229</v>
+        <v>260</v>
       </c>
     </row>
     <row r="30">
@@ -1234,10 +1232,10 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>195</v>
+        <v>225</v>
       </c>
       <c r="C30" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D30" t="n">
         <v>4</v>
@@ -1255,7 +1253,7 @@
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="n">
-        <v>229</v>
+        <v>260</v>
       </c>
     </row>
     <row r="31">
@@ -1265,19 +1263,19 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>26662</v>
+        <v>28073</v>
       </c>
       <c r="C31" t="n">
-        <v>436</v>
+        <v>486</v>
       </c>
       <c r="D31" t="n">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E31" t="n">
-        <v>119</v>
+        <v>110</v>
       </c>
       <c r="F31" t="n">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="G31" t="n">
         <v>25</v>
@@ -1292,7 +1290,7 @@
         <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>27470</v>
+        <v>28932</v>
       </c>
     </row>
     <row r="32">
@@ -1302,10 +1300,10 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>3608</v>
+        <v>3791</v>
       </c>
       <c r="C32" t="n">
-        <v>110</v>
+        <v>140</v>
       </c>
       <c r="D32" t="n">
         <v>6</v>
@@ -1323,7 +1321,7 @@
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="n">
-        <v>3737</v>
+        <v>3950</v>
       </c>
     </row>
     <row r="33">
@@ -1333,19 +1331,19 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1273</v>
+        <v>1411</v>
       </c>
       <c r="C33" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D33" t="n">
         <v>5</v>
       </c>
       <c r="E33" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F33" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G33" t="n">
         <v>1</v>
@@ -1356,7 +1354,7 @@
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="n">
-        <v>1295</v>
+        <v>1434</v>
       </c>
     </row>
     <row r="34">
@@ -1366,19 +1364,19 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>3263</v>
+        <v>3922</v>
       </c>
       <c r="C34" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D34" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E34" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F34" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G34" t="n">
         <v>12</v>
@@ -1387,7 +1385,7 @@
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="n">
-        <v>3405</v>
+        <v>4066</v>
       </c>
     </row>
     <row r="35">
@@ -1397,19 +1395,19 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>374</v>
+        <v>418</v>
       </c>
       <c r="C35" t="n">
         <v>8</v>
       </c>
       <c r="D35" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G35" t="n">
         <v>2</v>
@@ -1420,7 +1418,7 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="n">
-        <v>414</v>
+        <v>458</v>
       </c>
     </row>
     <row r="36">
@@ -1430,7 +1428,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1470</v>
+        <v>1572</v>
       </c>
       <c r="C36" t="n">
         <v>13</v>
@@ -1439,10 +1437,10 @@
         <v>5</v>
       </c>
       <c r="E36" t="n">
+        <v>4</v>
+      </c>
+      <c r="F36" t="n">
         <v>6</v>
-      </c>
-      <c r="F36" t="n">
-        <v>4</v>
       </c>
       <c r="G36" t="n">
         <v>1</v>
@@ -1451,7 +1449,7 @@
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="n">
-        <v>1499</v>
+        <v>1601</v>
       </c>
     </row>
     <row r="37">
@@ -1461,10 +1459,10 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>935</v>
+        <v>1220</v>
       </c>
       <c r="C37" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D37" t="n">
         <v>36</v>
@@ -1482,7 +1480,7 @@
       </c>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="n">
-        <v>1013</v>
+        <v>1294</v>
       </c>
     </row>
     <row r="38">
@@ -1492,19 +1490,19 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>8965</v>
+        <v>9302</v>
       </c>
       <c r="C38" t="n">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="D38" t="n">
         <v>13</v>
       </c>
       <c r="E38" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F38" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G38" t="n">
         <v>2</v>
@@ -1513,7 +1511,7 @@
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="n">
-        <v>9093</v>
+        <v>9441</v>
       </c>
     </row>
     <row r="39">
@@ -1523,19 +1521,19 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>791</v>
+        <v>948</v>
       </c>
       <c r="C39" t="n">
         <v>108</v>
       </c>
       <c r="D39" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E39" t="n">
         <v>10</v>
       </c>
       <c r="F39" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G39" t="n">
         <v>1</v>
@@ -1546,7 +1544,7 @@
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="n">
-        <v>937</v>
+        <v>1093</v>
       </c>
     </row>
     <row r="40">
@@ -1556,19 +1554,19 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1433</v>
+        <v>1599</v>
       </c>
       <c r="C40" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="D40" t="n">
         <v>9</v>
       </c>
       <c r="E40" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F40" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G40" t="n">
         <v>2</v>
@@ -1577,7 +1575,7 @@
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="n">
-        <v>1461</v>
+        <v>1635</v>
       </c>
     </row>
     <row r="41">
@@ -1587,19 +1585,19 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1215</v>
+        <v>231</v>
       </c>
       <c r="C41" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D41" t="n">
         <v>3</v>
       </c>
       <c r="E41" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F41" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="n">
@@ -1608,7 +1606,7 @@
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="n">
-        <v>1235</v>
+        <v>248</v>
       </c>
     </row>
     <row r="42">
@@ -1618,13 +1616,13 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>2262</v>
+        <v>2483</v>
       </c>
       <c r="C42" t="n">
         <v>8</v>
       </c>
       <c r="D42" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E42" t="n">
         <v>11</v>
@@ -1637,7 +1635,7 @@
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="n">
-        <v>2285</v>
+        <v>2507</v>
       </c>
     </row>
     <row r="43">
@@ -1647,10 +1645,10 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>1073</v>
+        <v>1176</v>
       </c>
       <c r="C43" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="D43" t="n">
         <v>8</v>
@@ -1668,7 +1666,7 @@
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="n">
-        <v>1096</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="44">
@@ -1678,19 +1676,19 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>3409</v>
+        <v>3394</v>
       </c>
       <c r="C44" t="n">
-        <v>2245</v>
+        <v>2273</v>
       </c>
       <c r="D44" t="n">
-        <v>1905</v>
+        <v>1964</v>
       </c>
       <c r="E44" t="n">
         <v>23</v>
       </c>
       <c r="F44" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G44" t="n">
         <v>4</v>
@@ -1705,7 +1703,7 @@
         <v>0</v>
       </c>
       <c r="K44" t="n">
-        <v>7592</v>
+        <v>7665</v>
       </c>
     </row>
     <row r="45">
@@ -1715,19 +1713,19 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>3409</v>
+        <v>3394</v>
       </c>
       <c r="C45" t="n">
-        <v>2245</v>
+        <v>2273</v>
       </c>
       <c r="D45" t="n">
-        <v>1905</v>
+        <v>1964</v>
       </c>
       <c r="E45" t="n">
         <v>23</v>
       </c>
       <c r="F45" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G45" t="n">
         <v>4</v>
@@ -1740,7 +1738,7 @@
       </c>
       <c r="J45" t="inlineStr"/>
       <c r="K45" t="n">
-        <v>7592</v>
+        <v>7665</v>
       </c>
     </row>
     <row r="46">
@@ -1750,19 +1748,19 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>32375</v>
+        <v>32857</v>
       </c>
       <c r="C46" t="n">
-        <v>8101</v>
+        <v>8149</v>
       </c>
       <c r="D46" t="n">
-        <v>272</v>
+        <v>314</v>
       </c>
       <c r="E46" t="n">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="F46" t="n">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="G46" t="n">
         <v>16</v>
@@ -1777,7 +1775,7 @@
         <v>0</v>
       </c>
       <c r="K46" t="n">
-        <v>40860</v>
+        <v>41433</v>
       </c>
     </row>
     <row r="47">
@@ -1787,19 +1785,19 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>9748</v>
+        <v>10035</v>
       </c>
       <c r="C47" t="n">
-        <v>2516</v>
+        <v>2579</v>
       </c>
       <c r="D47" t="n">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="E47" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F47" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G47" t="n">
         <v>4</v>
@@ -1810,7 +1808,7 @@
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="n">
-        <v>12348</v>
+        <v>12706</v>
       </c>
     </row>
     <row r="48">
@@ -1820,19 +1818,19 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>3913</v>
+        <v>3997</v>
       </c>
       <c r="C48" t="n">
-        <v>1098</v>
+        <v>1124</v>
       </c>
       <c r="D48" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="E48" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F48" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G48" t="n">
         <v>3</v>
@@ -1841,7 +1839,7 @@
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="n">
-        <v>5058</v>
+        <v>5173</v>
       </c>
     </row>
     <row r="49">
@@ -1851,19 +1849,19 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>8501</v>
+        <v>8380</v>
       </c>
       <c r="C49" t="n">
-        <v>1947</v>
+        <v>1840</v>
       </c>
       <c r="D49" t="n">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="E49" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F49" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="G49" t="n">
         <v>5</v>
@@ -1874,7 +1872,7 @@
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="n">
-        <v>10549</v>
+        <v>10330</v>
       </c>
     </row>
     <row r="50">
@@ -1884,19 +1882,19 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>4746</v>
+        <v>4855</v>
       </c>
       <c r="C50" t="n">
-        <v>1106</v>
+        <v>1129</v>
       </c>
       <c r="D50" t="n">
-        <v>93</v>
+        <v>107</v>
       </c>
       <c r="E50" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F50" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G50" t="n">
         <v>2</v>
@@ -1907,7 +1905,7 @@
       <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr"/>
       <c r="K50" t="n">
-        <v>5961</v>
+        <v>6107</v>
       </c>
     </row>
     <row r="51">
@@ -1917,19 +1915,19 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>5467</v>
+        <v>5590</v>
       </c>
       <c r="C51" t="n">
-        <v>1434</v>
+        <v>1477</v>
       </c>
       <c r="D51" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="E51" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F51" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G51" t="n">
         <v>2</v>
@@ -1938,7 +1936,7 @@
       <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr"/>
       <c r="K51" t="n">
-        <v>6944</v>
+        <v>7117</v>
       </c>
     </row>
     <row r="52">
@@ -1948,10 +1946,10 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>1110</v>
+        <v>1146</v>
       </c>
       <c r="C52" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D52" t="n">
         <v>3</v>
@@ -1975,7 +1973,7 @@
         <v>0</v>
       </c>
       <c r="K52" t="n">
-        <v>1131</v>
+        <v>1168</v>
       </c>
     </row>
     <row r="53">
@@ -1985,10 +1983,10 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>1110</v>
+        <v>1146</v>
       </c>
       <c r="C53" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D53" t="n">
         <v>3</v>
@@ -2006,7 +2004,7 @@
       <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr"/>
       <c r="K53" t="n">
-        <v>1131</v>
+        <v>1168</v>
       </c>
     </row>
     <row r="54">
@@ -2016,25 +2014,25 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>75989</v>
+        <v>77424</v>
       </c>
       <c r="C54" t="n">
-        <v>11248</v>
+        <v>11410</v>
       </c>
       <c r="D54" t="n">
-        <v>2416</v>
+        <v>2515</v>
       </c>
       <c r="E54" t="n">
-        <v>242</v>
+        <v>220</v>
       </c>
       <c r="F54" t="n">
-        <v>110</v>
+        <v>137</v>
       </c>
       <c r="G54" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H54" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I54" t="n">
         <v>2</v>
@@ -2043,7 +2041,7 @@
         <v>0</v>
       </c>
       <c r="K54" t="n">
-        <v>90079</v>
+        <v>91780</v>
       </c>
     </row>
   </sheetData>
@@ -2119,10 +2117,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>883</v>
+        <v>1026</v>
       </c>
       <c r="C2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D2" t="n">
         <v>14</v>
@@ -2143,7 +2141,7 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>919</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="3">
@@ -2153,16 +2151,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>652</v>
+        <v>789</v>
       </c>
       <c r="C3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F3" t="n">
         <v>2</v>
@@ -2177,7 +2175,7 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>670</v>
+        <v>808</v>
       </c>
     </row>
     <row r="4">
@@ -2187,19 +2185,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10033</v>
+        <v>10288</v>
       </c>
       <c r="C4" t="n">
-        <v>2529</v>
+        <v>2615</v>
       </c>
       <c r="D4" t="n">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="E4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G4" t="n">
         <v>4</v>
@@ -2211,7 +2209,7 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>12648</v>
+        <v>12996</v>
       </c>
     </row>
     <row r="5">
@@ -2221,16 +2219,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2426</v>
+        <v>1291</v>
       </c>
       <c r="C5" t="n">
-        <v>127</v>
+        <v>110</v>
       </c>
       <c r="D5" t="n">
         <v>7</v>
       </c>
       <c r="E5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
@@ -2245,7 +2243,7 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>2567</v>
+        <v>1414</v>
       </c>
     </row>
     <row r="6">
@@ -2255,10 +2253,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1586</v>
+        <v>1702</v>
       </c>
       <c r="C6" t="n">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="D6" t="n">
         <v>10</v>
@@ -2279,7 +2277,7 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>1637</v>
+        <v>1760</v>
       </c>
     </row>
     <row r="7">
@@ -2289,19 +2287,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>816</v>
+        <v>907</v>
       </c>
       <c r="C7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D7" t="n">
         <v>7</v>
       </c>
       <c r="E7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -2313,7 +2311,7 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>833</v>
+        <v>925</v>
       </c>
     </row>
     <row r="8">
@@ -2323,10 +2321,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>635</v>
+        <v>719</v>
       </c>
       <c r="C8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D8" t="n">
         <v>6</v>
@@ -2347,7 +2345,7 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>654</v>
+        <v>737</v>
       </c>
     </row>
     <row r="9">
@@ -2357,7 +2355,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>604</v>
+        <v>633</v>
       </c>
       <c r="C9" t="n">
         <v>25</v>
@@ -2381,7 +2379,7 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>632</v>
+        <v>661</v>
       </c>
     </row>
     <row r="10">
@@ -2391,7 +2389,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="C10" t="n">
         <v>1</v>
@@ -2415,7 +2413,7 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>86</v>
+        <v>92</v>
       </c>
     </row>
     <row r="11">
@@ -2425,7 +2423,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="C11" t="n">
         <v>8</v>
@@ -2449,7 +2447,7 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>141</v>
+        <v>155</v>
       </c>
     </row>
     <row r="12">
@@ -2459,19 +2457,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4101</v>
+        <v>4178</v>
       </c>
       <c r="C12" t="n">
-        <v>1095</v>
+        <v>1124</v>
       </c>
       <c r="D12" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="E12" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F12" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G12" t="n">
         <v>4</v>
@@ -2483,7 +2481,7 @@
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>5246</v>
+        <v>5357</v>
       </c>
     </row>
     <row r="13">
@@ -2493,7 +2491,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="C13" t="n">
         <v>4</v>
@@ -2517,7 +2515,7 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>166</v>
+        <v>169</v>
       </c>
     </row>
     <row r="14">
@@ -2527,7 +2525,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>52</v>
+        <v>67</v>
       </c>
       <c r="C14" t="n">
         <v>2</v>
@@ -2551,7 +2549,7 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>65</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15">
@@ -2561,7 +2559,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>201</v>
+        <v>279</v>
       </c>
       <c r="C15" t="n">
         <v>8</v>
@@ -2585,7 +2583,7 @@
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>214</v>
+        <v>292</v>
       </c>
     </row>
     <row r="16">
@@ -2595,7 +2593,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1063</v>
+        <v>1129</v>
       </c>
       <c r="C16" t="n">
         <v>8</v>
@@ -2604,10 +2602,10 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
@@ -2619,7 +2617,7 @@
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>1085</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="17">
@@ -2629,7 +2627,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="C17" t="n">
         <v>2</v>
@@ -2653,7 +2651,7 @@
         <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="18">
@@ -2663,10 +2661,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>452</v>
+        <v>459</v>
       </c>
       <c r="C18" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D18" t="n">
         <v>1</v>
@@ -2687,7 +2685,7 @@
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>464</v>
+        <v>472</v>
       </c>
     </row>
     <row r="19">
@@ -2697,7 +2695,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>721</v>
+        <v>817</v>
       </c>
       <c r="C19" t="n">
         <v>29</v>
@@ -2709,7 +2707,7 @@
         <v>16</v>
       </c>
       <c r="F19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G19" t="n">
         <v>2</v>
@@ -2721,7 +2719,7 @@
         <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>813</v>
+        <v>910</v>
       </c>
     </row>
     <row r="20">
@@ -2731,10 +2729,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1126</v>
+        <v>1175</v>
       </c>
       <c r="C20" t="n">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="D20" t="n">
         <v>2</v>
@@ -2755,7 +2753,7 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>1161</v>
+        <v>1220</v>
       </c>
     </row>
     <row r="21">
@@ -2765,7 +2763,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C21" t="n">
         <v>0</v>
@@ -2789,7 +2787,7 @@
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="22">
@@ -2799,10 +2797,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>617</v>
+        <v>630</v>
       </c>
       <c r="C22" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D22" t="n">
         <v>5</v>
@@ -2823,7 +2821,7 @@
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>640</v>
+        <v>654</v>
       </c>
     </row>
     <row r="23">
@@ -2833,7 +2831,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>937</v>
+        <v>976</v>
       </c>
       <c r="C23" t="n">
         <v>16</v>
@@ -2857,7 +2855,7 @@
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>956</v>
+        <v>995</v>
       </c>
     </row>
     <row r="24">
@@ -2867,19 +2865,19 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>919</v>
+        <v>931</v>
       </c>
       <c r="C24" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D24" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
@@ -2891,7 +2889,7 @@
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>954</v>
+        <v>969</v>
       </c>
     </row>
     <row r="25">
@@ -2901,7 +2899,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="C25" t="n">
         <v>3</v>
@@ -2925,7 +2923,7 @@
         <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="26">
@@ -2935,19 +2933,19 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>4089</v>
+        <v>4106</v>
       </c>
       <c r="C26" t="n">
-        <v>2326</v>
+        <v>2356</v>
       </c>
       <c r="D26" t="n">
-        <v>1839</v>
+        <v>1896</v>
       </c>
       <c r="E26" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F26" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G26" t="n">
         <v>4</v>
@@ -2959,7 +2957,7 @@
         <v>1</v>
       </c>
       <c r="J26" t="n">
-        <v>8296</v>
+        <v>8402</v>
       </c>
     </row>
     <row r="27">
@@ -2969,19 +2967,19 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1121</v>
+        <v>1236</v>
       </c>
       <c r="C27" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="D27" t="n">
         <v>10</v>
       </c>
       <c r="E27" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G27" t="n">
         <v>2</v>
@@ -2993,7 +2991,7 @@
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>1148</v>
+        <v>1271</v>
       </c>
     </row>
     <row r="28">
@@ -3003,19 +3001,19 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1377</v>
+        <v>1594</v>
       </c>
       <c r="C28" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D28" t="n">
         <v>9</v>
       </c>
       <c r="E28" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F28" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G28" t="n">
         <v>1</v>
@@ -3027,7 +3025,7 @@
         <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>1435</v>
+        <v>1653</v>
       </c>
     </row>
     <row r="29">
@@ -3037,7 +3035,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>405</v>
+        <v>440</v>
       </c>
       <c r="C29" t="n">
         <v>5</v>
@@ -3046,10 +3044,10 @@
         <v>3</v>
       </c>
       <c r="E29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G29" t="n">
         <v>1</v>
@@ -3061,7 +3059,7 @@
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>420</v>
+        <v>455</v>
       </c>
     </row>
     <row r="30">
@@ -3071,7 +3069,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C30" t="n">
         <v>7</v>
@@ -3095,7 +3093,7 @@
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="31">
@@ -3105,19 +3103,19 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>7937</v>
+        <v>7797</v>
       </c>
       <c r="C31" t="n">
-        <v>1781</v>
+        <v>1678</v>
       </c>
       <c r="D31" t="n">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="E31" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F31" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G31" t="n">
         <v>5</v>
@@ -3129,7 +3127,7 @@
         <v>0</v>
       </c>
       <c r="J31" t="n">
-        <v>9789</v>
+        <v>9551</v>
       </c>
     </row>
     <row r="32">
@@ -3139,10 +3137,10 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D32" t="n">
         <v>2</v>
@@ -3163,7 +3161,7 @@
         <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="33">
@@ -3173,7 +3171,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="C33" t="n">
         <v>5</v>
@@ -3197,7 +3195,7 @@
         <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>51</v>
+        <v>57</v>
       </c>
     </row>
     <row r="34">
@@ -3207,10 +3205,10 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>260</v>
+        <v>270</v>
       </c>
       <c r="C34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D34" t="n">
         <v>2</v>
@@ -3231,7 +3229,7 @@
         <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>264</v>
+        <v>275</v>
       </c>
     </row>
     <row r="35">
@@ -3241,7 +3239,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>775</v>
+        <v>796</v>
       </c>
       <c r="C35" t="n">
         <v>13</v>
@@ -3265,7 +3263,7 @@
         <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>791</v>
+        <v>812</v>
       </c>
     </row>
     <row r="36">
@@ -3275,10 +3273,10 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>2488</v>
+        <v>2622</v>
       </c>
       <c r="C36" t="n">
-        <v>84</v>
+        <v>104</v>
       </c>
       <c r="D36" t="n">
         <v>5</v>
@@ -3299,7 +3297,7 @@
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>2585</v>
+        <v>2739</v>
       </c>
     </row>
     <row r="37">
@@ -3309,7 +3307,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>452</v>
+        <v>463</v>
       </c>
       <c r="C37" t="n">
         <v>5</v>
@@ -3333,7 +3331,7 @@
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>458</v>
+        <v>469</v>
       </c>
     </row>
     <row r="38">
@@ -3343,7 +3341,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>332</v>
+        <v>384</v>
       </c>
       <c r="C38" t="n">
         <v>1</v>
@@ -3367,7 +3365,7 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>338</v>
+        <v>390</v>
       </c>
     </row>
     <row r="39">
@@ -3377,7 +3375,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>422</v>
+        <v>430</v>
       </c>
       <c r="C39" t="n">
         <v>8</v>
@@ -3401,7 +3399,7 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>438</v>
+        <v>446</v>
       </c>
     </row>
     <row r="40">
@@ -3411,7 +3409,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>442</v>
+        <v>488</v>
       </c>
       <c r="C40" t="n">
         <v>0</v>
@@ -3420,10 +3418,10 @@
         <v>4</v>
       </c>
       <c r="E40" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F40" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G40" t="n">
         <v>1</v>
@@ -3435,7 +3433,7 @@
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>453</v>
+        <v>499</v>
       </c>
     </row>
     <row r="41">
@@ -3445,19 +3443,19 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>710</v>
+        <v>142</v>
       </c>
       <c r="C41" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D41" t="n">
         <v>3</v>
       </c>
       <c r="E41" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G41" t="n">
         <v>0</v>
@@ -3469,7 +3467,7 @@
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>724</v>
+        <v>153</v>
       </c>
     </row>
     <row r="42">
@@ -3479,10 +3477,10 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>628</v>
+        <v>680</v>
       </c>
       <c r="C42" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D42" t="n">
         <v>1</v>
@@ -3503,7 +3501,7 @@
         <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>637</v>
+        <v>690</v>
       </c>
     </row>
     <row r="43">
@@ -3513,10 +3511,10 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>981</v>
+        <v>1042</v>
       </c>
       <c r="C43" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D43" t="n">
         <v>3</v>
@@ -3537,7 +3535,7 @@
         <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>995</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="44">
@@ -3547,10 +3545,10 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>912</v>
+        <v>953</v>
       </c>
       <c r="C44" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D44" t="n">
         <v>6</v>
@@ -3571,7 +3569,7 @@
         <v>1</v>
       </c>
       <c r="J44" t="n">
-        <v>946</v>
+        <v>988</v>
       </c>
     </row>
     <row r="45">
@@ -3581,7 +3579,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>510</v>
+        <v>110</v>
       </c>
       <c r="C45" t="n">
         <v>2</v>
@@ -3605,7 +3603,7 @@
         <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>516</v>
+        <v>116</v>
       </c>
     </row>
     <row r="46">
@@ -3615,7 +3613,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>567</v>
+        <v>697</v>
       </c>
       <c r="C46" t="n">
         <v>5</v>
@@ -3624,10 +3622,10 @@
         <v>6</v>
       </c>
       <c r="E46" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F46" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G46" t="n">
         <v>3</v>
@@ -3639,7 +3637,7 @@
         <v>0</v>
       </c>
       <c r="J46" t="n">
-        <v>591</v>
+        <v>721</v>
       </c>
     </row>
     <row r="47">
@@ -3649,10 +3647,10 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="C47" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D47" t="n">
         <v>5</v>
@@ -3673,7 +3671,7 @@
         <v>0</v>
       </c>
       <c r="J47" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="48">
@@ -3683,19 +3681,19 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>2897</v>
+        <v>3044</v>
       </c>
       <c r="C48" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D48" t="n">
         <v>15</v>
       </c>
       <c r="E48" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F48" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G48" t="n">
         <v>1</v>
@@ -3707,7 +3705,7 @@
         <v>0</v>
       </c>
       <c r="J48" t="n">
-        <v>2968</v>
+        <v>3117</v>
       </c>
     </row>
     <row r="49">
@@ -3717,7 +3715,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>611</v>
+        <v>627</v>
       </c>
       <c r="C49" t="n">
         <v>18</v>
@@ -3741,7 +3739,7 @@
         <v>0</v>
       </c>
       <c r="J49" t="n">
-        <v>632</v>
+        <v>648</v>
       </c>
     </row>
     <row r="50">
@@ -3751,10 +3749,10 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>348</v>
+        <v>377</v>
       </c>
       <c r="C50" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D50" t="n">
         <v>3</v>
@@ -3775,7 +3773,7 @@
         <v>0</v>
       </c>
       <c r="J50" t="n">
-        <v>362</v>
+        <v>393</v>
       </c>
     </row>
     <row r="51">
@@ -3785,13 +3783,13 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>790</v>
+        <v>866</v>
       </c>
       <c r="C51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E51" t="n">
         <v>3</v>
@@ -3809,7 +3807,7 @@
         <v>0</v>
       </c>
       <c r="J51" t="n">
-        <v>794</v>
+        <v>870</v>
       </c>
     </row>
     <row r="52">
@@ -3819,19 +3817,19 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>5741</v>
+        <v>5855</v>
       </c>
       <c r="C52" t="n">
-        <v>1244</v>
+        <v>1274</v>
       </c>
       <c r="D52" t="n">
-        <v>124</v>
+        <v>141</v>
       </c>
       <c r="E52" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F52" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G52" t="n">
         <v>2</v>
@@ -3843,7 +3841,7 @@
         <v>0</v>
       </c>
       <c r="J52" t="n">
-        <v>7127</v>
+        <v>7288</v>
       </c>
     </row>
     <row r="53">
@@ -3853,10 +3851,10 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>395</v>
+        <v>538</v>
       </c>
       <c r="C53" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D53" t="n">
         <v>10</v>
@@ -3877,7 +3875,7 @@
         <v>0</v>
       </c>
       <c r="J53" t="n">
-        <v>412</v>
+        <v>554</v>
       </c>
     </row>
     <row r="54">
@@ -3887,10 +3885,10 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="C54" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D54" t="n">
         <v>0</v>
@@ -3911,7 +3909,7 @@
         <v>0</v>
       </c>
       <c r="J54" t="n">
-        <v>216</v>
+        <v>222</v>
       </c>
     </row>
     <row r="55">
@@ -3921,19 +3919,19 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>5242</v>
+        <v>5352</v>
       </c>
       <c r="C55" t="n">
-        <v>1373</v>
+        <v>1413</v>
       </c>
       <c r="D55" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="E55" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F55" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G55" t="n">
         <v>2</v>
@@ -3945,7 +3943,7 @@
         <v>0</v>
       </c>
       <c r="J55" t="n">
-        <v>6658</v>
+        <v>6816</v>
       </c>
     </row>
     <row r="56">
@@ -3955,10 +3953,10 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>104</v>
+        <v>145</v>
       </c>
       <c r="C56" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D56" t="n">
         <v>1</v>
@@ -3979,7 +3977,7 @@
         <v>0</v>
       </c>
       <c r="J56" t="n">
-        <v>118</v>
+        <v>161</v>
       </c>
     </row>
     <row r="57">
@@ -3989,10 +3987,10 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="C57" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D57" t="n">
         <v>3</v>
@@ -4013,7 +4011,7 @@
         <v>0</v>
       </c>
       <c r="J57" t="n">
-        <v>433</v>
+        <v>436</v>
       </c>
     </row>
     <row r="58">
@@ -4023,16 +4021,16 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C58" t="n">
+        <v>2</v>
+      </c>
+      <c r="D58" t="n">
         <v>4</v>
       </c>
-      <c r="D58" t="n">
-        <v>5</v>
-      </c>
       <c r="E58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F58" t="n">
         <v>0</v>
@@ -4047,7 +4045,7 @@
         <v>0</v>
       </c>
       <c r="J58" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="59">
@@ -4057,7 +4055,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C59" t="n">
         <v>1</v>
@@ -4081,7 +4079,7 @@
         <v>0</v>
       </c>
       <c r="J59" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="60">
@@ -4091,7 +4089,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>906</v>
+        <v>989</v>
       </c>
       <c r="C60" t="n">
         <v>4</v>
@@ -4115,7 +4113,7 @@
         <v>0</v>
       </c>
       <c r="J60" t="n">
-        <v>921</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="61">
@@ -4125,10 +4123,10 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>1021</v>
+        <v>1118</v>
       </c>
       <c r="C61" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D61" t="n">
         <v>18</v>
@@ -4149,7 +4147,7 @@
         <v>0</v>
       </c>
       <c r="J61" t="n">
-        <v>1056</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="62">
@@ -4159,7 +4157,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>702</v>
+        <v>755</v>
       </c>
       <c r="C62" t="n">
         <v>18</v>
@@ -4168,10 +4166,10 @@
         <v>3</v>
       </c>
       <c r="E62" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G62" t="n">
         <v>0</v>
@@ -4183,7 +4181,7 @@
         <v>0</v>
       </c>
       <c r="J62" t="n">
-        <v>725</v>
+        <v>778</v>
       </c>
     </row>
     <row r="63">
@@ -4193,7 +4191,7 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>2164</v>
+        <v>2489</v>
       </c>
       <c r="C63" t="n">
         <v>14</v>
@@ -4208,16 +4206,16 @@
         <v>6</v>
       </c>
       <c r="G63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H63" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I63" t="n">
         <v>0</v>
       </c>
       <c r="J63" t="n">
-        <v>2211</v>
+        <v>2536</v>
       </c>
     </row>
     <row r="64">
@@ -4227,19 +4225,19 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>1168</v>
+        <v>1292</v>
       </c>
       <c r="C64" t="n">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="D64" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E64" t="n">
+        <v>2</v>
+      </c>
+      <c r="F64" t="n">
         <v>3</v>
-      </c>
-      <c r="F64" t="n">
-        <v>2</v>
       </c>
       <c r="G64" t="n">
         <v>3</v>
@@ -4251,7 +4249,7 @@
         <v>0</v>
       </c>
       <c r="J64" t="n">
-        <v>1332</v>
+        <v>1464</v>
       </c>
     </row>
     <row r="65">
@@ -4261,31 +4259,31 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>75989</v>
+        <v>77424</v>
       </c>
       <c r="C65" t="n">
-        <v>11248</v>
+        <v>11410</v>
       </c>
       <c r="D65" t="n">
-        <v>2416</v>
+        <v>2515</v>
       </c>
       <c r="E65" t="n">
-        <v>242</v>
+        <v>220</v>
       </c>
       <c r="F65" t="n">
-        <v>110</v>
+        <v>137</v>
       </c>
       <c r="G65" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H65" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I65" t="n">
         <v>2</v>
       </c>
       <c r="J65" t="n">
-        <v>90079</v>
+        <v>91780</v>
       </c>
     </row>
   </sheetData>
@@ -4361,19 +4359,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>9748</v>
+        <v>10035</v>
       </c>
       <c r="C2" t="n">
-        <v>2516</v>
+        <v>2579</v>
       </c>
       <c r="D2" t="n">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="E2" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G2" t="n">
         <v>4</v>
@@ -4385,7 +4383,7 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>12348</v>
+        <v>12706</v>
       </c>
     </row>
     <row r="3">
@@ -4395,19 +4393,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3913</v>
+        <v>3997</v>
       </c>
       <c r="C3" t="n">
-        <v>1098</v>
+        <v>1124</v>
       </c>
       <c r="D3" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="E3" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F3" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G3" t="n">
         <v>3</v>
@@ -4419,7 +4417,7 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>5058</v>
+        <v>5173</v>
       </c>
     </row>
     <row r="4">
@@ -4429,19 +4427,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3409</v>
+        <v>3394</v>
       </c>
       <c r="C4" t="n">
-        <v>2245</v>
+        <v>2273</v>
       </c>
       <c r="D4" t="n">
-        <v>1905</v>
+        <v>1964</v>
       </c>
       <c r="E4" t="n">
         <v>23</v>
       </c>
       <c r="F4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G4" t="n">
         <v>4</v>
@@ -4453,7 +4451,7 @@
         <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>7592</v>
+        <v>7665</v>
       </c>
     </row>
     <row r="5">
@@ -4463,10 +4461,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>195</v>
+        <v>225</v>
       </c>
       <c r="C5" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D5" t="n">
         <v>4</v>
@@ -4487,7 +4485,7 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>229</v>
+        <v>260</v>
       </c>
     </row>
     <row r="6">
@@ -4497,19 +4495,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2863</v>
+        <v>3010</v>
       </c>
       <c r="C6" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D6" t="n">
         <v>8</v>
       </c>
       <c r="E6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -4521,7 +4519,7 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>2925</v>
+        <v>3074</v>
       </c>
     </row>
     <row r="7">
@@ -4531,16 +4529,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1918</v>
+        <v>588</v>
       </c>
       <c r="C7" t="n">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="D7" t="n">
         <v>5</v>
       </c>
       <c r="E7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F7" t="n">
         <v>1</v>
@@ -4555,7 +4553,7 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>1967</v>
+        <v>617</v>
       </c>
     </row>
     <row r="8">
@@ -4565,10 +4563,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1595</v>
+        <v>1712</v>
       </c>
       <c r="C8" t="n">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="D8" t="n">
         <v>11</v>
@@ -4589,7 +4587,7 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>1647</v>
+        <v>1771</v>
       </c>
     </row>
     <row r="9">
@@ -4599,10 +4597,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>960</v>
+        <v>1021</v>
       </c>
       <c r="C9" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D9" t="n">
         <v>3</v>
@@ -4623,7 +4621,7 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>974</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="10">
@@ -4633,7 +4631,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>694</v>
+        <v>743</v>
       </c>
       <c r="C10" t="n">
         <v>17</v>
@@ -4642,10 +4640,10 @@
         <v>3</v>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -4657,7 +4655,7 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>716</v>
+        <v>765</v>
       </c>
     </row>
     <row r="11">
@@ -4667,31 +4665,31 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2694</v>
+        <v>3155</v>
       </c>
       <c r="C11" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D11" t="n">
+        <v>15</v>
+      </c>
+      <c r="E11" t="n">
         <v>16</v>
-      </c>
-      <c r="E11" t="n">
-        <v>15</v>
       </c>
       <c r="F11" t="n">
         <v>7</v>
       </c>
       <c r="G11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>2756</v>
+        <v>3218</v>
       </c>
     </row>
     <row r="12">
@@ -4701,10 +4699,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C12" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D12" t="n">
         <v>1</v>
@@ -4735,10 +4733,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C13" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
@@ -4769,7 +4767,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C14" t="n">
         <v>1</v>
@@ -4793,7 +4791,7 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15">
@@ -4803,10 +4801,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C15" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D15" t="n">
         <v>1</v>
@@ -4827,7 +4825,7 @@
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>121</v>
+        <v>125</v>
       </c>
     </row>
     <row r="16">
@@ -4837,10 +4835,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C16" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
@@ -4871,10 +4869,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="C17" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
@@ -4905,10 +4903,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C18" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
@@ -4939,13 +4937,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C19" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
@@ -4963,7 +4961,7 @@
         <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="20">
@@ -4973,10 +4971,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C20" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
@@ -4997,7 +4995,7 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="21">
@@ -5007,10 +5005,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="C21" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
@@ -5031,7 +5029,7 @@
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="22">
@@ -5041,10 +5039,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="C22" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
@@ -5065,7 +5063,7 @@
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="23">
@@ -5075,10 +5073,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="C23" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="D23" t="n">
         <v>2</v>
@@ -5099,7 +5097,7 @@
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>238</v>
+        <v>243</v>
       </c>
     </row>
     <row r="24">
@@ -5109,7 +5107,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>292</v>
+        <v>302</v>
       </c>
       <c r="C24" t="n">
         <v>9</v>
@@ -5133,7 +5131,7 @@
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>314</v>
+        <v>324</v>
       </c>
     </row>
     <row r="25">
@@ -5177,10 +5175,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>3608</v>
+        <v>3791</v>
       </c>
       <c r="C26" t="n">
-        <v>110</v>
+        <v>140</v>
       </c>
       <c r="D26" t="n">
         <v>6</v>
@@ -5201,7 +5199,7 @@
         <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>3737</v>
+        <v>3950</v>
       </c>
     </row>
     <row r="27">
@@ -5211,19 +5209,19 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1273</v>
+        <v>1411</v>
       </c>
       <c r="C27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D27" t="n">
         <v>5</v>
       </c>
       <c r="E27" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F27" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G27" t="n">
         <v>1</v>
@@ -5235,7 +5233,7 @@
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>1295</v>
+        <v>1434</v>
       </c>
     </row>
     <row r="28">
@@ -5245,19 +5243,19 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>3263</v>
+        <v>3922</v>
       </c>
       <c r="C28" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D28" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E28" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F28" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G28" t="n">
         <v>12</v>
@@ -5269,7 +5267,7 @@
         <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>3405</v>
+        <v>4066</v>
       </c>
     </row>
     <row r="29">
@@ -5279,19 +5277,19 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>374</v>
+        <v>418</v>
       </c>
       <c r="C29" t="n">
         <v>8</v>
       </c>
       <c r="D29" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G29" t="n">
         <v>2</v>
@@ -5303,7 +5301,7 @@
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>414</v>
+        <v>458</v>
       </c>
     </row>
     <row r="30">
@@ -5313,7 +5311,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1470</v>
+        <v>1572</v>
       </c>
       <c r="C30" t="n">
         <v>13</v>
@@ -5322,11 +5320,11 @@
         <v>5</v>
       </c>
       <c r="E30" t="n">
+        <v>4</v>
+      </c>
+      <c r="F30" t="n">
         <v>6</v>
       </c>
-      <c r="F30" t="n">
-        <v>4</v>
-      </c>
       <c r="G30" t="n">
         <v>1</v>
       </c>
@@ -5337,7 +5335,7 @@
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>1499</v>
+        <v>1601</v>
       </c>
     </row>
     <row r="31">
@@ -5347,10 +5345,10 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>935</v>
+        <v>1220</v>
       </c>
       <c r="C31" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D31" t="n">
         <v>36</v>
@@ -5371,7 +5369,7 @@
         <v>1</v>
       </c>
       <c r="J31" t="n">
-        <v>1013</v>
+        <v>1294</v>
       </c>
     </row>
     <row r="32">
@@ -5381,19 +5379,19 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>8965</v>
+        <v>9302</v>
       </c>
       <c r="C32" t="n">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="D32" t="n">
         <v>13</v>
       </c>
       <c r="E32" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F32" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G32" t="n">
         <v>2</v>
@@ -5405,7 +5403,7 @@
         <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>9093</v>
+        <v>9441</v>
       </c>
     </row>
     <row r="33">
@@ -5415,19 +5413,19 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>791</v>
+        <v>948</v>
       </c>
       <c r="C33" t="n">
         <v>108</v>
       </c>
       <c r="D33" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E33" t="n">
         <v>10</v>
       </c>
       <c r="F33" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G33" t="n">
         <v>1</v>
@@ -5439,7 +5437,7 @@
         <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>937</v>
+        <v>1093</v>
       </c>
     </row>
     <row r="34">
@@ -5449,19 +5447,19 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1433</v>
+        <v>1599</v>
       </c>
       <c r="C34" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="D34" t="n">
         <v>9</v>
       </c>
       <c r="E34" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G34" t="n">
         <v>2</v>
@@ -5473,7 +5471,7 @@
         <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>1461</v>
+        <v>1635</v>
       </c>
     </row>
     <row r="35">
@@ -5483,19 +5481,19 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1215</v>
+        <v>231</v>
       </c>
       <c r="C35" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D35" t="n">
         <v>3</v>
       </c>
       <c r="E35" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G35" t="n">
         <v>0</v>
@@ -5507,7 +5505,7 @@
         <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>1235</v>
+        <v>248</v>
       </c>
     </row>
     <row r="36">
@@ -5517,13 +5515,13 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>2262</v>
+        <v>2483</v>
       </c>
       <c r="C36" t="n">
         <v>8</v>
       </c>
       <c r="D36" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E36" t="n">
         <v>11</v>
@@ -5541,7 +5539,7 @@
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>2285</v>
+        <v>2507</v>
       </c>
     </row>
     <row r="37">
@@ -5551,10 +5549,10 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1073</v>
+        <v>1176</v>
       </c>
       <c r="C37" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="D37" t="n">
         <v>8</v>
@@ -5575,7 +5573,7 @@
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>1096</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="38">
@@ -5585,19 +5583,19 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>8501</v>
+        <v>8380</v>
       </c>
       <c r="C38" t="n">
-        <v>1947</v>
+        <v>1840</v>
       </c>
       <c r="D38" t="n">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="E38" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F38" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="G38" t="n">
         <v>5</v>
@@ -5609,7 +5607,7 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>10549</v>
+        <v>10330</v>
       </c>
     </row>
     <row r="39">
@@ -5619,10 +5617,10 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1110</v>
+        <v>1146</v>
       </c>
       <c r="C39" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D39" t="n">
         <v>3</v>
@@ -5643,7 +5641,7 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>1131</v>
+        <v>1168</v>
       </c>
     </row>
     <row r="40">
@@ -5653,19 +5651,19 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>4746</v>
+        <v>4855</v>
       </c>
       <c r="C40" t="n">
-        <v>1106</v>
+        <v>1129</v>
       </c>
       <c r="D40" t="n">
-        <v>93</v>
+        <v>107</v>
       </c>
       <c r="E40" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F40" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G40" t="n">
         <v>2</v>
@@ -5677,7 +5675,7 @@
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>5961</v>
+        <v>6107</v>
       </c>
     </row>
     <row r="41">
@@ -5687,19 +5685,19 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>5467</v>
+        <v>5590</v>
       </c>
       <c r="C41" t="n">
-        <v>1434</v>
+        <v>1477</v>
       </c>
       <c r="D41" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="E41" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F41" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G41" t="n">
         <v>2</v>
@@ -5711,7 +5709,7 @@
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>6944</v>
+        <v>7117</v>
       </c>
     </row>
     <row r="42">
@@ -5721,31 +5719,31 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>75989</v>
+        <v>77424</v>
       </c>
       <c r="C42" t="n">
-        <v>11248</v>
+        <v>11410</v>
       </c>
       <c r="D42" t="n">
-        <v>2416</v>
+        <v>2515</v>
       </c>
       <c r="E42" t="n">
-        <v>242</v>
+        <v>220</v>
       </c>
       <c r="F42" t="n">
-        <v>110</v>
+        <v>137</v>
       </c>
       <c r="G42" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H42" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I42" t="n">
         <v>2</v>
       </c>
       <c r="J42" t="n">
-        <v>90079</v>
+        <v>91780</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add Telegram Bot alerts and one-time macOS Terminal popup for expired session
</commit_message>
<xml_diff>
--- a/BaoCao_TonKho.xlsx
+++ b/BaoCao_TonKho.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>05/06/2026 00:52:34</t>
+          <t>05/06/2026 01:02:39</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -579,16 +579,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>10229</v>
+        <v>5469</v>
       </c>
       <c r="C7" t="n">
-        <v>154</v>
+        <v>140</v>
       </c>
       <c r="D7" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="E7" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F7" t="n">
         <v>15</v>
@@ -606,7 +606,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>10482</v>
+        <v>5699</v>
       </c>
     </row>
     <row r="8">
@@ -616,13 +616,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3010</v>
+        <v>2088</v>
       </c>
       <c r="C8" t="n">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="D8" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E8" t="n">
         <v>7</v>
@@ -637,7 +637,7 @@
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="n">
-        <v>3074</v>
+        <v>2141</v>
       </c>
     </row>
     <row r="9">
@@ -647,13 +647,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>588</v>
+        <v>111</v>
       </c>
       <c r="C9" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D9" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E9" t="n">
         <v>3</v>
@@ -668,7 +668,7 @@
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="n">
-        <v>617</v>
+        <v>139</v>
       </c>
     </row>
     <row r="10">
@@ -678,16 +678,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1712</v>
+        <v>1099</v>
       </c>
       <c r="C10" t="n">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D10" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
@@ -695,7 +695,7 @@
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="n">
-        <v>1771</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="11">
@@ -705,13 +705,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1021</v>
+        <v>691</v>
       </c>
       <c r="C11" t="n">
         <v>10</v>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E11" t="n">
         <v>2</v>
@@ -724,7 +724,7 @@
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="n">
-        <v>1037</v>
+        <v>706</v>
       </c>
     </row>
     <row r="12">
@@ -734,10 +734,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>743</v>
+        <v>490</v>
       </c>
       <c r="C12" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D12" t="n">
         <v>3</v>
@@ -751,7 +751,7 @@
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="n">
-        <v>765</v>
+        <v>509</v>
       </c>
     </row>
     <row r="13">
@@ -761,13 +761,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3155</v>
+        <v>990</v>
       </c>
       <c r="C13" t="n">
         <v>19</v>
       </c>
       <c r="D13" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E13" t="n">
         <v>16</v>
@@ -784,7 +784,7 @@
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="n">
-        <v>3218</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="14">
@@ -794,10 +794,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1500</v>
+        <v>1318</v>
       </c>
       <c r="C14" t="n">
-        <v>307</v>
+        <v>330</v>
       </c>
       <c r="D14" t="n">
         <v>13</v>
@@ -821,7 +821,7 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>1840</v>
+        <v>1681</v>
       </c>
     </row>
     <row r="15">
@@ -831,10 +831,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="C15" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D15" t="n">
         <v>1</v>
@@ -846,7 +846,7 @@
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="n">
-        <v>94</v>
+        <v>89</v>
       </c>
     </row>
     <row r="16">
@@ -856,10 +856,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>123</v>
+        <v>113</v>
       </c>
       <c r="C16" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
@@ -871,7 +871,7 @@
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="n">
-        <v>144</v>
+        <v>135</v>
       </c>
     </row>
     <row r="17">
@@ -881,10 +881,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
@@ -896,7 +896,7 @@
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18">
@@ -906,10 +906,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="C18" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D18" t="n">
         <v>1</v>
@@ -923,7 +923,7 @@
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="n">
-        <v>125</v>
+        <v>115</v>
       </c>
     </row>
     <row r="19">
@@ -933,10 +933,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="C19" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="n">
@@ -952,7 +952,7 @@
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="n">
-        <v>109</v>
+        <v>99</v>
       </c>
     </row>
     <row r="20">
@@ -962,10 +962,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="C20" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
@@ -977,7 +977,7 @@
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="n">
-        <v>137</v>
+        <v>128</v>
       </c>
     </row>
     <row r="21">
@@ -987,10 +987,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="C21" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
@@ -1004,7 +1004,7 @@
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="n">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="22">
@@ -1014,10 +1014,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="C22" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D22" t="n">
         <v>3</v>
@@ -1031,7 +1031,7 @@
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="n">
-        <v>129</v>
+        <v>118</v>
       </c>
     </row>
     <row r="23">
@@ -1041,7 +1041,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="C23" t="n">
         <v>13</v>
@@ -1056,7 +1056,7 @@
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="n">
-        <v>74</v>
+        <v>68</v>
       </c>
     </row>
     <row r="24">
@@ -1066,10 +1066,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>143</v>
+        <v>126</v>
       </c>
       <c r="C24" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr"/>
@@ -1079,7 +1079,7 @@
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="n">
-        <v>173</v>
+        <v>161</v>
       </c>
     </row>
     <row r="25">
@@ -1089,10 +1089,10 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="C25" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr"/>
@@ -1102,7 +1102,7 @@
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="n">
-        <v>124</v>
+        <v>115</v>
       </c>
     </row>
     <row r="26">
@@ -1112,10 +1112,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>198</v>
+        <v>170</v>
       </c>
       <c r="C26" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D26" t="n">
         <v>2</v>
@@ -1129,7 +1129,7 @@
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="n">
-        <v>243</v>
+        <v>217</v>
       </c>
     </row>
     <row r="27">
@@ -1139,7 +1139,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>302</v>
+        <v>260</v>
       </c>
       <c r="C27" t="n">
         <v>9</v>
@@ -1160,7 +1160,7 @@
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="n">
-        <v>324</v>
+        <v>282</v>
       </c>
     </row>
     <row r="28">
@@ -1170,7 +1170,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C28" t="n">
         <v>9</v>
@@ -1185,7 +1185,7 @@
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="n">
-        <v>77</v>
+        <v>73</v>
       </c>
     </row>
     <row r="29">
@@ -1195,10 +1195,10 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>225</v>
+        <v>134</v>
       </c>
       <c r="C29" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D29" t="n">
         <v>4</v>
@@ -1222,7 +1222,7 @@
         <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>260</v>
+        <v>167</v>
       </c>
     </row>
     <row r="30">
@@ -1232,10 +1232,10 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>225</v>
+        <v>134</v>
       </c>
       <c r="C30" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D30" t="n">
         <v>4</v>
@@ -1253,7 +1253,7 @@
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="n">
-        <v>260</v>
+        <v>167</v>
       </c>
     </row>
     <row r="31">
@@ -1263,16 +1263,16 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>28073</v>
+        <v>17095</v>
       </c>
       <c r="C31" t="n">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="D31" t="n">
-        <v>172</v>
+        <v>142</v>
       </c>
       <c r="E31" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="F31" t="n">
         <v>60</v>
@@ -1290,7 +1290,7 @@
         <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>28932</v>
+        <v>17924</v>
       </c>
     </row>
     <row r="32">
@@ -1300,13 +1300,13 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>3791</v>
+        <v>2563</v>
       </c>
       <c r="C32" t="n">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="D32" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E32" t="n">
         <v>5</v>
@@ -1321,7 +1321,7 @@
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="n">
-        <v>3950</v>
+        <v>2726</v>
       </c>
     </row>
     <row r="33">
@@ -1331,13 +1331,13 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1411</v>
+        <v>775</v>
       </c>
       <c r="C33" t="n">
         <v>5</v>
       </c>
       <c r="D33" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E33" t="n">
         <v>6</v>
@@ -1354,7 +1354,7 @@
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="n">
-        <v>1434</v>
+        <v>797</v>
       </c>
     </row>
     <row r="34">
@@ -1364,16 +1364,16 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>3922</v>
+        <v>1414</v>
       </c>
       <c r="C34" t="n">
         <v>47</v>
       </c>
       <c r="D34" t="n">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="E34" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F34" t="n">
         <v>19</v>
@@ -1385,7 +1385,7 @@
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="n">
-        <v>4066</v>
+        <v>1548</v>
       </c>
     </row>
     <row r="35">
@@ -1395,7 +1395,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>418</v>
+        <v>300</v>
       </c>
       <c r="C35" t="n">
         <v>8</v>
@@ -1418,7 +1418,7 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="n">
-        <v>458</v>
+        <v>340</v>
       </c>
     </row>
     <row r="36">
@@ -1428,16 +1428,16 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1572</v>
+        <v>1014</v>
       </c>
       <c r="C36" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D36" t="n">
+        <v>2</v>
+      </c>
+      <c r="E36" t="n">
         <v>5</v>
-      </c>
-      <c r="E36" t="n">
-        <v>4</v>
       </c>
       <c r="F36" t="n">
         <v>6</v>
@@ -1449,7 +1449,7 @@
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="n">
-        <v>1601</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="37">
@@ -1459,13 +1459,13 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1220</v>
+        <v>329</v>
       </c>
       <c r="C37" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D37" t="n">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="E37" t="n">
         <v>15</v>
@@ -1480,7 +1480,7 @@
       </c>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="n">
-        <v>1294</v>
+        <v>396</v>
       </c>
     </row>
     <row r="38">
@@ -1490,10 +1490,10 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>9302</v>
+        <v>7601</v>
       </c>
       <c r="C38" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D38" t="n">
         <v>13</v>
@@ -1511,7 +1511,7 @@
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="n">
-        <v>9441</v>
+        <v>7737</v>
       </c>
     </row>
     <row r="39">
@@ -1521,13 +1521,13 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>948</v>
+        <v>458</v>
       </c>
       <c r="C39" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="D39" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E39" t="n">
         <v>10</v>
@@ -1544,7 +1544,7 @@
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="n">
-        <v>1093</v>
+        <v>597</v>
       </c>
     </row>
     <row r="40">
@@ -1554,13 +1554,13 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1599</v>
+        <v>700</v>
       </c>
       <c r="C40" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D40" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E40" t="n">
         <v>7</v>
@@ -1575,7 +1575,7 @@
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="n">
-        <v>1635</v>
+        <v>733</v>
       </c>
     </row>
     <row r="41">
@@ -1585,10 +1585,10 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>231</v>
+        <v>20</v>
       </c>
       <c r="C41" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D41" t="n">
         <v>3</v>
@@ -1606,7 +1606,7 @@
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="n">
-        <v>248</v>
+        <v>36</v>
       </c>
     </row>
     <row r="42">
@@ -1616,13 +1616,13 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>2483</v>
+        <v>1329</v>
       </c>
       <c r="C42" t="n">
         <v>8</v>
       </c>
       <c r="D42" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E42" t="n">
         <v>11</v>
@@ -1635,7 +1635,7 @@
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="n">
-        <v>2507</v>
+        <v>1352</v>
       </c>
     </row>
     <row r="43">
@@ -1645,10 +1645,10 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>1176</v>
+        <v>592</v>
       </c>
       <c r="C43" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D43" t="n">
         <v>8</v>
@@ -1666,7 +1666,7 @@
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="n">
-        <v>1205</v>
+        <v>620</v>
       </c>
     </row>
     <row r="44">
@@ -1676,13 +1676,13 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>3394</v>
+        <v>2860</v>
       </c>
       <c r="C44" t="n">
-        <v>2273</v>
+        <v>2169</v>
       </c>
       <c r="D44" t="n">
-        <v>1964</v>
+        <v>1768</v>
       </c>
       <c r="E44" t="n">
         <v>23</v>
@@ -1703,7 +1703,7 @@
         <v>0</v>
       </c>
       <c r="K44" t="n">
-        <v>7665</v>
+        <v>6831</v>
       </c>
     </row>
     <row r="45">
@@ -1713,13 +1713,13 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>3394</v>
+        <v>2860</v>
       </c>
       <c r="C45" t="n">
-        <v>2273</v>
+        <v>2169</v>
       </c>
       <c r="D45" t="n">
-        <v>1964</v>
+        <v>1768</v>
       </c>
       <c r="E45" t="n">
         <v>23</v>
@@ -1738,7 +1738,7 @@
       </c>
       <c r="J45" t="inlineStr"/>
       <c r="K45" t="n">
-        <v>7665</v>
+        <v>6831</v>
       </c>
     </row>
     <row r="46">
@@ -1748,25 +1748,25 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>32857</v>
+        <v>24079</v>
       </c>
       <c r="C46" t="n">
-        <v>8149</v>
+        <v>7737</v>
       </c>
       <c r="D46" t="n">
-        <v>314</v>
+        <v>283</v>
       </c>
       <c r="E46" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F46" t="n">
         <v>44</v>
       </c>
       <c r="G46" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H46" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I46" t="n">
         <v>0</v>
@@ -1775,7 +1775,7 @@
         <v>0</v>
       </c>
       <c r="K46" t="n">
-        <v>41433</v>
+        <v>32214</v>
       </c>
     </row>
     <row r="47">
@@ -1785,30 +1785,30 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>10035</v>
+        <v>7096</v>
       </c>
       <c r="C47" t="n">
-        <v>2579</v>
+        <v>2428</v>
       </c>
       <c r="D47" t="n">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="E47" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F47" t="n">
         <v>7</v>
       </c>
       <c r="G47" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="n">
-        <v>12706</v>
+        <v>9612</v>
       </c>
     </row>
     <row r="48">
@@ -1818,13 +1818,13 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>3997</v>
+        <v>3015</v>
       </c>
       <c r="C48" t="n">
-        <v>1124</v>
+        <v>1066</v>
       </c>
       <c r="D48" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E48" t="n">
         <v>8</v>
@@ -1839,7 +1839,7 @@
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="n">
-        <v>5173</v>
+        <v>4131</v>
       </c>
     </row>
     <row r="49">
@@ -1849,13 +1849,13 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>8380</v>
+        <v>6193</v>
       </c>
       <c r="C49" t="n">
-        <v>1840</v>
+        <v>1760</v>
       </c>
       <c r="D49" t="n">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="E49" t="n">
         <v>16</v>
@@ -1872,7 +1872,7 @@
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="n">
-        <v>10330</v>
+        <v>8054</v>
       </c>
     </row>
     <row r="50">
@@ -1882,16 +1882,16 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>4855</v>
+        <v>3606</v>
       </c>
       <c r="C50" t="n">
-        <v>1129</v>
+        <v>1096</v>
       </c>
       <c r="D50" t="n">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="E50" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F50" t="n">
         <v>4</v>
@@ -1905,7 +1905,7 @@
       <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr"/>
       <c r="K50" t="n">
-        <v>6107</v>
+        <v>4813</v>
       </c>
     </row>
     <row r="51">
@@ -1915,13 +1915,13 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>5590</v>
+        <v>4169</v>
       </c>
       <c r="C51" t="n">
-        <v>1477</v>
+        <v>1387</v>
       </c>
       <c r="D51" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E51" t="n">
         <v>5</v>
@@ -1936,7 +1936,7 @@
       <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr"/>
       <c r="K51" t="n">
-        <v>7117</v>
+        <v>5604</v>
       </c>
     </row>
     <row r="52">
@@ -1946,13 +1946,13 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>1146</v>
+        <v>882</v>
       </c>
       <c r="C52" t="n">
         <v>14</v>
       </c>
       <c r="D52" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E52" t="n">
         <v>1</v>
@@ -1973,7 +1973,7 @@
         <v>0</v>
       </c>
       <c r="K52" t="n">
-        <v>1168</v>
+        <v>903</v>
       </c>
     </row>
     <row r="53">
@@ -1983,13 +1983,13 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>1146</v>
+        <v>882</v>
       </c>
       <c r="C53" t="n">
         <v>14</v>
       </c>
       <c r="D53" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E53" t="n">
         <v>1</v>
@@ -2004,7 +2004,7 @@
       <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr"/>
       <c r="K53" t="n">
-        <v>1168</v>
+        <v>903</v>
       </c>
     </row>
     <row r="54">
@@ -2014,25 +2014,25 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>77424</v>
+        <v>51837</v>
       </c>
       <c r="C54" t="n">
-        <v>11410</v>
+        <v>10899</v>
       </c>
       <c r="D54" t="n">
-        <v>2515</v>
+        <v>2247</v>
       </c>
       <c r="E54" t="n">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="F54" t="n">
         <v>137</v>
       </c>
       <c r="G54" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H54" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I54" t="n">
         <v>2</v>
@@ -2041,7 +2041,7 @@
         <v>0</v>
       </c>
       <c r="K54" t="n">
-        <v>91780</v>
+        <v>65419</v>
       </c>
     </row>
   </sheetData>
@@ -2117,10 +2117,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1026</v>
+        <v>372</v>
       </c>
       <c r="C2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2" t="n">
         <v>14</v>
@@ -2141,7 +2141,7 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>1061</v>
+        <v>408</v>
       </c>
     </row>
     <row r="3">
@@ -2151,7 +2151,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>789</v>
+        <v>200</v>
       </c>
       <c r="C3" t="n">
         <v>7</v>
@@ -2175,7 +2175,7 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>808</v>
+        <v>219</v>
       </c>
     </row>
     <row r="4">
@@ -2185,31 +2185,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10288</v>
+        <v>7372</v>
       </c>
       <c r="C4" t="n">
-        <v>2615</v>
+        <v>2483</v>
       </c>
       <c r="D4" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="E4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F4" t="n">
         <v>8</v>
       </c>
       <c r="G4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>12996</v>
+        <v>9944</v>
       </c>
     </row>
     <row r="5">
@@ -2219,13 +2219,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1291</v>
+        <v>428</v>
       </c>
       <c r="C5" t="n">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="D5" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E5" t="n">
         <v>3</v>
@@ -2243,7 +2243,7 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>1414</v>
+        <v>546</v>
       </c>
     </row>
     <row r="6">
@@ -2253,16 +2253,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1702</v>
+        <v>1086</v>
       </c>
       <c r="C6" t="n">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D6" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
@@ -2277,7 +2277,7 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>1760</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="7">
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>907</v>
+        <v>506</v>
       </c>
       <c r="C7" t="n">
         <v>5</v>
@@ -2311,7 +2311,7 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>925</v>
+        <v>524</v>
       </c>
     </row>
     <row r="8">
@@ -2321,13 +2321,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>719</v>
+        <v>244</v>
       </c>
       <c r="C8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E8" t="n">
         <v>1</v>
@@ -2345,7 +2345,7 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>737</v>
+        <v>260</v>
       </c>
     </row>
     <row r="9">
@@ -2355,10 +2355,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>633</v>
+        <v>487</v>
       </c>
       <c r="C9" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D9" t="n">
         <v>2</v>
@@ -2379,7 +2379,7 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>661</v>
+        <v>514</v>
       </c>
     </row>
     <row r="10">
@@ -2389,7 +2389,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>90</v>
+        <v>69</v>
       </c>
       <c r="C10" t="n">
         <v>1</v>
@@ -2413,7 +2413,7 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>92</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11">
@@ -2423,13 +2423,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>139</v>
+        <v>69</v>
       </c>
       <c r="C11" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D11" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E11" t="n">
         <v>2</v>
@@ -2447,7 +2447,7 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>155</v>
+        <v>82</v>
       </c>
     </row>
     <row r="12">
@@ -2457,13 +2457,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4178</v>
+        <v>3192</v>
       </c>
       <c r="C12" t="n">
-        <v>1124</v>
+        <v>1075</v>
       </c>
       <c r="D12" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E12" t="n">
         <v>9</v>
@@ -2481,7 +2481,7 @@
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>5357</v>
+        <v>4320</v>
       </c>
     </row>
     <row r="13">
@@ -2491,7 +2491,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>163</v>
+        <v>138</v>
       </c>
       <c r="C13" t="n">
         <v>4</v>
@@ -2515,7 +2515,7 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>169</v>
+        <v>144</v>
       </c>
     </row>
     <row r="14">
@@ -2525,13 +2525,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>67</v>
+        <v>40</v>
       </c>
       <c r="C14" t="n">
         <v>2</v>
       </c>
       <c r="D14" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E14" t="n">
         <v>1</v>
@@ -2549,7 +2549,7 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>80</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15">
@@ -2559,7 +2559,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>279</v>
+        <v>62</v>
       </c>
       <c r="C15" t="n">
         <v>8</v>
@@ -2583,7 +2583,7 @@
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>292</v>
+        <v>75</v>
       </c>
     </row>
     <row r="16">
@@ -2593,16 +2593,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1129</v>
+        <v>742</v>
       </c>
       <c r="C16" t="n">
+        <v>10</v>
+      </c>
+      <c r="D16" t="n">
         <v>8</v>
       </c>
-      <c r="D16" t="n">
-        <v>10</v>
-      </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F16" t="n">
         <v>2</v>
@@ -2617,7 +2617,7 @@
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>1151</v>
+        <v>765</v>
       </c>
     </row>
     <row r="17">
@@ -2627,7 +2627,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>179</v>
+        <v>142</v>
       </c>
       <c r="C17" t="n">
         <v>2</v>
@@ -2651,7 +2651,7 @@
         <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>183</v>
+        <v>146</v>
       </c>
     </row>
     <row r="18">
@@ -2661,13 +2661,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>459</v>
+        <v>390</v>
       </c>
       <c r="C18" t="n">
         <v>12</v>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
@@ -2685,7 +2685,7 @@
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>472</v>
+        <v>402</v>
       </c>
     </row>
     <row r="19">
@@ -2695,13 +2695,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>817</v>
+        <v>410</v>
       </c>
       <c r="C19" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D19" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E19" t="n">
         <v>16</v>
@@ -2719,7 +2719,7 @@
         <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>910</v>
+        <v>499</v>
       </c>
     </row>
     <row r="20">
@@ -2729,10 +2729,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1175</v>
+        <v>813</v>
       </c>
       <c r="C20" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="D20" t="n">
         <v>2</v>
@@ -2753,7 +2753,7 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>1220</v>
+        <v>862</v>
       </c>
     </row>
     <row r="21">
@@ -2763,13 +2763,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>43</v>
+        <v>21</v>
       </c>
       <c r="C21" t="n">
         <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E21" t="n">
         <v>2</v>
@@ -2787,7 +2787,7 @@
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>49</v>
+        <v>26</v>
       </c>
     </row>
     <row r="22">
@@ -2797,10 +2797,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>630</v>
+        <v>512</v>
       </c>
       <c r="C22" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D22" t="n">
         <v>5</v>
@@ -2821,7 +2821,7 @@
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>654</v>
+        <v>535</v>
       </c>
     </row>
     <row r="23">
@@ -2831,10 +2831,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>976</v>
+        <v>804</v>
       </c>
       <c r="C23" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D23" t="n">
         <v>3</v>
@@ -2855,7 +2855,7 @@
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>995</v>
+        <v>822</v>
       </c>
     </row>
     <row r="24">
@@ -2865,10 +2865,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>931</v>
+        <v>798</v>
       </c>
       <c r="C24" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D24" t="n">
         <v>10</v>
@@ -2889,7 +2889,7 @@
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>969</v>
+        <v>835</v>
       </c>
     </row>
     <row r="25">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>183</v>
+        <v>30</v>
       </c>
       <c r="C25" t="n">
         <v>3</v>
@@ -2923,7 +2923,7 @@
         <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>189</v>
+        <v>36</v>
       </c>
     </row>
     <row r="26">
@@ -2933,13 +2933,13 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>4106</v>
+        <v>3427</v>
       </c>
       <c r="C26" t="n">
-        <v>2356</v>
+        <v>2247</v>
       </c>
       <c r="D26" t="n">
-        <v>1896</v>
+        <v>1701</v>
       </c>
       <c r="E26" t="n">
         <v>27</v>
@@ -2957,7 +2957,7 @@
         <v>1</v>
       </c>
       <c r="J26" t="n">
-        <v>8402</v>
+        <v>7419</v>
       </c>
     </row>
     <row r="27">
@@ -2967,13 +2967,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1236</v>
+        <v>543</v>
       </c>
       <c r="C27" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D27" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E27" t="n">
         <v>6</v>
@@ -2991,7 +2991,7 @@
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>1271</v>
+        <v>575</v>
       </c>
     </row>
     <row r="28">
@@ -3001,13 +3001,13 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1594</v>
+        <v>1025</v>
       </c>
       <c r="C28" t="n">
         <v>35</v>
       </c>
       <c r="D28" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E28" t="n">
         <v>7</v>
@@ -3025,7 +3025,7 @@
         <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>1653</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="29">
@@ -3035,13 +3035,13 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>440</v>
+        <v>276</v>
       </c>
       <c r="C29" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E29" t="n">
         <v>2</v>
@@ -3059,7 +3059,7 @@
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>455</v>
+        <v>289</v>
       </c>
     </row>
     <row r="30">
@@ -3069,7 +3069,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="C30" t="n">
         <v>7</v>
@@ -3093,7 +3093,7 @@
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>41</v>
+        <v>27</v>
       </c>
     </row>
     <row r="31">
@@ -3103,13 +3103,13 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>7797</v>
+        <v>5790</v>
       </c>
       <c r="C31" t="n">
-        <v>1678</v>
+        <v>1601</v>
       </c>
       <c r="D31" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="E31" t="n">
         <v>17</v>
@@ -3127,7 +3127,7 @@
         <v>0</v>
       </c>
       <c r="J31" t="n">
-        <v>9551</v>
+        <v>7463</v>
       </c>
     </row>
     <row r="32">
@@ -3137,13 +3137,13 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="C32" t="n">
         <v>2</v>
       </c>
       <c r="D32" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E32" t="n">
         <v>2</v>
@@ -3161,7 +3161,7 @@
         <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>53</v>
+        <v>34</v>
       </c>
     </row>
     <row r="33">
@@ -3171,7 +3171,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="C33" t="n">
         <v>5</v>
@@ -3195,7 +3195,7 @@
         <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="34">
@@ -3205,10 +3205,10 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>270</v>
+        <v>225</v>
       </c>
       <c r="C34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D34" t="n">
         <v>2</v>
@@ -3229,7 +3229,7 @@
         <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>275</v>
+        <v>231</v>
       </c>
     </row>
     <row r="35">
@@ -3239,10 +3239,10 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>796</v>
+        <v>679</v>
       </c>
       <c r="C35" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D35" t="n">
         <v>1</v>
@@ -3263,7 +3263,7 @@
         <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>812</v>
+        <v>694</v>
       </c>
     </row>
     <row r="36">
@@ -3273,13 +3273,13 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>2622</v>
+        <v>1756</v>
       </c>
       <c r="C36" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="D36" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E36" t="n">
         <v>2</v>
@@ -3297,7 +3297,7 @@
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>2739</v>
+        <v>1873</v>
       </c>
     </row>
     <row r="37">
@@ -3307,7 +3307,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>463</v>
+        <v>397</v>
       </c>
       <c r="C37" t="n">
         <v>5</v>
@@ -3331,7 +3331,7 @@
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>469</v>
+        <v>403</v>
       </c>
     </row>
     <row r="38">
@@ -3341,7 +3341,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>384</v>
+        <v>175</v>
       </c>
       <c r="C38" t="n">
         <v>1</v>
@@ -3365,7 +3365,7 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>390</v>
+        <v>181</v>
       </c>
     </row>
     <row r="39">
@@ -3375,10 +3375,10 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>430</v>
+        <v>363</v>
       </c>
       <c r="C39" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D39" t="n">
         <v>2</v>
@@ -3399,7 +3399,7 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>446</v>
+        <v>380</v>
       </c>
     </row>
     <row r="40">
@@ -3409,13 +3409,13 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>488</v>
+        <v>259</v>
       </c>
       <c r="C40" t="n">
         <v>0</v>
       </c>
       <c r="D40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E40" t="n">
         <v>3</v>
@@ -3433,7 +3433,7 @@
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>499</v>
+        <v>269</v>
       </c>
     </row>
     <row r="41">
@@ -3443,7 +3443,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>142</v>
+        <v>21</v>
       </c>
       <c r="C41" t="n">
         <v>2</v>
@@ -3467,7 +3467,7 @@
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>153</v>
+        <v>32</v>
       </c>
     </row>
     <row r="42">
@@ -3477,7 +3477,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>680</v>
+        <v>379</v>
       </c>
       <c r="C42" t="n">
         <v>5</v>
@@ -3501,7 +3501,7 @@
         <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>690</v>
+        <v>389</v>
       </c>
     </row>
     <row r="43">
@@ -3511,13 +3511,13 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>1042</v>
+        <v>708</v>
       </c>
       <c r="C43" t="n">
         <v>10</v>
       </c>
       <c r="D43" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E43" t="n">
         <v>2</v>
@@ -3535,7 +3535,7 @@
         <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>1058</v>
+        <v>723</v>
       </c>
     </row>
     <row r="44">
@@ -3545,10 +3545,10 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>953</v>
+        <v>738</v>
       </c>
       <c r="C44" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D44" t="n">
         <v>6</v>
@@ -3569,7 +3569,7 @@
         <v>1</v>
       </c>
       <c r="J44" t="n">
-        <v>988</v>
+        <v>775</v>
       </c>
     </row>
     <row r="45">
@@ -3579,10 +3579,10 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>110</v>
+        <v>20</v>
       </c>
       <c r="C45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D45" t="n">
         <v>1</v>
@@ -3603,7 +3603,7 @@
         <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>116</v>
+        <v>25</v>
       </c>
     </row>
     <row r="46">
@@ -3613,16 +3613,16 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>697</v>
+        <v>223</v>
       </c>
       <c r="C46" t="n">
+        <v>4</v>
+      </c>
+      <c r="D46" t="n">
+        <v>4</v>
+      </c>
+      <c r="E46" t="n">
         <v>5</v>
-      </c>
-      <c r="D46" t="n">
-        <v>6</v>
-      </c>
-      <c r="E46" t="n">
-        <v>4</v>
       </c>
       <c r="F46" t="n">
         <v>6</v>
@@ -3637,7 +3637,7 @@
         <v>0</v>
       </c>
       <c r="J46" t="n">
-        <v>721</v>
+        <v>245</v>
       </c>
     </row>
     <row r="47">
@@ -3647,13 +3647,13 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>92</v>
+        <v>54</v>
       </c>
       <c r="C47" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D47" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E47" t="n">
         <v>2</v>
@@ -3671,7 +3671,7 @@
         <v>0</v>
       </c>
       <c r="J47" t="n">
-        <v>101</v>
+        <v>63</v>
       </c>
     </row>
     <row r="48">
@@ -3681,13 +3681,13 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>3044</v>
+        <v>2106</v>
       </c>
       <c r="C48" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="D48" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E48" t="n">
         <v>7</v>
@@ -3705,7 +3705,7 @@
         <v>0</v>
       </c>
       <c r="J48" t="n">
-        <v>3117</v>
+        <v>2166</v>
       </c>
     </row>
     <row r="49">
@@ -3715,7 +3715,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>627</v>
+        <v>541</v>
       </c>
       <c r="C49" t="n">
         <v>18</v>
@@ -3739,7 +3739,7 @@
         <v>0</v>
       </c>
       <c r="J49" t="n">
-        <v>648</v>
+        <v>562</v>
       </c>
     </row>
     <row r="50">
@@ -3749,10 +3749,10 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>377</v>
+        <v>265</v>
       </c>
       <c r="C50" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D50" t="n">
         <v>3</v>
@@ -3773,7 +3773,7 @@
         <v>0</v>
       </c>
       <c r="J50" t="n">
-        <v>393</v>
+        <v>279</v>
       </c>
     </row>
     <row r="51">
@@ -3783,7 +3783,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>866</v>
+        <v>473</v>
       </c>
       <c r="C51" t="n">
         <v>0</v>
@@ -3807,7 +3807,7 @@
         <v>0</v>
       </c>
       <c r="J51" t="n">
-        <v>870</v>
+        <v>477</v>
       </c>
     </row>
     <row r="52">
@@ -3817,16 +3817,16 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>5855</v>
+        <v>4393</v>
       </c>
       <c r="C52" t="n">
-        <v>1274</v>
+        <v>1241</v>
       </c>
       <c r="D52" t="n">
-        <v>141</v>
+        <v>124</v>
       </c>
       <c r="E52" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F52" t="n">
         <v>5</v>
@@ -3841,7 +3841,7 @@
         <v>0</v>
       </c>
       <c r="J52" t="n">
-        <v>7288</v>
+        <v>5777</v>
       </c>
     </row>
     <row r="53">
@@ -3851,13 +3851,13 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>538</v>
+        <v>168</v>
       </c>
       <c r="C53" t="n">
         <v>6</v>
       </c>
       <c r="D53" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E53" t="n">
         <v>0</v>
@@ -3875,7 +3875,7 @@
         <v>0</v>
       </c>
       <c r="J53" t="n">
-        <v>554</v>
+        <v>182</v>
       </c>
     </row>
     <row r="54">
@@ -3885,10 +3885,10 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>216</v>
+        <v>177</v>
       </c>
       <c r="C54" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D54" t="n">
         <v>0</v>
@@ -3909,7 +3909,7 @@
         <v>0</v>
       </c>
       <c r="J54" t="n">
-        <v>222</v>
+        <v>182</v>
       </c>
     </row>
     <row r="55">
@@ -3919,13 +3919,13 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>5352</v>
+        <v>4040</v>
       </c>
       <c r="C55" t="n">
-        <v>1413</v>
+        <v>1332</v>
       </c>
       <c r="D55" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E55" t="n">
         <v>5</v>
@@ -3943,7 +3943,7 @@
         <v>0</v>
       </c>
       <c r="J55" t="n">
-        <v>6816</v>
+        <v>5421</v>
       </c>
     </row>
     <row r="56">
@@ -3953,10 +3953,10 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>145</v>
+        <v>31</v>
       </c>
       <c r="C56" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D56" t="n">
         <v>1</v>
@@ -3977,7 +3977,7 @@
         <v>0</v>
       </c>
       <c r="J56" t="n">
-        <v>161</v>
+        <v>48</v>
       </c>
     </row>
     <row r="57">
@@ -3987,10 +3987,10 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>412</v>
+        <v>347</v>
       </c>
       <c r="C57" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D57" t="n">
         <v>3</v>
@@ -4011,7 +4011,7 @@
         <v>0</v>
       </c>
       <c r="J57" t="n">
-        <v>436</v>
+        <v>370</v>
       </c>
     </row>
     <row r="58">
@@ -4021,13 +4021,13 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="C58" t="n">
         <v>2</v>
       </c>
       <c r="D58" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E58" t="n">
         <v>2</v>
@@ -4045,7 +4045,7 @@
         <v>0</v>
       </c>
       <c r="J58" t="n">
-        <v>48</v>
+        <v>30</v>
       </c>
     </row>
     <row r="59">
@@ -4055,7 +4055,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="C59" t="n">
         <v>1</v>
@@ -4079,7 +4079,7 @@
         <v>0</v>
       </c>
       <c r="J59" t="n">
-        <v>47</v>
+        <v>32</v>
       </c>
     </row>
     <row r="60">
@@ -4089,13 +4089,13 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>989</v>
+        <v>557</v>
       </c>
       <c r="C60" t="n">
         <v>4</v>
       </c>
       <c r="D60" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E60" t="n">
         <v>6</v>
@@ -4113,7 +4113,7 @@
         <v>0</v>
       </c>
       <c r="J60" t="n">
-        <v>1004</v>
+        <v>571</v>
       </c>
     </row>
     <row r="61">
@@ -4123,10 +4123,10 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>1118</v>
+        <v>547</v>
       </c>
       <c r="C61" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D61" t="n">
         <v>18</v>
@@ -4147,7 +4147,7 @@
         <v>0</v>
       </c>
       <c r="J61" t="n">
-        <v>1159</v>
+        <v>587</v>
       </c>
     </row>
     <row r="62">
@@ -4157,10 +4157,10 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>755</v>
+        <v>496</v>
       </c>
       <c r="C62" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D62" t="n">
         <v>3</v>
@@ -4181,7 +4181,7 @@
         <v>0</v>
       </c>
       <c r="J62" t="n">
-        <v>778</v>
+        <v>516</v>
       </c>
     </row>
     <row r="63">
@@ -4191,13 +4191,13 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>2489</v>
+        <v>893</v>
       </c>
       <c r="C63" t="n">
         <v>14</v>
       </c>
       <c r="D63" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E63" t="n">
         <v>8</v>
@@ -4215,7 +4215,7 @@
         <v>0</v>
       </c>
       <c r="J63" t="n">
-        <v>2536</v>
+        <v>937</v>
       </c>
     </row>
     <row r="64">
@@ -4225,13 +4225,13 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>1292</v>
+        <v>681</v>
       </c>
       <c r="C64" t="n">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="D64" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E64" t="n">
         <v>2</v>
@@ -4249,7 +4249,7 @@
         <v>0</v>
       </c>
       <c r="J64" t="n">
-        <v>1464</v>
+        <v>840</v>
       </c>
     </row>
     <row r="65">
@@ -4259,31 +4259,31 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>77424</v>
+        <v>51837</v>
       </c>
       <c r="C65" t="n">
-        <v>11410</v>
+        <v>10899</v>
       </c>
       <c r="D65" t="n">
-        <v>2515</v>
+        <v>2247</v>
       </c>
       <c r="E65" t="n">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="F65" t="n">
         <v>137</v>
       </c>
       <c r="G65" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H65" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I65" t="n">
         <v>2</v>
       </c>
       <c r="J65" t="n">
-        <v>91780</v>
+        <v>65419</v>
       </c>
     </row>
   </sheetData>
@@ -4359,31 +4359,31 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>10035</v>
+        <v>7096</v>
       </c>
       <c r="C2" t="n">
-        <v>2579</v>
+        <v>2428</v>
       </c>
       <c r="D2" t="n">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="E2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F2" t="n">
         <v>7</v>
       </c>
       <c r="G2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>12706</v>
+        <v>9612</v>
       </c>
     </row>
     <row r="3">
@@ -4393,13 +4393,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3997</v>
+        <v>3015</v>
       </c>
       <c r="C3" t="n">
-        <v>1124</v>
+        <v>1066</v>
       </c>
       <c r="D3" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E3" t="n">
         <v>8</v>
@@ -4417,7 +4417,7 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>5173</v>
+        <v>4131</v>
       </c>
     </row>
     <row r="4">
@@ -4427,13 +4427,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3394</v>
+        <v>2860</v>
       </c>
       <c r="C4" t="n">
-        <v>2273</v>
+        <v>2169</v>
       </c>
       <c r="D4" t="n">
-        <v>1964</v>
+        <v>1768</v>
       </c>
       <c r="E4" t="n">
         <v>23</v>
@@ -4451,7 +4451,7 @@
         <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>7665</v>
+        <v>6831</v>
       </c>
     </row>
     <row r="5">
@@ -4461,10 +4461,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>225</v>
+        <v>134</v>
       </c>
       <c r="C5" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D5" t="n">
         <v>4</v>
@@ -4485,7 +4485,7 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>260</v>
+        <v>167</v>
       </c>
     </row>
     <row r="6">
@@ -4495,13 +4495,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3010</v>
+        <v>2088</v>
       </c>
       <c r="C6" t="n">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="D6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E6" t="n">
         <v>7</v>
@@ -4519,7 +4519,7 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>3074</v>
+        <v>2141</v>
       </c>
     </row>
     <row r="7">
@@ -4529,13 +4529,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>588</v>
+        <v>111</v>
       </c>
       <c r="C7" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>
@@ -4553,7 +4553,7 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>617</v>
+        <v>139</v>
       </c>
     </row>
     <row r="8">
@@ -4563,16 +4563,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1712</v>
+        <v>1099</v>
       </c>
       <c r="C8" t="n">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D8" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
@@ -4587,7 +4587,7 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>1771</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="9">
@@ -4597,13 +4597,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1021</v>
+        <v>691</v>
       </c>
       <c r="C9" t="n">
         <v>10</v>
       </c>
       <c r="D9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E9" t="n">
         <v>2</v>
@@ -4621,7 +4621,7 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>1037</v>
+        <v>706</v>
       </c>
     </row>
     <row r="10">
@@ -4631,10 +4631,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>743</v>
+        <v>490</v>
       </c>
       <c r="C10" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D10" t="n">
         <v>3</v>
@@ -4655,7 +4655,7 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>765</v>
+        <v>509</v>
       </c>
     </row>
     <row r="11">
@@ -4665,13 +4665,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3155</v>
+        <v>990</v>
       </c>
       <c r="C11" t="n">
         <v>19</v>
       </c>
       <c r="D11" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E11" t="n">
         <v>16</v>
@@ -4689,7 +4689,7 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>3218</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="12">
@@ -4699,10 +4699,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="C12" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D12" t="n">
         <v>1</v>
@@ -4723,7 +4723,7 @@
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>94</v>
+        <v>89</v>
       </c>
     </row>
     <row r="13">
@@ -4733,10 +4733,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>123</v>
+        <v>113</v>
       </c>
       <c r="C13" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
@@ -4757,7 +4757,7 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>144</v>
+        <v>135</v>
       </c>
     </row>
     <row r="14">
@@ -4767,10 +4767,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
@@ -4791,7 +4791,7 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="15">
@@ -4801,10 +4801,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="C15" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D15" t="n">
         <v>1</v>
@@ -4825,7 +4825,7 @@
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>125</v>
+        <v>115</v>
       </c>
     </row>
     <row r="16">
@@ -4835,10 +4835,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="C16" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
@@ -4859,7 +4859,7 @@
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>109</v>
+        <v>99</v>
       </c>
     </row>
     <row r="17">
@@ -4869,10 +4869,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="C17" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
@@ -4893,7 +4893,7 @@
         <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>137</v>
+        <v>128</v>
       </c>
     </row>
     <row r="18">
@@ -4903,10 +4903,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="C18" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
@@ -4927,7 +4927,7 @@
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="19">
@@ -4937,10 +4937,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="C19" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D19" t="n">
         <v>3</v>
@@ -4961,7 +4961,7 @@
         <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>129</v>
+        <v>118</v>
       </c>
     </row>
     <row r="20">
@@ -4971,7 +4971,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="C20" t="n">
         <v>13</v>
@@ -4995,7 +4995,7 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>74</v>
+        <v>68</v>
       </c>
     </row>
     <row r="21">
@@ -5005,10 +5005,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>143</v>
+        <v>126</v>
       </c>
       <c r="C21" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
@@ -5029,7 +5029,7 @@
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>173</v>
+        <v>161</v>
       </c>
     </row>
     <row r="22">
@@ -5039,10 +5039,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="C22" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
@@ -5063,7 +5063,7 @@
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>124</v>
+        <v>115</v>
       </c>
     </row>
     <row r="23">
@@ -5073,10 +5073,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>198</v>
+        <v>170</v>
       </c>
       <c r="C23" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D23" t="n">
         <v>2</v>
@@ -5097,7 +5097,7 @@
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>243</v>
+        <v>217</v>
       </c>
     </row>
     <row r="24">
@@ -5107,7 +5107,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>302</v>
+        <v>260</v>
       </c>
       <c r="C24" t="n">
         <v>9</v>
@@ -5131,7 +5131,7 @@
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>324</v>
+        <v>282</v>
       </c>
     </row>
     <row r="25">
@@ -5141,7 +5141,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C25" t="n">
         <v>9</v>
@@ -5165,7 +5165,7 @@
         <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>77</v>
+        <v>73</v>
       </c>
     </row>
     <row r="26">
@@ -5175,13 +5175,13 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>3791</v>
+        <v>2563</v>
       </c>
       <c r="C26" t="n">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="D26" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E26" t="n">
         <v>5</v>
@@ -5199,7 +5199,7 @@
         <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>3950</v>
+        <v>2726</v>
       </c>
     </row>
     <row r="27">
@@ -5209,13 +5209,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1411</v>
+        <v>775</v>
       </c>
       <c r="C27" t="n">
         <v>5</v>
       </c>
       <c r="D27" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E27" t="n">
         <v>6</v>
@@ -5233,7 +5233,7 @@
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>1434</v>
+        <v>797</v>
       </c>
     </row>
     <row r="28">
@@ -5243,16 +5243,16 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>3922</v>
+        <v>1414</v>
       </c>
       <c r="C28" t="n">
         <v>47</v>
       </c>
       <c r="D28" t="n">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="E28" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F28" t="n">
         <v>19</v>
@@ -5267,7 +5267,7 @@
         <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>4066</v>
+        <v>1548</v>
       </c>
     </row>
     <row r="29">
@@ -5277,7 +5277,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>418</v>
+        <v>300</v>
       </c>
       <c r="C29" t="n">
         <v>8</v>
@@ -5301,7 +5301,7 @@
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>458</v>
+        <v>340</v>
       </c>
     </row>
     <row r="30">
@@ -5311,16 +5311,16 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1572</v>
+        <v>1014</v>
       </c>
       <c r="C30" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D30" t="n">
+        <v>2</v>
+      </c>
+      <c r="E30" t="n">
         <v>5</v>
-      </c>
-      <c r="E30" t="n">
-        <v>4</v>
       </c>
       <c r="F30" t="n">
         <v>6</v>
@@ -5335,7 +5335,7 @@
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>1601</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="31">
@@ -5345,13 +5345,13 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1220</v>
+        <v>329</v>
       </c>
       <c r="C31" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D31" t="n">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="E31" t="n">
         <v>15</v>
@@ -5369,7 +5369,7 @@
         <v>1</v>
       </c>
       <c r="J31" t="n">
-        <v>1294</v>
+        <v>396</v>
       </c>
     </row>
     <row r="32">
@@ -5379,10 +5379,10 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>9302</v>
+        <v>7601</v>
       </c>
       <c r="C32" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D32" t="n">
         <v>13</v>
@@ -5403,7 +5403,7 @@
         <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>9441</v>
+        <v>7737</v>
       </c>
     </row>
     <row r="33">
@@ -5413,13 +5413,13 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>948</v>
+        <v>458</v>
       </c>
       <c r="C33" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="D33" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E33" t="n">
         <v>10</v>
@@ -5437,7 +5437,7 @@
         <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>1093</v>
+        <v>597</v>
       </c>
     </row>
     <row r="34">
@@ -5447,13 +5447,13 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1599</v>
+        <v>700</v>
       </c>
       <c r="C34" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D34" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E34" t="n">
         <v>7</v>
@@ -5471,7 +5471,7 @@
         <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>1635</v>
+        <v>733</v>
       </c>
     </row>
     <row r="35">
@@ -5481,10 +5481,10 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>231</v>
+        <v>20</v>
       </c>
       <c r="C35" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D35" t="n">
         <v>3</v>
@@ -5505,7 +5505,7 @@
         <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>248</v>
+        <v>36</v>
       </c>
     </row>
     <row r="36">
@@ -5515,13 +5515,13 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>2483</v>
+        <v>1329</v>
       </c>
       <c r="C36" t="n">
         <v>8</v>
       </c>
       <c r="D36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E36" t="n">
         <v>11</v>
@@ -5539,7 +5539,7 @@
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>2507</v>
+        <v>1352</v>
       </c>
     </row>
     <row r="37">
@@ -5549,10 +5549,10 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1176</v>
+        <v>592</v>
       </c>
       <c r="C37" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D37" t="n">
         <v>8</v>
@@ -5573,7 +5573,7 @@
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>1205</v>
+        <v>620</v>
       </c>
     </row>
     <row r="38">
@@ -5583,13 +5583,13 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>8380</v>
+        <v>6193</v>
       </c>
       <c r="C38" t="n">
-        <v>1840</v>
+        <v>1760</v>
       </c>
       <c r="D38" t="n">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="E38" t="n">
         <v>16</v>
@@ -5607,7 +5607,7 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>10330</v>
+        <v>8054</v>
       </c>
     </row>
     <row r="39">
@@ -5617,13 +5617,13 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1146</v>
+        <v>882</v>
       </c>
       <c r="C39" t="n">
         <v>14</v>
       </c>
       <c r="D39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E39" t="n">
         <v>1</v>
@@ -5641,7 +5641,7 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>1168</v>
+        <v>903</v>
       </c>
     </row>
     <row r="40">
@@ -5651,16 +5651,16 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>4855</v>
+        <v>3606</v>
       </c>
       <c r="C40" t="n">
-        <v>1129</v>
+        <v>1096</v>
       </c>
       <c r="D40" t="n">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="E40" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F40" t="n">
         <v>4</v>
@@ -5675,7 +5675,7 @@
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>6107</v>
+        <v>4813</v>
       </c>
     </row>
     <row r="41">
@@ -5685,13 +5685,13 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>5590</v>
+        <v>4169</v>
       </c>
       <c r="C41" t="n">
-        <v>1477</v>
+        <v>1387</v>
       </c>
       <c r="D41" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E41" t="n">
         <v>5</v>
@@ -5709,7 +5709,7 @@
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>7117</v>
+        <v>5604</v>
       </c>
     </row>
     <row r="42">
@@ -5719,31 +5719,31 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>77424</v>
+        <v>51837</v>
       </c>
       <c r="C42" t="n">
-        <v>11410</v>
+        <v>10899</v>
       </c>
       <c r="D42" t="n">
-        <v>2515</v>
+        <v>2247</v>
       </c>
       <c r="E42" t="n">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="F42" t="n">
         <v>137</v>
       </c>
       <c r="G42" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H42" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I42" t="n">
         <v>2</v>
       </c>
       <c r="J42" t="n">
-        <v>91780</v>
+        <v>65419</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): manual update to 95,728 matching Metabase
</commit_message>
<xml_diff>
--- a/BaoCao_TonKho.xlsx
+++ b/BaoCao_TonKho.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>05/06/2026 01:02:39</t>
+          <t>05/06/2026 01:34:11</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -579,13 +579,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>5469</v>
+        <v>11132</v>
       </c>
       <c r="C7" t="n">
-        <v>140</v>
+        <v>164</v>
       </c>
       <c r="D7" t="n">
-        <v>35</v>
+        <v>52</v>
       </c>
       <c r="E7" t="n">
         <v>31</v>
@@ -606,7 +606,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>5699</v>
+        <v>11403</v>
       </c>
     </row>
     <row r="8">
@@ -616,13 +616,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2088</v>
+        <v>3364</v>
       </c>
       <c r="C8" t="n">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="D8" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E8" t="n">
         <v>7</v>
@@ -637,7 +637,7 @@
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="n">
-        <v>2141</v>
+        <v>3434</v>
       </c>
     </row>
     <row r="9">
@@ -647,13 +647,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>111</v>
+        <v>787</v>
       </c>
       <c r="C9" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="D9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E9" t="n">
         <v>3</v>
@@ -668,7 +668,7 @@
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="n">
-        <v>139</v>
+        <v>806</v>
       </c>
     </row>
     <row r="10">
@@ -678,13 +678,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1099</v>
+        <v>1894</v>
       </c>
       <c r="C10" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="D10" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E10" t="n">
         <v>3</v>
@@ -695,7 +695,7 @@
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="n">
-        <v>1154</v>
+        <v>1960</v>
       </c>
     </row>
     <row r="11">
@@ -705,13 +705,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>691</v>
+        <v>1128</v>
       </c>
       <c r="C11" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E11" t="n">
         <v>2</v>
@@ -724,7 +724,7 @@
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="n">
-        <v>706</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="12">
@@ -734,13 +734,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>490</v>
+        <v>845</v>
       </c>
       <c r="C12" t="n">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="D12" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="n">
@@ -751,7 +751,7 @@
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="n">
-        <v>509</v>
+        <v>877</v>
       </c>
     </row>
     <row r="13">
@@ -761,13 +761,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>990</v>
+        <v>3114</v>
       </c>
       <c r="C13" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D13" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="E13" t="n">
         <v>16</v>
@@ -784,7 +784,7 @@
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="n">
-        <v>1050</v>
+        <v>3178</v>
       </c>
     </row>
     <row r="14">
@@ -794,13 +794,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1318</v>
+        <v>1240</v>
       </c>
       <c r="C14" t="n">
-        <v>330</v>
+        <v>459</v>
       </c>
       <c r="D14" t="n">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="E14" t="n">
         <v>6</v>
@@ -809,10 +809,10 @@
         <v>11</v>
       </c>
       <c r="G14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>1681</v>
+        <v>1744</v>
       </c>
     </row>
     <row r="15">
@@ -831,13 +831,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C15" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
@@ -846,7 +846,7 @@
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="n">
-        <v>89</v>
+        <v>94</v>
       </c>
     </row>
     <row r="16">
@@ -856,10 +856,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="C16" t="n">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
@@ -871,7 +871,7 @@
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="n">
-        <v>135</v>
+        <v>148</v>
       </c>
     </row>
     <row r="17">
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="C17" t="n">
         <v>2</v>
@@ -896,7 +896,7 @@
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="n">
-        <v>18</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18">
@@ -906,13 +906,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="C18" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E18" t="n">
         <v>1</v>
@@ -923,7 +923,7 @@
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="n">
-        <v>115</v>
+        <v>131</v>
       </c>
     </row>
     <row r="19">
@@ -933,10 +933,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C19" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="n">
@@ -952,7 +952,7 @@
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="n">
-        <v>99</v>
+        <v>111</v>
       </c>
     </row>
     <row r="20">
@@ -962,10 +962,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C20" t="n">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
@@ -977,7 +977,7 @@
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="n">
-        <v>128</v>
+        <v>146</v>
       </c>
     </row>
     <row r="21">
@@ -987,10 +987,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C21" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
@@ -1004,7 +1004,7 @@
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="n">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
     <row r="22">
@@ -1017,10 +1017,10 @@
         <v>80</v>
       </c>
       <c r="C22" t="n">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="D22" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="n">
@@ -1031,7 +1031,7 @@
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="n">
-        <v>118</v>
+        <v>132</v>
       </c>
     </row>
     <row r="23">
@@ -1041,10 +1041,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="C23" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
@@ -1056,7 +1056,7 @@
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
     </row>
     <row r="24">
@@ -1066,10 +1066,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="C24" t="n">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr"/>
@@ -1079,7 +1079,7 @@
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="n">
-        <v>161</v>
+        <v>180</v>
       </c>
     </row>
     <row r="25">
@@ -1089,10 +1089,10 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C25" t="n">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr"/>
@@ -1102,7 +1102,7 @@
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="n">
-        <v>115</v>
+        <v>127</v>
       </c>
     </row>
     <row r="26">
@@ -1112,10 +1112,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>170</v>
+        <v>187</v>
       </c>
       <c r="C26" t="n">
-        <v>44</v>
+        <v>71</v>
       </c>
       <c r="D26" t="n">
         <v>2</v>
@@ -1129,7 +1129,7 @@
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="n">
-        <v>217</v>
+        <v>261</v>
       </c>
     </row>
     <row r="27">
@@ -1139,13 +1139,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>260</v>
+        <v>136</v>
       </c>
       <c r="C27" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D27" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E27" t="n">
         <v>1</v>
@@ -1153,14 +1153,14 @@
       <c r="F27" t="n">
         <v>5</v>
       </c>
-      <c r="G27" t="n">
-        <v>1</v>
-      </c>
-      <c r="H27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="n">
+        <v>1</v>
+      </c>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="n">
-        <v>282</v>
+        <v>157</v>
       </c>
     </row>
     <row r="28">
@@ -1170,10 +1170,10 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C28" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr"/>
@@ -1185,7 +1185,7 @@
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="n">
-        <v>73</v>
+        <v>78</v>
       </c>
     </row>
     <row r="29">
@@ -1195,7 +1195,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>134</v>
+        <v>349</v>
       </c>
       <c r="C29" t="n">
         <v>25</v>
@@ -1222,7 +1222,7 @@
         <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>167</v>
+        <v>382</v>
       </c>
     </row>
     <row r="30">
@@ -1232,7 +1232,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>134</v>
+        <v>349</v>
       </c>
       <c r="C30" t="n">
         <v>25</v>
@@ -1253,7 +1253,7 @@
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="n">
-        <v>167</v>
+        <v>382</v>
       </c>
     </row>
     <row r="31">
@@ -1263,25 +1263,25 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>17095</v>
+        <v>28225</v>
       </c>
       <c r="C31" t="n">
-        <v>484</v>
+        <v>753</v>
       </c>
       <c r="D31" t="n">
-        <v>142</v>
+        <v>164</v>
       </c>
       <c r="E31" t="n">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="F31" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G31" t="n">
         <v>25</v>
       </c>
       <c r="H31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I31" t="n">
         <v>1</v>
@@ -1290,7 +1290,7 @@
         <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>17924</v>
+        <v>29348</v>
       </c>
     </row>
     <row r="32">
@@ -1300,28 +1300,30 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>2563</v>
+        <v>4044</v>
       </c>
       <c r="C32" t="n">
-        <v>147</v>
+        <v>360</v>
       </c>
       <c r="D32" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E32" t="n">
         <v>5</v>
       </c>
       <c r="F32" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G32" t="n">
-        <v>2</v>
-      </c>
-      <c r="H32" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H32" t="n">
+        <v>1</v>
+      </c>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="n">
-        <v>2726</v>
+        <v>4422</v>
       </c>
     </row>
     <row r="33">
@@ -1331,13 +1333,13 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>775</v>
+        <v>1644</v>
       </c>
       <c r="C33" t="n">
+        <v>13</v>
+      </c>
+      <c r="D33" t="n">
         <v>5</v>
-      </c>
-      <c r="D33" t="n">
-        <v>4</v>
       </c>
       <c r="E33" t="n">
         <v>6</v>
@@ -1354,7 +1356,7 @@
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="n">
-        <v>797</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="34">
@@ -1364,16 +1366,16 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1414</v>
+        <v>2984</v>
       </c>
       <c r="C34" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D34" t="n">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="E34" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F34" t="n">
         <v>19</v>
@@ -1385,7 +1387,7 @@
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="n">
-        <v>1548</v>
+        <v>3129</v>
       </c>
     </row>
     <row r="35">
@@ -1395,10 +1397,10 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>300</v>
+        <v>474</v>
       </c>
       <c r="C35" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D35" t="n">
         <v>10</v>
@@ -1418,7 +1420,7 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="n">
-        <v>340</v>
+        <v>517</v>
       </c>
     </row>
     <row r="36">
@@ -1428,13 +1430,13 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1014</v>
+        <v>1760</v>
       </c>
       <c r="C36" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="D36" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E36" t="n">
         <v>5</v>
@@ -1449,7 +1451,7 @@
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="n">
-        <v>1042</v>
+        <v>1804</v>
       </c>
     </row>
     <row r="37">
@@ -1459,16 +1461,16 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>329</v>
+        <v>2799</v>
       </c>
       <c r="C37" t="n">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="D37" t="n">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="E37" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="n">
@@ -1480,7 +1482,7 @@
       </c>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="n">
-        <v>396</v>
+        <v>2884</v>
       </c>
     </row>
     <row r="38">
@@ -1490,10 +1492,10 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>7601</v>
+        <v>3557</v>
       </c>
       <c r="C38" t="n">
-        <v>100</v>
+        <v>69</v>
       </c>
       <c r="D38" t="n">
         <v>13</v>
@@ -1511,7 +1513,7 @@
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="n">
-        <v>7737</v>
+        <v>3662</v>
       </c>
     </row>
     <row r="39">
@@ -1521,22 +1523,22 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>458</v>
+        <v>4386</v>
       </c>
       <c r="C39" t="n">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="D39" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E39" t="n">
         <v>10</v>
       </c>
       <c r="F39" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H39" t="n">
         <v>1</v>
@@ -1544,7 +1546,7 @@
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="n">
-        <v>597</v>
+        <v>4530</v>
       </c>
     </row>
     <row r="40">
@@ -1554,16 +1556,16 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>700</v>
+        <v>1902</v>
       </c>
       <c r="C40" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="D40" t="n">
         <v>8</v>
       </c>
       <c r="E40" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F40" t="n">
         <v>4</v>
@@ -1575,7 +1577,7 @@
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="n">
-        <v>733</v>
+        <v>1949</v>
       </c>
     </row>
     <row r="41">
@@ -1585,10 +1587,10 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>20</v>
+        <v>341</v>
       </c>
       <c r="C41" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D41" t="n">
         <v>3</v>
@@ -1606,7 +1608,7 @@
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="n">
-        <v>36</v>
+        <v>360</v>
       </c>
     </row>
     <row r="42">
@@ -1616,13 +1618,13 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1329</v>
+        <v>3013</v>
       </c>
       <c r="C42" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="D42" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E42" t="n">
         <v>11</v>
@@ -1635,7 +1637,7 @@
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="n">
-        <v>1352</v>
+        <v>3044</v>
       </c>
     </row>
     <row r="43">
@@ -1645,16 +1647,16 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>592</v>
+        <v>1321</v>
       </c>
       <c r="C43" t="n">
-        <v>13</v>
+        <v>36</v>
       </c>
       <c r="D43" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E43" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F43" t="n">
         <v>1</v>
@@ -1666,7 +1668,7 @@
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="n">
-        <v>620</v>
+        <v>1372</v>
       </c>
     </row>
     <row r="44">
@@ -1676,26 +1678,26 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>2860</v>
+        <v>3300</v>
       </c>
       <c r="C44" t="n">
-        <v>2169</v>
+        <v>2289</v>
       </c>
       <c r="D44" t="n">
-        <v>1768</v>
+        <v>1852</v>
       </c>
       <c r="E44" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F44" t="n">
         <v>3</v>
       </c>
       <c r="G44" t="n">
+        <v>3</v>
+      </c>
+      <c r="H44" t="n">
         <v>4</v>
       </c>
-      <c r="H44" t="n">
-        <v>3</v>
-      </c>
       <c r="I44" t="n">
         <v>1</v>
       </c>
@@ -1703,7 +1705,7 @@
         <v>0</v>
       </c>
       <c r="K44" t="n">
-        <v>6831</v>
+        <v>7478</v>
       </c>
     </row>
     <row r="45">
@@ -1713,32 +1715,32 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>2860</v>
+        <v>3300</v>
       </c>
       <c r="C45" t="n">
-        <v>2169</v>
+        <v>2289</v>
       </c>
       <c r="D45" t="n">
-        <v>1768</v>
+        <v>1852</v>
       </c>
       <c r="E45" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F45" t="n">
         <v>3</v>
       </c>
       <c r="G45" t="n">
+        <v>3</v>
+      </c>
+      <c r="H45" t="n">
         <v>4</v>
-      </c>
-      <c r="H45" t="n">
-        <v>3</v>
       </c>
       <c r="I45" t="n">
         <v>1</v>
       </c>
       <c r="J45" t="inlineStr"/>
       <c r="K45" t="n">
-        <v>6831</v>
+        <v>7478</v>
       </c>
     </row>
     <row r="46">
@@ -1748,16 +1750,16 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>24079</v>
+        <v>32632</v>
       </c>
       <c r="C46" t="n">
-        <v>7737</v>
+        <v>11011</v>
       </c>
       <c r="D46" t="n">
-        <v>283</v>
+        <v>326</v>
       </c>
       <c r="E46" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F46" t="n">
         <v>44</v>
@@ -1775,7 +1777,7 @@
         <v>0</v>
       </c>
       <c r="K46" t="n">
-        <v>32214</v>
+        <v>44085</v>
       </c>
     </row>
     <row r="47">
@@ -1785,16 +1787,16 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>7096</v>
+        <v>10148</v>
       </c>
       <c r="C47" t="n">
-        <v>2428</v>
+        <v>3566</v>
       </c>
       <c r="D47" t="n">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="E47" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F47" t="n">
         <v>7</v>
@@ -1808,7 +1810,7 @@
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="n">
-        <v>9612</v>
+        <v>13809</v>
       </c>
     </row>
     <row r="48">
@@ -1818,13 +1820,13 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>3015</v>
+        <v>3923</v>
       </c>
       <c r="C48" t="n">
-        <v>1066</v>
+        <v>1458</v>
       </c>
       <c r="D48" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="E48" t="n">
         <v>8</v>
@@ -1839,7 +1841,7 @@
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="n">
-        <v>4131</v>
+        <v>5435</v>
       </c>
     </row>
     <row r="49">
@@ -1849,13 +1851,13 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>6193</v>
+        <v>8136</v>
       </c>
       <c r="C49" t="n">
-        <v>1760</v>
+        <v>2482</v>
       </c>
       <c r="D49" t="n">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="E49" t="n">
         <v>16</v>
@@ -1872,7 +1874,7 @@
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="n">
-        <v>8054</v>
+        <v>10730</v>
       </c>
     </row>
     <row r="50">
@@ -1882,13 +1884,13 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>3606</v>
+        <v>4784</v>
       </c>
       <c r="C50" t="n">
-        <v>1096</v>
+        <v>1574</v>
       </c>
       <c r="D50" t="n">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="E50" t="n">
         <v>9</v>
@@ -1905,7 +1907,7 @@
       <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr"/>
       <c r="K50" t="n">
-        <v>4813</v>
+        <v>6485</v>
       </c>
     </row>
     <row r="51">
@@ -1915,13 +1917,13 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>4169</v>
+        <v>5641</v>
       </c>
       <c r="C51" t="n">
-        <v>1387</v>
+        <v>1931</v>
       </c>
       <c r="D51" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="E51" t="n">
         <v>5</v>
@@ -1936,7 +1938,7 @@
       <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr"/>
       <c r="K51" t="n">
-        <v>5604</v>
+        <v>7626</v>
       </c>
     </row>
     <row r="52">
@@ -1946,22 +1948,22 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>882</v>
+        <v>1260</v>
       </c>
       <c r="C52" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="D52" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E52" t="n">
         <v>1</v>
       </c>
       <c r="F52" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H52" t="n">
         <v>0</v>
@@ -1973,7 +1975,7 @@
         <v>0</v>
       </c>
       <c r="K52" t="n">
-        <v>903</v>
+        <v>1288</v>
       </c>
     </row>
     <row r="53">
@@ -1983,28 +1985,28 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>882</v>
+        <v>1260</v>
       </c>
       <c r="C53" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="D53" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E53" t="n">
         <v>1</v>
       </c>
       <c r="F53" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr"/>
       <c r="K53" t="n">
-        <v>903</v>
+        <v>1288</v>
       </c>
     </row>
     <row r="54">
@@ -2014,25 +2016,25 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>51837</v>
+        <v>78138</v>
       </c>
       <c r="C54" t="n">
-        <v>10899</v>
+        <v>14721</v>
       </c>
       <c r="D54" t="n">
-        <v>2247</v>
+        <v>2426</v>
       </c>
       <c r="E54" t="n">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="F54" t="n">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="G54" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H54" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="I54" t="n">
         <v>2</v>
@@ -2041,7 +2043,7 @@
         <v>0</v>
       </c>
       <c r="K54" t="n">
-        <v>65419</v>
+        <v>95728</v>
       </c>
     </row>
   </sheetData>
@@ -2117,16 +2119,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>372</v>
+        <v>678</v>
       </c>
       <c r="C2" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F2" t="n">
         <v>5</v>
@@ -2141,7 +2143,7 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>408</v>
+        <v>712</v>
       </c>
     </row>
     <row r="3">
@@ -2151,13 +2153,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>200</v>
+        <v>1052</v>
       </c>
       <c r="C3" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E3" t="n">
         <v>8</v>
@@ -2175,7 +2177,7 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>219</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="4">
@@ -2185,16 +2187,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7372</v>
+        <v>10251</v>
       </c>
       <c r="C4" t="n">
-        <v>2483</v>
+        <v>3652</v>
       </c>
       <c r="D4" t="n">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="E4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F4" t="n">
         <v>8</v>
@@ -2209,7 +2211,7 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>9944</v>
+        <v>14003</v>
       </c>
     </row>
     <row r="5">
@@ -2219,13 +2221,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>428</v>
+        <v>1443</v>
       </c>
       <c r="C5" t="n">
-        <v>107</v>
+        <v>132</v>
       </c>
       <c r="D5" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E5" t="n">
         <v>3</v>
@@ -2243,7 +2245,7 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>546</v>
+        <v>1588</v>
       </c>
     </row>
     <row r="6">
@@ -2253,13 +2255,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1086</v>
+        <v>1881</v>
       </c>
       <c r="C6" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="D6" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E6" t="n">
         <v>3</v>
@@ -2277,7 +2279,7 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>1140</v>
+        <v>1946</v>
       </c>
     </row>
     <row r="7">
@@ -2287,10 +2289,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>506</v>
+        <v>1040</v>
       </c>
       <c r="C7" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D7" t="n">
         <v>7</v>
@@ -2311,7 +2313,7 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>524</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="8">
@@ -2321,14 +2323,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>244</v>
+        <v>671</v>
       </c>
       <c r="C8" t="n">
+        <v>8</v>
+      </c>
+      <c r="D8" t="n">
         <v>6</v>
       </c>
-      <c r="D8" t="n">
-        <v>5</v>
-      </c>
       <c r="E8" t="n">
         <v>1</v>
       </c>
@@ -2345,7 +2347,7 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>260</v>
+        <v>690</v>
       </c>
     </row>
     <row r="9">
@@ -2355,10 +2357,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>487</v>
+        <v>238</v>
       </c>
       <c r="C9" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D9" t="n">
         <v>2</v>
@@ -2379,7 +2381,7 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>514</v>
+        <v>269</v>
       </c>
     </row>
     <row r="10">
@@ -2389,7 +2391,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>69</v>
+        <v>31</v>
       </c>
       <c r="C10" t="n">
         <v>1</v>
@@ -2413,7 +2415,7 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>71</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11">
@@ -2423,14 +2425,14 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>69</v>
+        <v>261</v>
       </c>
       <c r="C11" t="n">
+        <v>8</v>
+      </c>
+      <c r="D11" t="n">
         <v>6</v>
       </c>
-      <c r="D11" t="n">
-        <v>5</v>
-      </c>
       <c r="E11" t="n">
         <v>2</v>
       </c>
@@ -2447,7 +2449,7 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>82</v>
+        <v>277</v>
       </c>
     </row>
     <row r="12">
@@ -2457,13 +2459,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3192</v>
+        <v>4050</v>
       </c>
       <c r="C12" t="n">
-        <v>1075</v>
+        <v>1472</v>
       </c>
       <c r="D12" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="E12" t="n">
         <v>9</v>
@@ -2481,7 +2483,7 @@
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>4320</v>
+        <v>5579</v>
       </c>
     </row>
     <row r="13">
@@ -2491,7 +2493,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>138</v>
+        <v>57</v>
       </c>
       <c r="C13" t="n">
         <v>4</v>
@@ -2515,7 +2517,7 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>144</v>
+        <v>63</v>
       </c>
     </row>
     <row r="14">
@@ -2525,13 +2527,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>40</v>
+        <v>181</v>
       </c>
       <c r="C14" t="n">
         <v>2</v>
       </c>
       <c r="D14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E14" t="n">
         <v>1</v>
@@ -2549,7 +2551,7 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>52</v>
+        <v>194</v>
       </c>
     </row>
     <row r="15">
@@ -2559,10 +2561,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>62</v>
+        <v>358</v>
       </c>
       <c r="C15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D15" t="n">
         <v>2</v>
@@ -2583,7 +2585,7 @@
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>75</v>
+        <v>372</v>
       </c>
     </row>
     <row r="16">
@@ -2593,13 +2595,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>742</v>
+        <v>1249</v>
       </c>
       <c r="C16" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E16" t="n">
         <v>3</v>
@@ -2617,7 +2619,7 @@
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>765</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="17">
@@ -2627,7 +2629,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>142</v>
+        <v>87</v>
       </c>
       <c r="C17" t="n">
         <v>2</v>
@@ -2651,7 +2653,7 @@
         <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>146</v>
+        <v>91</v>
       </c>
     </row>
     <row r="18">
@@ -2661,13 +2663,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>390</v>
+        <v>182</v>
       </c>
       <c r="C18" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
@@ -2685,7 +2687,7 @@
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>402</v>
+        <v>190</v>
       </c>
     </row>
     <row r="19">
@@ -2695,13 +2697,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>410</v>
+        <v>1866</v>
       </c>
       <c r="C19" t="n">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="D19" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="E19" t="n">
         <v>16</v>
@@ -2719,7 +2721,7 @@
         <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>499</v>
+        <v>1967</v>
       </c>
     </row>
     <row r="20">
@@ -2729,10 +2731,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>813</v>
+        <v>1231</v>
       </c>
       <c r="C20" t="n">
-        <v>41</v>
+        <v>104</v>
       </c>
       <c r="D20" t="n">
         <v>2</v>
@@ -2741,19 +2743,19 @@
         <v>3</v>
       </c>
       <c r="F20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I20" t="n">
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>862</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="21">
@@ -2763,13 +2765,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="C21" t="n">
         <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E21" t="n">
         <v>2</v>
@@ -2787,7 +2789,7 @@
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>26</v>
+        <v>64</v>
       </c>
     </row>
     <row r="22">
@@ -2797,10 +2799,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>512</v>
+        <v>269</v>
       </c>
       <c r="C22" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D22" t="n">
         <v>5</v>
@@ -2821,7 +2823,7 @@
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>535</v>
+        <v>288</v>
       </c>
     </row>
     <row r="23">
@@ -2831,10 +2833,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>804</v>
+        <v>385</v>
       </c>
       <c r="C23" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="D23" t="n">
         <v>3</v>
@@ -2855,7 +2857,7 @@
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>822</v>
+        <v>394</v>
       </c>
     </row>
     <row r="24">
@@ -2865,13 +2867,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>798</v>
+        <v>284</v>
       </c>
       <c r="C24" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D24" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
@@ -2889,7 +2891,7 @@
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>835</v>
+        <v>321</v>
       </c>
     </row>
     <row r="25">
@@ -2899,7 +2901,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>30</v>
+        <v>212</v>
       </c>
       <c r="C25" t="n">
         <v>3</v>
@@ -2923,7 +2925,7 @@
         <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>36</v>
+        <v>218</v>
       </c>
     </row>
     <row r="26">
@@ -2933,31 +2935,31 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>3427</v>
+        <v>6832</v>
       </c>
       <c r="C26" t="n">
-        <v>2247</v>
+        <v>2380</v>
       </c>
       <c r="D26" t="n">
-        <v>1701</v>
+        <v>1781</v>
       </c>
       <c r="E26" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F26" t="n">
         <v>8</v>
       </c>
       <c r="G26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H26" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I26" t="n">
         <v>1</v>
       </c>
       <c r="J26" t="n">
-        <v>7419</v>
+        <v>11039</v>
       </c>
     </row>
     <row r="27">
@@ -2967,16 +2969,16 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>543</v>
+        <v>1472</v>
       </c>
       <c r="C27" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="D27" t="n">
         <v>9</v>
       </c>
       <c r="E27" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F27" t="n">
         <v>3</v>
@@ -2991,7 +2993,7 @@
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>575</v>
+        <v>1518</v>
       </c>
     </row>
     <row r="28">
@@ -3001,22 +3003,22 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1025</v>
+        <v>2139</v>
       </c>
       <c r="C28" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="D28" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E28" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F28" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G28" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H28" t="n">
         <v>0</v>
@@ -3025,7 +3027,7 @@
         <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>1082</v>
+        <v>2205</v>
       </c>
     </row>
     <row r="29">
@@ -3035,13 +3037,13 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>276</v>
+        <v>501</v>
       </c>
       <c r="C29" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="D29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E29" t="n">
         <v>2</v>
@@ -3059,7 +3061,7 @@
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>289</v>
+        <v>521</v>
       </c>
     </row>
     <row r="30">
@@ -3069,10 +3071,10 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="C30" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D30" t="n">
         <v>0</v>
@@ -3093,7 +3095,7 @@
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>27</v>
+        <v>45</v>
       </c>
     </row>
     <row r="31">
@@ -3103,13 +3105,13 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>5790</v>
+        <v>7480</v>
       </c>
       <c r="C31" t="n">
-        <v>1601</v>
+        <v>2274</v>
       </c>
       <c r="D31" t="n">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="E31" t="n">
         <v>17</v>
@@ -3127,7 +3129,7 @@
         <v>0</v>
       </c>
       <c r="J31" t="n">
-        <v>7463</v>
+        <v>9832</v>
       </c>
     </row>
     <row r="32">
@@ -3137,13 +3139,13 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>30</v>
+        <v>85</v>
       </c>
       <c r="C32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D32" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E32" t="n">
         <v>2</v>
@@ -3161,7 +3163,7 @@
         <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>34</v>
+        <v>92</v>
       </c>
     </row>
     <row r="33">
@@ -3171,7 +3173,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>36</v>
+        <v>68</v>
       </c>
       <c r="C33" t="n">
         <v>5</v>
@@ -3195,7 +3197,7 @@
         <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>43</v>
+        <v>75</v>
       </c>
     </row>
     <row r="34">
@@ -3205,10 +3207,10 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>225</v>
+        <v>97</v>
       </c>
       <c r="C34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D34" t="n">
         <v>2</v>
@@ -3229,7 +3231,7 @@
         <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>231</v>
+        <v>102</v>
       </c>
     </row>
     <row r="35">
@@ -3239,10 +3241,10 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>679</v>
+        <v>341</v>
       </c>
       <c r="C35" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D35" t="n">
         <v>1</v>
@@ -3263,7 +3265,7 @@
         <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>694</v>
+        <v>350</v>
       </c>
     </row>
     <row r="36">
@@ -3273,13 +3275,13 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1756</v>
+        <v>2819</v>
       </c>
       <c r="C36" t="n">
-        <v>107</v>
+        <v>257</v>
       </c>
       <c r="D36" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E36" t="n">
         <v>2</v>
@@ -3288,16 +3290,16 @@
         <v>4</v>
       </c>
       <c r="G36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>1873</v>
+        <v>3089</v>
       </c>
     </row>
     <row r="37">
@@ -3307,10 +3309,10 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>397</v>
+        <v>188</v>
       </c>
       <c r="C37" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D37" t="n">
         <v>1</v>
@@ -3331,7 +3333,7 @@
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>403</v>
+        <v>193</v>
       </c>
     </row>
     <row r="38">
@@ -3341,7 +3343,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>175</v>
+        <v>452</v>
       </c>
       <c r="C38" t="n">
         <v>1</v>
@@ -3365,7 +3367,7 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>181</v>
+        <v>458</v>
       </c>
     </row>
     <row r="39">
@@ -3375,10 +3377,10 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>363</v>
+        <v>114</v>
       </c>
       <c r="C39" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D39" t="n">
         <v>2</v>
@@ -3399,7 +3401,7 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>380</v>
+        <v>132</v>
       </c>
     </row>
     <row r="40">
@@ -3409,10 +3411,10 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>259</v>
+        <v>577</v>
       </c>
       <c r="C40" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D40" t="n">
         <v>3</v>
@@ -3433,7 +3435,7 @@
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>269</v>
+        <v>590</v>
       </c>
     </row>
     <row r="41">
@@ -3443,10 +3445,10 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>21</v>
+        <v>214</v>
       </c>
       <c r="C41" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D41" t="n">
         <v>3</v>
@@ -3467,7 +3469,7 @@
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>32</v>
+        <v>227</v>
       </c>
     </row>
     <row r="42">
@@ -3477,10 +3479,10 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>379</v>
+        <v>788</v>
       </c>
       <c r="C42" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D42" t="n">
         <v>1</v>
@@ -3501,7 +3503,7 @@
         <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>389</v>
+        <v>800</v>
       </c>
     </row>
     <row r="43">
@@ -3511,13 +3513,13 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>708</v>
+        <v>1152</v>
       </c>
       <c r="C43" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D43" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E43" t="n">
         <v>2</v>
@@ -3535,7 +3537,7 @@
         <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>723</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="44">
@@ -3545,10 +3547,10 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>738</v>
+        <v>355</v>
       </c>
       <c r="C44" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D44" t="n">
         <v>6</v>
@@ -3569,7 +3571,7 @@
         <v>1</v>
       </c>
       <c r="J44" t="n">
-        <v>775</v>
+        <v>393</v>
       </c>
     </row>
     <row r="45">
@@ -3579,10 +3581,10 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>20</v>
+        <v>145</v>
       </c>
       <c r="C45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D45" t="n">
         <v>1</v>
@@ -3603,7 +3605,7 @@
         <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>25</v>
+        <v>151</v>
       </c>
     </row>
     <row r="46">
@@ -3613,13 +3615,13 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>223</v>
+        <v>556</v>
       </c>
       <c r="C46" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D46" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E46" t="n">
         <v>5</v>
@@ -3637,7 +3639,7 @@
         <v>0</v>
       </c>
       <c r="J46" t="n">
-        <v>245</v>
+        <v>580</v>
       </c>
     </row>
     <row r="47">
@@ -3647,13 +3649,13 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>54</v>
+        <v>129</v>
       </c>
       <c r="C47" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D47" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E47" t="n">
         <v>2</v>
@@ -3671,7 +3673,7 @@
         <v>0</v>
       </c>
       <c r="J47" t="n">
-        <v>63</v>
+        <v>141</v>
       </c>
     </row>
     <row r="48">
@@ -3681,13 +3683,13 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>2106</v>
+        <v>3394</v>
       </c>
       <c r="C48" t="n">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="D48" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E48" t="n">
         <v>7</v>
@@ -3705,7 +3707,7 @@
         <v>0</v>
       </c>
       <c r="J48" t="n">
-        <v>2166</v>
+        <v>3473</v>
       </c>
     </row>
     <row r="49">
@@ -3715,10 +3717,10 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>541</v>
+        <v>265</v>
       </c>
       <c r="C49" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="D49" t="n">
         <v>2</v>
@@ -3739,7 +3741,7 @@
         <v>0</v>
       </c>
       <c r="J49" t="n">
-        <v>562</v>
+        <v>276</v>
       </c>
     </row>
     <row r="50">
@@ -3749,10 +3751,10 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>265</v>
+        <v>197</v>
       </c>
       <c r="C50" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D50" t="n">
         <v>3</v>
@@ -3773,7 +3775,7 @@
         <v>0</v>
       </c>
       <c r="J50" t="n">
-        <v>279</v>
+        <v>214</v>
       </c>
     </row>
     <row r="51">
@@ -3783,10 +3785,10 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>473</v>
+        <v>1079</v>
       </c>
       <c r="C51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D51" t="n">
         <v>1</v>
@@ -3807,7 +3809,7 @@
         <v>0</v>
       </c>
       <c r="J51" t="n">
-        <v>477</v>
+        <v>1084</v>
       </c>
     </row>
     <row r="52">
@@ -3817,13 +3819,13 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>4393</v>
+        <v>5687</v>
       </c>
       <c r="C52" t="n">
-        <v>1241</v>
+        <v>1786</v>
       </c>
       <c r="D52" t="n">
-        <v>124</v>
+        <v>146</v>
       </c>
       <c r="E52" t="n">
         <v>10</v>
@@ -3841,7 +3843,7 @@
         <v>0</v>
       </c>
       <c r="J52" t="n">
-        <v>5777</v>
+        <v>7638</v>
       </c>
     </row>
     <row r="53">
@@ -3851,13 +3853,13 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>168</v>
+        <v>480</v>
       </c>
       <c r="C53" t="n">
         <v>6</v>
       </c>
       <c r="D53" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E53" t="n">
         <v>0</v>
@@ -3875,7 +3877,7 @@
         <v>0</v>
       </c>
       <c r="J53" t="n">
-        <v>182</v>
+        <v>496</v>
       </c>
     </row>
     <row r="54">
@@ -3885,7 +3887,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>177</v>
+        <v>77</v>
       </c>
       <c r="C54" t="n">
         <v>5</v>
@@ -3909,7 +3911,7 @@
         <v>0</v>
       </c>
       <c r="J54" t="n">
-        <v>182</v>
+        <v>82</v>
       </c>
     </row>
     <row r="55">
@@ -3919,13 +3921,13 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>4040</v>
+        <v>5294</v>
       </c>
       <c r="C55" t="n">
-        <v>1332</v>
+        <v>1838</v>
       </c>
       <c r="D55" t="n">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="E55" t="n">
         <v>5</v>
@@ -3943,7 +3945,7 @@
         <v>0</v>
       </c>
       <c r="J55" t="n">
-        <v>5421</v>
+        <v>7193</v>
       </c>
     </row>
     <row r="56">
@@ -3953,10 +3955,10 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>31</v>
+        <v>191</v>
       </c>
       <c r="C56" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D56" t="n">
         <v>1</v>
@@ -3977,7 +3979,7 @@
         <v>0</v>
       </c>
       <c r="J56" t="n">
-        <v>48</v>
+        <v>212</v>
       </c>
     </row>
     <row r="57">
@@ -3987,10 +3989,10 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>347</v>
+        <v>136</v>
       </c>
       <c r="C57" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D57" t="n">
         <v>3</v>
@@ -4011,7 +4013,7 @@
         <v>0</v>
       </c>
       <c r="J57" t="n">
-        <v>370</v>
+        <v>160</v>
       </c>
     </row>
     <row r="58">
@@ -4021,7 +4023,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>23</v>
+        <v>55</v>
       </c>
       <c r="C58" t="n">
         <v>2</v>
@@ -4030,7 +4032,7 @@
         <v>3</v>
       </c>
       <c r="E58" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F58" t="n">
         <v>0</v>
@@ -4045,7 +4047,7 @@
         <v>0</v>
       </c>
       <c r="J58" t="n">
-        <v>30</v>
+        <v>63</v>
       </c>
     </row>
     <row r="59">
@@ -4055,10 +4057,10 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>28</v>
+        <v>58</v>
       </c>
       <c r="C59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D59" t="n">
         <v>0</v>
@@ -4079,7 +4081,7 @@
         <v>0</v>
       </c>
       <c r="J59" t="n">
-        <v>32</v>
+        <v>63</v>
       </c>
     </row>
     <row r="60">
@@ -4089,13 +4091,13 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>557</v>
+        <v>1170</v>
       </c>
       <c r="C60" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D60" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E60" t="n">
         <v>6</v>
@@ -4113,7 +4115,7 @@
         <v>0</v>
       </c>
       <c r="J60" t="n">
-        <v>571</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="61">
@@ -4123,16 +4125,16 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>547</v>
+        <v>1259</v>
       </c>
       <c r="C61" t="n">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D61" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E61" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F61" t="n">
         <v>1</v>
@@ -4147,7 +4149,7 @@
         <v>0</v>
       </c>
       <c r="J61" t="n">
-        <v>587</v>
+        <v>1322</v>
       </c>
     </row>
     <row r="62">
@@ -4157,13 +4159,13 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>496</v>
+        <v>858</v>
       </c>
       <c r="C62" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D62" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E62" t="n">
         <v>0</v>
@@ -4181,7 +4183,7 @@
         <v>0</v>
       </c>
       <c r="J62" t="n">
-        <v>516</v>
+        <v>891</v>
       </c>
     </row>
     <row r="63">
@@ -4191,13 +4193,13 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>893</v>
+        <v>2336</v>
       </c>
       <c r="C63" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D63" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E63" t="n">
         <v>8</v>
@@ -4215,7 +4217,7 @@
         <v>0</v>
       </c>
       <c r="J63" t="n">
-        <v>937</v>
+        <v>2385</v>
       </c>
     </row>
     <row r="64">
@@ -4225,13 +4227,13 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>681</v>
+        <v>1049</v>
       </c>
       <c r="C64" t="n">
-        <v>137</v>
+        <v>188</v>
       </c>
       <c r="D64" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="E64" t="n">
         <v>2</v>
@@ -4249,7 +4251,7 @@
         <v>0</v>
       </c>
       <c r="J64" t="n">
-        <v>840</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="65">
@@ -4259,31 +4261,31 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>51837</v>
+        <v>78138</v>
       </c>
       <c r="C65" t="n">
-        <v>10899</v>
+        <v>14721</v>
       </c>
       <c r="D65" t="n">
-        <v>2247</v>
+        <v>2426</v>
       </c>
       <c r="E65" t="n">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="F65" t="n">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="G65" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H65" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="I65" t="n">
         <v>2</v>
       </c>
       <c r="J65" t="n">
-        <v>65419</v>
+        <v>95728</v>
       </c>
     </row>
   </sheetData>
@@ -4359,16 +4361,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>7096</v>
+        <v>10148</v>
       </c>
       <c r="C2" t="n">
-        <v>2428</v>
+        <v>3566</v>
       </c>
       <c r="D2" t="n">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="E2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F2" t="n">
         <v>7</v>
@@ -4383,7 +4385,7 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>9612</v>
+        <v>13809</v>
       </c>
     </row>
     <row r="3">
@@ -4393,13 +4395,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3015</v>
+        <v>3923</v>
       </c>
       <c r="C3" t="n">
-        <v>1066</v>
+        <v>1458</v>
       </c>
       <c r="D3" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="E3" t="n">
         <v>8</v>
@@ -4417,7 +4419,7 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>4131</v>
+        <v>5435</v>
       </c>
     </row>
     <row r="4">
@@ -4427,31 +4429,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2860</v>
+        <v>3300</v>
       </c>
       <c r="C4" t="n">
-        <v>2169</v>
+        <v>2289</v>
       </c>
       <c r="D4" t="n">
-        <v>1768</v>
+        <v>1852</v>
       </c>
       <c r="E4" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F4" t="n">
         <v>3</v>
       </c>
       <c r="G4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H4" t="n">
         <v>4</v>
       </c>
-      <c r="H4" t="n">
-        <v>3</v>
-      </c>
       <c r="I4" t="n">
         <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>6831</v>
+        <v>7478</v>
       </c>
     </row>
     <row r="5">
@@ -4461,7 +4463,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>134</v>
+        <v>349</v>
       </c>
       <c r="C5" t="n">
         <v>25</v>
@@ -4485,7 +4487,7 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>167</v>
+        <v>382</v>
       </c>
     </row>
     <row r="6">
@@ -4495,13 +4497,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2088</v>
+        <v>3364</v>
       </c>
       <c r="C6" t="n">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="D6" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E6" t="n">
         <v>7</v>
@@ -4519,7 +4521,7 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>2141</v>
+        <v>3434</v>
       </c>
     </row>
     <row r="7">
@@ -4529,13 +4531,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>111</v>
+        <v>787</v>
       </c>
       <c r="C7" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>
@@ -4553,7 +4555,7 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>139</v>
+        <v>806</v>
       </c>
     </row>
     <row r="8">
@@ -4563,13 +4565,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1099</v>
+        <v>1894</v>
       </c>
       <c r="C8" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="D8" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E8" t="n">
         <v>3</v>
@@ -4587,7 +4589,7 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>1154</v>
+        <v>1960</v>
       </c>
     </row>
     <row r="9">
@@ -4597,13 +4599,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>691</v>
+        <v>1128</v>
       </c>
       <c r="C9" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E9" t="n">
         <v>2</v>
@@ -4621,7 +4623,7 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>706</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="10">
@@ -4631,13 +4633,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>490</v>
+        <v>845</v>
       </c>
       <c r="C10" t="n">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="D10" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -4655,7 +4657,7 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>509</v>
+        <v>877</v>
       </c>
     </row>
     <row r="11">
@@ -4665,13 +4667,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>990</v>
+        <v>3114</v>
       </c>
       <c r="C11" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D11" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="E11" t="n">
         <v>16</v>
@@ -4689,7 +4691,7 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>1050</v>
+        <v>3178</v>
       </c>
     </row>
     <row r="12">
@@ -4699,13 +4701,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C12" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
@@ -4723,7 +4725,7 @@
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>89</v>
+        <v>94</v>
       </c>
     </row>
     <row r="13">
@@ -4733,10 +4735,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="C13" t="n">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
@@ -4757,7 +4759,7 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>135</v>
+        <v>148</v>
       </c>
     </row>
     <row r="14">
@@ -4767,7 +4769,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="C14" t="n">
         <v>2</v>
@@ -4791,7 +4793,7 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>18</v>
+        <v>33</v>
       </c>
     </row>
     <row r="15">
@@ -4801,13 +4803,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="C15" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E15" t="n">
         <v>1</v>
@@ -4825,7 +4827,7 @@
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>115</v>
+        <v>131</v>
       </c>
     </row>
     <row r="16">
@@ -4835,10 +4837,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C16" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
@@ -4859,7 +4861,7 @@
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>99</v>
+        <v>111</v>
       </c>
     </row>
     <row r="17">
@@ -4869,10 +4871,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C17" t="n">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
@@ -4893,7 +4895,7 @@
         <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>128</v>
+        <v>146</v>
       </c>
     </row>
     <row r="18">
@@ -4903,10 +4905,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C18" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
@@ -4927,7 +4929,7 @@
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
     <row r="19">
@@ -4940,10 +4942,10 @@
         <v>80</v>
       </c>
       <c r="C19" t="n">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="D19" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
@@ -4961,7 +4963,7 @@
         <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>118</v>
+        <v>132</v>
       </c>
     </row>
     <row r="20">
@@ -4971,10 +4973,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="C20" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
@@ -4995,7 +4997,7 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
     </row>
     <row r="21">
@@ -5005,10 +5007,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="C21" t="n">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
@@ -5029,7 +5031,7 @@
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>161</v>
+        <v>180</v>
       </c>
     </row>
     <row r="22">
@@ -5039,10 +5041,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C22" t="n">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
@@ -5063,7 +5065,7 @@
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>115</v>
+        <v>127</v>
       </c>
     </row>
     <row r="23">
@@ -5073,10 +5075,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>170</v>
+        <v>187</v>
       </c>
       <c r="C23" t="n">
-        <v>44</v>
+        <v>71</v>
       </c>
       <c r="D23" t="n">
         <v>2</v>
@@ -5097,7 +5099,7 @@
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>217</v>
+        <v>261</v>
       </c>
     </row>
     <row r="24">
@@ -5107,13 +5109,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>260</v>
+        <v>136</v>
       </c>
       <c r="C24" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D24" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E24" t="n">
         <v>1</v>
@@ -5122,16 +5124,16 @@
         <v>5</v>
       </c>
       <c r="G24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I24" t="n">
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>282</v>
+        <v>157</v>
       </c>
     </row>
     <row r="25">
@@ -5141,10 +5143,10 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C25" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
@@ -5165,7 +5167,7 @@
         <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>73</v>
+        <v>78</v>
       </c>
     </row>
     <row r="26">
@@ -5175,31 +5177,31 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2563</v>
+        <v>4044</v>
       </c>
       <c r="C26" t="n">
-        <v>147</v>
+        <v>360</v>
       </c>
       <c r="D26" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E26" t="n">
         <v>5</v>
       </c>
       <c r="F26" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I26" t="n">
         <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>2726</v>
+        <v>4422</v>
       </c>
     </row>
     <row r="27">
@@ -5209,13 +5211,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>775</v>
+        <v>1644</v>
       </c>
       <c r="C27" t="n">
+        <v>13</v>
+      </c>
+      <c r="D27" t="n">
         <v>5</v>
-      </c>
-      <c r="D27" t="n">
-        <v>4</v>
       </c>
       <c r="E27" t="n">
         <v>6</v>
@@ -5233,7 +5235,7 @@
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>797</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="28">
@@ -5243,16 +5245,16 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1414</v>
+        <v>2984</v>
       </c>
       <c r="C28" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D28" t="n">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="E28" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F28" t="n">
         <v>19</v>
@@ -5267,7 +5269,7 @@
         <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>1548</v>
+        <v>3129</v>
       </c>
     </row>
     <row r="29">
@@ -5277,10 +5279,10 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>300</v>
+        <v>474</v>
       </c>
       <c r="C29" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D29" t="n">
         <v>10</v>
@@ -5301,7 +5303,7 @@
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>340</v>
+        <v>517</v>
       </c>
     </row>
     <row r="30">
@@ -5311,13 +5313,13 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1014</v>
+        <v>1760</v>
       </c>
       <c r="C30" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="D30" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E30" t="n">
         <v>5</v>
@@ -5335,7 +5337,7 @@
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>1042</v>
+        <v>1804</v>
       </c>
     </row>
     <row r="31">
@@ -5345,16 +5347,16 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>329</v>
+        <v>2799</v>
       </c>
       <c r="C31" t="n">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="D31" t="n">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="E31" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F31" t="n">
         <v>0</v>
@@ -5369,7 +5371,7 @@
         <v>1</v>
       </c>
       <c r="J31" t="n">
-        <v>396</v>
+        <v>2884</v>
       </c>
     </row>
     <row r="32">
@@ -5379,10 +5381,10 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>7601</v>
+        <v>3557</v>
       </c>
       <c r="C32" t="n">
-        <v>100</v>
+        <v>69</v>
       </c>
       <c r="D32" t="n">
         <v>13</v>
@@ -5403,7 +5405,7 @@
         <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>7737</v>
+        <v>3662</v>
       </c>
     </row>
     <row r="33">
@@ -5413,22 +5415,22 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>458</v>
+        <v>4386</v>
       </c>
       <c r="C33" t="n">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="D33" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E33" t="n">
         <v>10</v>
       </c>
       <c r="F33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H33" t="n">
         <v>1</v>
@@ -5437,7 +5439,7 @@
         <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>597</v>
+        <v>4530</v>
       </c>
     </row>
     <row r="34">
@@ -5447,16 +5449,16 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>700</v>
+        <v>1902</v>
       </c>
       <c r="C34" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="D34" t="n">
         <v>8</v>
       </c>
       <c r="E34" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F34" t="n">
         <v>4</v>
@@ -5471,7 +5473,7 @@
         <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>733</v>
+        <v>1949</v>
       </c>
     </row>
     <row r="35">
@@ -5481,10 +5483,10 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>20</v>
+        <v>341</v>
       </c>
       <c r="C35" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D35" t="n">
         <v>3</v>
@@ -5505,7 +5507,7 @@
         <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>36</v>
+        <v>360</v>
       </c>
     </row>
     <row r="36">
@@ -5515,13 +5517,13 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1329</v>
+        <v>3013</v>
       </c>
       <c r="C36" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="D36" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E36" t="n">
         <v>11</v>
@@ -5539,7 +5541,7 @@
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>1352</v>
+        <v>3044</v>
       </c>
     </row>
     <row r="37">
@@ -5549,16 +5551,16 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>592</v>
+        <v>1321</v>
       </c>
       <c r="C37" t="n">
-        <v>13</v>
+        <v>36</v>
       </c>
       <c r="D37" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E37" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F37" t="n">
         <v>1</v>
@@ -5573,7 +5575,7 @@
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>620</v>
+        <v>1372</v>
       </c>
     </row>
     <row r="38">
@@ -5583,13 +5585,13 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>6193</v>
+        <v>8136</v>
       </c>
       <c r="C38" t="n">
-        <v>1760</v>
+        <v>2482</v>
       </c>
       <c r="D38" t="n">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="E38" t="n">
         <v>16</v>
@@ -5607,7 +5609,7 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>8054</v>
+        <v>10730</v>
       </c>
     </row>
     <row r="39">
@@ -5617,22 +5619,22 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>882</v>
+        <v>1260</v>
       </c>
       <c r="C39" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="D39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E39" t="n">
         <v>1</v>
       </c>
       <c r="F39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H39" t="n">
         <v>0</v>
@@ -5641,7 +5643,7 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>903</v>
+        <v>1288</v>
       </c>
     </row>
     <row r="40">
@@ -5651,13 +5653,13 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>3606</v>
+        <v>4784</v>
       </c>
       <c r="C40" t="n">
-        <v>1096</v>
+        <v>1574</v>
       </c>
       <c r="D40" t="n">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="E40" t="n">
         <v>9</v>
@@ -5675,7 +5677,7 @@
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>4813</v>
+        <v>6485</v>
       </c>
     </row>
     <row r="41">
@@ -5685,13 +5687,13 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>4169</v>
+        <v>5641</v>
       </c>
       <c r="C41" t="n">
-        <v>1387</v>
+        <v>1931</v>
       </c>
       <c r="D41" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="E41" t="n">
         <v>5</v>
@@ -5709,7 +5711,7 @@
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>5604</v>
+        <v>7626</v>
       </c>
     </row>
     <row r="42">
@@ -5719,31 +5721,31 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>51837</v>
+        <v>78138</v>
       </c>
       <c r="C42" t="n">
-        <v>10899</v>
+        <v>14721</v>
       </c>
       <c r="D42" t="n">
-        <v>2247</v>
+        <v>2426</v>
       </c>
       <c r="E42" t="n">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="F42" t="n">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="G42" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H42" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="I42" t="n">
         <v>2</v>
       </c>
       <c r="J42" t="n">
-        <v>65419</v>
+        <v>95728</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Cập nhật dữ liệu tồn kho 05/06/2026 04:17
</commit_message>
<xml_diff>
--- a/BaoCao_TonKho.xlsx
+++ b/BaoCao_TonKho.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>05/06/2026 02:51:45</t>
+          <t>05/06/2026 04:17:50</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -579,19 +579,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>8497</v>
+        <v>8043</v>
       </c>
       <c r="C7" t="n">
-        <v>190</v>
+        <v>623</v>
       </c>
       <c r="D7" t="n">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="E7" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F7" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G7" t="n">
         <v>4</v>
@@ -606,7 +606,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>8816</v>
+        <v>8788</v>
       </c>
     </row>
     <row r="8">
@@ -616,19 +616,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>634</v>
+        <v>821</v>
       </c>
       <c r="C8" t="n">
-        <v>11</v>
+        <v>45</v>
       </c>
       <c r="D8" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E8" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
@@ -637,7 +637,7 @@
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="n">
-        <v>663</v>
+        <v>886</v>
       </c>
     </row>
     <row r="9">
@@ -647,13 +647,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1064</v>
+        <v>1343</v>
       </c>
       <c r="C9" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D9" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E9" t="n">
         <v>3</v>
@@ -668,7 +668,7 @@
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="n">
-        <v>1088</v>
+        <v>1373</v>
       </c>
     </row>
     <row r="10">
@@ -678,16 +678,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2252</v>
+        <v>461</v>
       </c>
       <c r="C10" t="n">
-        <v>72</v>
+        <v>35</v>
       </c>
       <c r="D10" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="E10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
@@ -695,7 +695,7 @@
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="n">
-        <v>2357</v>
+        <v>506</v>
       </c>
     </row>
     <row r="11">
@@ -705,16 +705,16 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1284</v>
+        <v>1166</v>
       </c>
       <c r="C11" t="n">
-        <v>22</v>
+        <v>261</v>
       </c>
       <c r="D11" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F11" t="n">
         <v>1</v>
@@ -724,7 +724,7 @@
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="n">
-        <v>1313</v>
+        <v>1438</v>
       </c>
     </row>
     <row r="12">
@@ -734,13 +734,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>934</v>
+        <v>822</v>
       </c>
       <c r="C12" t="n">
-        <v>38</v>
+        <v>221</v>
       </c>
       <c r="D12" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="n">
@@ -751,7 +751,7 @@
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="n">
-        <v>981</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="13">
@@ -761,19 +761,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2329</v>
+        <v>3430</v>
       </c>
       <c r="C13" t="n">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="D13" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E13" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F13" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G13" t="n">
         <v>2</v>
@@ -784,7 +784,7 @@
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="n">
-        <v>2414</v>
+        <v>3529</v>
       </c>
     </row>
     <row r="14">
@@ -794,10 +794,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>877</v>
+        <v>478</v>
       </c>
       <c r="C14" t="n">
-        <v>679</v>
+        <v>445</v>
       </c>
       <c r="D14" t="n">
         <v>41</v>
@@ -806,7 +806,7 @@
         <v>5</v>
       </c>
       <c r="F14" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G14" t="n">
         <v>1</v>
@@ -821,7 +821,7 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>1616</v>
+        <v>984</v>
       </c>
     </row>
     <row r="15">
@@ -831,13 +831,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="C15" t="n">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="D15" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
@@ -846,7 +846,7 @@
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="n">
-        <v>97</v>
+        <v>105</v>
       </c>
     </row>
     <row r="16">
@@ -856,22 +856,24 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>76</v>
+        <v>14</v>
       </c>
       <c r="C16" t="n">
-        <v>76</v>
-      </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" t="inlineStr"/>
+        <v>61</v>
+      </c>
+      <c r="D16" t="n">
+        <v>4</v>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="n">
-        <v>153</v>
+        <v>80</v>
       </c>
     </row>
     <row r="17">
@@ -881,12 +883,14 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="C17" t="n">
-        <v>3</v>
-      </c>
-      <c r="D17" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="n">
         <v>1</v>
@@ -896,7 +900,7 @@
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="n">
-        <v>21</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18">
@@ -906,13 +910,11 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>52</v>
-      </c>
-      <c r="C18" t="n">
-        <v>74</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="C18" t="inlineStr"/>
       <c r="D18" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E18" t="n">
         <v>1</v>
@@ -923,7 +925,7 @@
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="n">
-        <v>136</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19">
@@ -933,11 +935,9 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>57</v>
-      </c>
-      <c r="C19" t="n">
-        <v>57</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="n">
         <v>1</v>
@@ -952,7 +952,7 @@
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="n">
-        <v>117</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20">
@@ -962,10 +962,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>88</v>
+        <v>9</v>
       </c>
       <c r="C20" t="n">
-        <v>65</v>
+        <v>4</v>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
@@ -977,7 +977,7 @@
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="n">
-        <v>154</v>
+        <v>14</v>
       </c>
     </row>
     <row r="21">
@@ -987,13 +987,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C21" t="n">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="D21" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E21" t="n">
         <v>1</v>
@@ -1006,7 +1006,7 @@
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
     </row>
     <row r="22">
@@ -1016,15 +1016,15 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>58</v>
+        <v>1</v>
       </c>
       <c r="C22" t="n">
-        <v>66</v>
-      </c>
-      <c r="D22" t="n">
-        <v>15</v>
-      </c>
-      <c r="E22" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="n">
+        <v>1</v>
+      </c>
       <c r="F22" t="n">
         <v>1</v>
       </c>
@@ -1033,7 +1033,7 @@
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="n">
-        <v>140</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23">
@@ -1043,10 +1043,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="C23" t="n">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="D23" t="n">
         <v>1</v>
@@ -1060,7 +1060,7 @@
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="n">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="24">
@@ -1070,10 +1070,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>113</v>
+        <v>16</v>
       </c>
       <c r="C24" t="n">
-        <v>79</v>
+        <v>17</v>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr"/>
@@ -1083,7 +1083,7 @@
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="n">
-        <v>192</v>
+        <v>33</v>
       </c>
     </row>
     <row r="25">
@@ -1093,12 +1093,14 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>76</v>
+        <v>45</v>
       </c>
       <c r="C25" t="n">
-        <v>58</v>
-      </c>
-      <c r="D25" t="inlineStr"/>
+        <v>93</v>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
@@ -1106,7 +1108,7 @@
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="n">
-        <v>134</v>
+        <v>139</v>
       </c>
     </row>
     <row r="26">
@@ -1116,13 +1118,13 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="C26" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D26" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="n">
@@ -1133,7 +1135,7 @@
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="n">
-        <v>34</v>
+        <v>47</v>
       </c>
     </row>
     <row r="27">
@@ -1143,13 +1145,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>139</v>
+        <v>199</v>
       </c>
       <c r="C27" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="D27" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="n">
@@ -1162,7 +1164,7 @@
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="n">
-        <v>191</v>
+        <v>256</v>
       </c>
     </row>
     <row r="28">
@@ -1175,7 +1177,7 @@
         <v>53</v>
       </c>
       <c r="C28" t="n">
-        <v>37</v>
+        <v>60</v>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr"/>
@@ -1187,7 +1189,7 @@
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="n">
-        <v>91</v>
+        <v>114</v>
       </c>
     </row>
     <row r="29">
@@ -1197,19 +1199,19 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>669</v>
+        <v>753</v>
       </c>
       <c r="C29" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="D29" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="E29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G29" t="n">
         <v>0</v>
@@ -1224,7 +1226,7 @@
         <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>705</v>
+        <v>801</v>
       </c>
     </row>
     <row r="30">
@@ -1234,19 +1236,17 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>669</v>
+        <v>753</v>
       </c>
       <c r="C30" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="D30" t="n">
-        <v>11</v>
-      </c>
-      <c r="E30" t="n">
-        <v>1</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="E30" t="inlineStr"/>
       <c r="F30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
@@ -1255,7 +1255,7 @@
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="n">
-        <v>705</v>
+        <v>801</v>
       </c>
     </row>
     <row r="31">
@@ -1265,25 +1265,25 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>26814</v>
+        <v>27391</v>
       </c>
       <c r="C31" t="n">
-        <v>910</v>
+        <v>2950</v>
       </c>
       <c r="D31" t="n">
-        <v>161</v>
+        <v>200</v>
       </c>
       <c r="E31" t="n">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F31" t="n">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="G31" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H31" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I31" t="n">
         <v>1</v>
@@ -1292,7 +1292,7 @@
         <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>28081</v>
+        <v>30743</v>
       </c>
     </row>
     <row r="32">
@@ -1302,13 +1302,13 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1309</v>
+        <v>1081</v>
       </c>
       <c r="C32" t="n">
-        <v>53</v>
+        <v>549</v>
       </c>
       <c r="D32" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E32" t="n">
         <v>5</v>
@@ -1325,7 +1325,7 @@
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="n">
-        <v>1383</v>
+        <v>1657</v>
       </c>
     </row>
     <row r="33">
@@ -1335,16 +1335,16 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>2021</v>
+        <v>2249</v>
       </c>
       <c r="C33" t="n">
-        <v>37</v>
+        <v>123</v>
       </c>
       <c r="D33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E33" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F33" t="n">
         <v>1</v>
@@ -1358,7 +1358,7 @@
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="n">
-        <v>2070</v>
+        <v>2384</v>
       </c>
     </row>
     <row r="34">
@@ -1368,30 +1368,30 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>6327</v>
+        <v>4031</v>
       </c>
       <c r="C34" t="n">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="D34" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E34" t="n">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="F34" t="n">
         <v>19</v>
       </c>
       <c r="G34" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="n">
-        <v>6485</v>
+        <v>4215</v>
       </c>
     </row>
     <row r="35">
@@ -1401,19 +1401,19 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>600</v>
+        <v>542</v>
       </c>
       <c r="C35" t="n">
-        <v>41</v>
+        <v>146</v>
       </c>
       <c r="D35" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F35" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G35" t="n">
         <v>2</v>
@@ -1424,7 +1424,7 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="n">
-        <v>674</v>
+        <v>723</v>
       </c>
     </row>
     <row r="36">
@@ -1434,26 +1434,26 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>546</v>
+        <v>725</v>
       </c>
       <c r="C36" t="n">
+        <v>37</v>
+      </c>
+      <c r="D36" t="n">
         <v>7</v>
       </c>
-      <c r="D36" t="n">
-        <v>5</v>
-      </c>
       <c r="E36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="n">
-        <v>564</v>
+        <v>775</v>
       </c>
     </row>
     <row r="37">
@@ -1463,16 +1463,16 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>3763</v>
+        <v>3963</v>
       </c>
       <c r="C37" t="n">
-        <v>66</v>
+        <v>126</v>
       </c>
       <c r="D37" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="E37" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="n">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="n">
-        <v>3882</v>
+        <v>4147</v>
       </c>
     </row>
     <row r="38">
@@ -1494,16 +1494,16 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>3934</v>
+        <v>3648</v>
       </c>
       <c r="C38" t="n">
-        <v>469</v>
+        <v>1344</v>
       </c>
       <c r="D38" t="n">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="E38" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F38" t="n">
         <v>7</v>
@@ -1515,7 +1515,7 @@
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="n">
-        <v>4444</v>
+        <v>5050</v>
       </c>
     </row>
     <row r="39">
@@ -1525,30 +1525,28 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>2516</v>
+        <v>4486</v>
       </c>
       <c r="C39" t="n">
-        <v>17</v>
+        <v>68</v>
       </c>
       <c r="D39" t="n">
+        <v>14</v>
+      </c>
+      <c r="E39" t="n">
         <v>12</v>
-      </c>
-      <c r="E39" t="n">
-        <v>11</v>
       </c>
       <c r="F39" t="n">
         <v>3</v>
       </c>
-      <c r="G39" t="n">
-        <v>1</v>
-      </c>
+      <c r="G39" t="inlineStr"/>
       <c r="H39" t="n">
         <v>2</v>
       </c>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="n">
-        <v>2562</v>
+        <v>4585</v>
       </c>
     </row>
     <row r="40">
@@ -1558,13 +1556,13 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>2380</v>
+        <v>2521</v>
       </c>
       <c r="C40" t="n">
-        <v>63</v>
+        <v>248</v>
       </c>
       <c r="D40" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E40" t="n">
         <v>8</v>
@@ -1579,7 +1577,7 @@
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="n">
-        <v>2464</v>
+        <v>2792</v>
       </c>
     </row>
     <row r="41">
@@ -1589,13 +1587,13 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>570</v>
+        <v>671</v>
       </c>
       <c r="C41" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="D41" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E41" t="n">
         <v>5</v>
@@ -1610,7 +1608,7 @@
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="n">
-        <v>588</v>
+        <v>696</v>
       </c>
     </row>
     <row r="42">
@@ -1620,26 +1618,26 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1228</v>
+        <v>1763</v>
       </c>
       <c r="C42" t="n">
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="D42" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E42" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="n">
-        <v>1260</v>
+        <v>1814</v>
       </c>
     </row>
     <row r="43">
@@ -1649,19 +1647,19 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>1620</v>
+        <v>1711</v>
       </c>
       <c r="C43" t="n">
-        <v>71</v>
+        <v>179</v>
       </c>
       <c r="D43" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E43" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F43" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G43" t="n">
         <v>1</v>
@@ -1670,7 +1668,7 @@
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="n">
-        <v>1705</v>
+        <v>1905</v>
       </c>
     </row>
     <row r="44">
@@ -1680,19 +1678,19 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>1425</v>
+        <v>2144</v>
       </c>
       <c r="C44" t="n">
-        <v>219</v>
+        <v>268</v>
       </c>
       <c r="D44" t="n">
-        <v>115</v>
+        <v>162</v>
       </c>
       <c r="E44" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F44" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G44" t="n">
         <v>3</v>
@@ -1707,7 +1705,7 @@
         <v>0</v>
       </c>
       <c r="K44" t="n">
-        <v>1786</v>
+        <v>2598</v>
       </c>
     </row>
     <row r="45">
@@ -1717,19 +1715,19 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>1425</v>
+        <v>2144</v>
       </c>
       <c r="C45" t="n">
-        <v>219</v>
+        <v>268</v>
       </c>
       <c r="D45" t="n">
-        <v>115</v>
+        <v>162</v>
       </c>
       <c r="E45" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F45" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G45" t="n">
         <v>3</v>
@@ -1742,7 +1740,7 @@
       </c>
       <c r="J45" t="inlineStr"/>
       <c r="K45" t="n">
-        <v>1786</v>
+        <v>2598</v>
       </c>
     </row>
     <row r="46">
@@ -1752,22 +1750,22 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>33891</v>
+        <v>20750</v>
       </c>
       <c r="C46" t="n">
-        <v>15211</v>
+        <v>16325</v>
       </c>
       <c r="D46" t="n">
-        <v>414</v>
+        <v>1012</v>
       </c>
       <c r="E46" t="n">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="F46" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="G46" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H46" t="n">
         <v>7</v>
@@ -1779,7 +1777,7 @@
         <v>0</v>
       </c>
       <c r="K46" t="n">
-        <v>49618</v>
+        <v>38181</v>
       </c>
     </row>
     <row r="47">
@@ -1789,16 +1787,16 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>10877</v>
+        <v>8310</v>
       </c>
       <c r="C47" t="n">
-        <v>4956</v>
+        <v>7027</v>
       </c>
       <c r="D47" t="n">
-        <v>101</v>
+        <v>306</v>
       </c>
       <c r="E47" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F47" t="n">
         <v>8</v>
@@ -1812,7 +1810,7 @@
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="n">
-        <v>15957</v>
+        <v>15663</v>
       </c>
     </row>
     <row r="48">
@@ -1822,19 +1820,19 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>4092</v>
+        <v>978</v>
       </c>
       <c r="C48" t="n">
-        <v>1982</v>
+        <v>366</v>
       </c>
       <c r="D48" t="n">
-        <v>39</v>
+        <v>76</v>
       </c>
       <c r="E48" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F48" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G48" t="n">
         <v>2</v>
@@ -1845,7 +1843,7 @@
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="n">
-        <v>6136</v>
+        <v>1441</v>
       </c>
     </row>
     <row r="49">
@@ -1855,19 +1853,19 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>8217</v>
+        <v>6081</v>
       </c>
       <c r="C49" t="n">
-        <v>3320</v>
+        <v>4706</v>
       </c>
       <c r="D49" t="n">
-        <v>91</v>
+        <v>225</v>
       </c>
       <c r="E49" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F49" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G49" t="n">
         <v>5</v>
@@ -1878,7 +1876,7 @@
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="n">
-        <v>11658</v>
+        <v>11041</v>
       </c>
     </row>
     <row r="50">
@@ -1888,22 +1886,22 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>4871</v>
+        <v>1706</v>
       </c>
       <c r="C50" t="n">
-        <v>2173</v>
+        <v>1097</v>
       </c>
       <c r="D50" t="n">
-        <v>130</v>
+        <v>98</v>
       </c>
       <c r="E50" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F50" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H50" t="n">
         <v>2</v>
@@ -1911,7 +1909,7 @@
       <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr"/>
       <c r="K50" t="n">
-        <v>7190</v>
+        <v>2915</v>
       </c>
     </row>
     <row r="51">
@@ -1921,19 +1919,19 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>5834</v>
+        <v>3675</v>
       </c>
       <c r="C51" t="n">
-        <v>2780</v>
+        <v>3129</v>
       </c>
       <c r="D51" t="n">
-        <v>53</v>
+        <v>307</v>
       </c>
       <c r="E51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F51" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G51" t="n">
         <v>2</v>
@@ -1942,7 +1940,7 @@
       <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr"/>
       <c r="K51" t="n">
-        <v>8677</v>
+        <v>7121</v>
       </c>
     </row>
     <row r="52">
@@ -1952,13 +1950,13 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>1584</v>
+        <v>1257</v>
       </c>
       <c r="C52" t="n">
-        <v>39</v>
+        <v>654</v>
       </c>
       <c r="D52" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E52" t="n">
         <v>1</v>
@@ -1979,7 +1977,7 @@
         <v>0</v>
       </c>
       <c r="K52" t="n">
-        <v>1631</v>
+        <v>1923</v>
       </c>
     </row>
     <row r="53">
@@ -1989,13 +1987,13 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>1584</v>
+        <v>1257</v>
       </c>
       <c r="C53" t="n">
-        <v>39</v>
+        <v>654</v>
       </c>
       <c r="D53" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E53" t="n">
         <v>1</v>
@@ -2010,7 +2008,7 @@
       <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr"/>
       <c r="K53" t="n">
-        <v>1631</v>
+        <v>1923</v>
       </c>
     </row>
     <row r="54">
@@ -2020,25 +2018,25 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>73757</v>
+        <v>60816</v>
       </c>
       <c r="C54" t="n">
-        <v>17270</v>
+        <v>21293</v>
       </c>
       <c r="D54" t="n">
-        <v>818</v>
+        <v>1504</v>
       </c>
       <c r="E54" t="n">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="F54" t="n">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="G54" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H54" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I54" t="n">
         <v>2</v>
@@ -2047,7 +2045,7 @@
         <v>0</v>
       </c>
       <c r="K54" t="n">
-        <v>92253</v>
+        <v>84018</v>
       </c>
     </row>
   </sheetData>
@@ -2123,16 +2121,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1423</v>
+        <v>938</v>
       </c>
       <c r="C2" t="n">
         <v>14</v>
       </c>
       <c r="D2" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F2" t="n">
         <v>5</v>
@@ -2147,7 +2145,7 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>1460</v>
+        <v>974</v>
       </c>
     </row>
     <row r="3">
@@ -2157,20 +2155,20 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>998</v>
+        <v>1268</v>
       </c>
       <c r="C3" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F3" t="n">
         <v>3</v>
       </c>
-      <c r="E3" t="n">
-        <v>8</v>
-      </c>
-      <c r="F3" t="n">
-        <v>2</v>
-      </c>
       <c r="G3" t="n">
         <v>2</v>
       </c>
@@ -2181,7 +2179,7 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>1022</v>
+        <v>1295</v>
       </c>
     </row>
     <row r="4">
@@ -2191,19 +2189,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10589</v>
+        <v>8086</v>
       </c>
       <c r="C4" t="n">
-        <v>5009</v>
+        <v>7134</v>
       </c>
       <c r="D4" t="n">
-        <v>100</v>
+        <v>326</v>
       </c>
       <c r="E4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G4" t="n">
         <v>3</v>
@@ -2215,7 +2213,7 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>15724</v>
+        <v>15570</v>
       </c>
     </row>
     <row r="5">
@@ -2225,16 +2223,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1714</v>
+        <v>1751</v>
       </c>
       <c r="C5" t="n">
-        <v>177</v>
+        <v>18</v>
       </c>
       <c r="D5" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
@@ -2249,7 +2247,7 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>1906</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="6">
@@ -2259,16 +2257,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2243</v>
+        <v>554</v>
       </c>
       <c r="C6" t="n">
-        <v>66</v>
+        <v>33</v>
       </c>
       <c r="D6" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
@@ -2283,7 +2281,7 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>2342</v>
+        <v>599</v>
       </c>
     </row>
     <row r="7">
@@ -2293,17 +2291,17 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1261</v>
+        <v>1390</v>
       </c>
       <c r="C7" t="n">
-        <v>24</v>
+        <v>76</v>
       </c>
       <c r="D7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" t="n">
         <v>4</v>
       </c>
-      <c r="E7" t="n">
-        <v>3</v>
-      </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
@@ -2317,7 +2315,7 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>1293</v>
+        <v>1474</v>
       </c>
     </row>
     <row r="8">
@@ -2327,16 +2325,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1047</v>
+        <v>754</v>
       </c>
       <c r="C8" t="n">
+        <v>12</v>
+      </c>
+      <c r="D8" t="n">
         <v>8</v>
       </c>
-      <c r="D8" t="n">
-        <v>9</v>
-      </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F8" t="n">
         <v>2</v>
@@ -2351,7 +2349,7 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>1069</v>
+        <v>780</v>
       </c>
     </row>
     <row r="9">
@@ -2361,13 +2359,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C9" t="n">
-        <v>26</v>
+        <v>70</v>
       </c>
       <c r="D9" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E9" t="n">
         <v>1</v>
@@ -2385,7 +2383,7 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>300</v>
+        <v>345</v>
       </c>
     </row>
     <row r="10">
@@ -2395,10 +2393,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -2419,7 +2417,7 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>37</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11">
@@ -2429,19 +2427,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>316</v>
+        <v>350</v>
       </c>
       <c r="C11" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="D11" t="n">
         <v>4</v>
       </c>
       <c r="E11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
@@ -2453,7 +2451,7 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>333</v>
+        <v>378</v>
       </c>
     </row>
     <row r="12">
@@ -2463,19 +2461,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4174</v>
+        <v>1041</v>
       </c>
       <c r="C12" t="n">
-        <v>2010</v>
+        <v>398</v>
       </c>
       <c r="D12" t="n">
-        <v>39</v>
+        <v>75</v>
       </c>
       <c r="E12" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F12" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G12" t="n">
         <v>3</v>
@@ -2487,7 +2485,7 @@
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>6249</v>
+        <v>1538</v>
       </c>
     </row>
     <row r="13">
@@ -2497,10 +2495,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="C13" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="D13" t="n">
         <v>1</v>
@@ -2521,7 +2519,7 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
     </row>
     <row r="14">
@@ -2531,10 +2529,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1136</v>
+        <v>1226</v>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D14" t="n">
         <v>3</v>
@@ -2555,7 +2553,7 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>1144</v>
+        <v>1239</v>
       </c>
     </row>
     <row r="15">
@@ -2565,10 +2563,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>510</v>
+        <v>557</v>
       </c>
       <c r="C15" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="D15" t="n">
         <v>1</v>
@@ -2589,7 +2587,7 @@
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>517</v>
+        <v>574</v>
       </c>
     </row>
     <row r="16">
@@ -2599,10 +2597,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>386</v>
+        <v>511</v>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="D16" t="n">
         <v>4</v>
@@ -2623,7 +2621,7 @@
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>395</v>
+        <v>542</v>
       </c>
     </row>
     <row r="17">
@@ -2633,10 +2631,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="C17" t="n">
-        <v>5</v>
+        <v>35</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
@@ -2657,7 +2655,7 @@
         <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>100</v>
+        <v>121</v>
       </c>
     </row>
     <row r="18">
@@ -2667,13 +2665,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>172</v>
+        <v>151</v>
       </c>
       <c r="C18" t="n">
-        <v>31</v>
+        <v>84</v>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
@@ -2691,7 +2689,7 @@
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>203</v>
+        <v>236</v>
       </c>
     </row>
     <row r="19">
@@ -2701,16 +2699,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2300</v>
+        <v>2383</v>
       </c>
       <c r="C19" t="n">
-        <v>75</v>
+        <v>186</v>
       </c>
       <c r="D19" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E19" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F19" t="n">
         <v>3</v>
@@ -2725,7 +2723,7 @@
         <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>2431</v>
+        <v>2626</v>
       </c>
     </row>
     <row r="20">
@@ -2735,13 +2733,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>491</v>
+        <v>393</v>
       </c>
       <c r="C20" t="n">
-        <v>14</v>
+        <v>174</v>
       </c>
       <c r="D20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E20" t="n">
         <v>3</v>
@@ -2759,7 +2757,7 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>513</v>
+        <v>576</v>
       </c>
     </row>
     <row r="21">
@@ -2772,16 +2770,16 @@
         <v>84</v>
       </c>
       <c r="C21" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="D21" t="n">
         <v>3</v>
       </c>
       <c r="E21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
@@ -2793,7 +2791,7 @@
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>93</v>
+        <v>99</v>
       </c>
     </row>
     <row r="22">
@@ -2803,10 +2801,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>274</v>
+        <v>265</v>
       </c>
       <c r="C22" t="n">
-        <v>40</v>
+        <v>105</v>
       </c>
       <c r="D22" t="n">
         <v>1</v>
@@ -2827,7 +2825,7 @@
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>317</v>
+        <v>373</v>
       </c>
     </row>
     <row r="23">
@@ -2837,10 +2835,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>374</v>
+        <v>325</v>
       </c>
       <c r="C23" t="n">
-        <v>70</v>
+        <v>181</v>
       </c>
       <c r="D23" t="n">
         <v>1</v>
@@ -2861,7 +2859,7 @@
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>445</v>
+        <v>507</v>
       </c>
     </row>
     <row r="24">
@@ -2871,13 +2869,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>312</v>
+        <v>260</v>
       </c>
       <c r="C24" t="n">
-        <v>34</v>
+        <v>120</v>
       </c>
       <c r="D24" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E24" t="n">
         <v>1</v>
@@ -2895,7 +2893,7 @@
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>357</v>
+        <v>393</v>
       </c>
     </row>
     <row r="25">
@@ -2905,10 +2903,10 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>264</v>
+        <v>281</v>
       </c>
       <c r="C25" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
@@ -2929,7 +2927,7 @@
         <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>268</v>
+        <v>288</v>
       </c>
     </row>
     <row r="26">
@@ -2939,19 +2937,19 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2795</v>
+        <v>4762</v>
       </c>
       <c r="C26" t="n">
-        <v>373</v>
+        <v>396</v>
       </c>
       <c r="D26" t="n">
-        <v>126</v>
+        <v>177</v>
       </c>
       <c r="E26" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F26" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G26" t="n">
         <v>3</v>
@@ -2963,7 +2961,7 @@
         <v>1</v>
       </c>
       <c r="J26" t="n">
-        <v>3329</v>
+        <v>5367</v>
       </c>
     </row>
     <row r="27">
@@ -2973,13 +2971,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1830</v>
+        <v>1915</v>
       </c>
       <c r="C27" t="n">
-        <v>55</v>
+        <v>212</v>
       </c>
       <c r="D27" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E27" t="n">
         <v>7</v>
@@ -2997,7 +2995,7 @@
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>1903</v>
+        <v>2147</v>
       </c>
     </row>
     <row r="28">
@@ -3007,13 +3005,13 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>3220</v>
+        <v>2716</v>
       </c>
       <c r="C28" t="n">
-        <v>56</v>
+        <v>685</v>
       </c>
       <c r="D28" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="E28" t="n">
         <v>8</v>
@@ -3022,7 +3020,7 @@
         <v>5</v>
       </c>
       <c r="G28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H28" t="n">
         <v>0</v>
@@ -3031,7 +3029,7 @@
         <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>3299</v>
+        <v>3430</v>
       </c>
     </row>
     <row r="29">
@@ -3041,19 +3039,19 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>151</v>
+        <v>198</v>
       </c>
       <c r="C29" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D29" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G29" t="n">
         <v>0</v>
@@ -3065,7 +3063,7 @@
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>163</v>
+        <v>219</v>
       </c>
     </row>
     <row r="30">
@@ -3075,13 +3073,13 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C30" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E30" t="n">
         <v>0</v>
@@ -3099,7 +3097,7 @@
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>47</v>
+        <v>52</v>
       </c>
     </row>
     <row r="31">
@@ -3109,19 +3107,19 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>7439</v>
+        <v>5946</v>
       </c>
       <c r="C31" t="n">
-        <v>3063</v>
+        <v>4783</v>
       </c>
       <c r="D31" t="n">
-        <v>53</v>
+        <v>204</v>
       </c>
       <c r="E31" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F31" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G31" t="n">
         <v>5</v>
@@ -3133,7 +3131,7 @@
         <v>0</v>
       </c>
       <c r="J31" t="n">
-        <v>10588</v>
+        <v>10965</v>
       </c>
     </row>
     <row r="32">
@@ -3143,13 +3141,13 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C32" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="D32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E32" t="n">
         <v>2</v>
@@ -3167,7 +3165,7 @@
         <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>113</v>
+        <v>126</v>
       </c>
     </row>
     <row r="33">
@@ -3177,16 +3175,16 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>44</v>
+        <v>107</v>
       </c>
       <c r="C33" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F33" t="n">
         <v>0</v>
@@ -3201,7 +3199,7 @@
         <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>47</v>
+        <v>112</v>
       </c>
     </row>
     <row r="34">
@@ -3211,10 +3209,10 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="C34" t="n">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="D34" t="n">
         <v>0</v>
@@ -3235,7 +3233,7 @@
         <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>124</v>
+        <v>151</v>
       </c>
     </row>
     <row r="35">
@@ -3245,13 +3243,13 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>323</v>
+        <v>263</v>
       </c>
       <c r="C35" t="n">
-        <v>53</v>
+        <v>166</v>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E35" t="n">
         <v>0</v>
@@ -3269,7 +3267,7 @@
         <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>378</v>
+        <v>433</v>
       </c>
     </row>
     <row r="36">
@@ -3279,13 +3277,13 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1124</v>
+        <v>988</v>
       </c>
       <c r="C36" t="n">
-        <v>39</v>
+        <v>376</v>
       </c>
       <c r="D36" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E36" t="n">
         <v>2</v>
@@ -3303,7 +3301,7 @@
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>1177</v>
+        <v>1383</v>
       </c>
     </row>
     <row r="37">
@@ -3313,10 +3311,10 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="C37" t="n">
-        <v>24</v>
+        <v>74</v>
       </c>
       <c r="D37" t="n">
         <v>0</v>
@@ -3337,7 +3335,7 @@
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>218</v>
+        <v>258</v>
       </c>
     </row>
     <row r="38">
@@ -3347,10 +3345,10 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>567</v>
+        <v>615</v>
       </c>
       <c r="C38" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="D38" t="n">
         <v>2</v>
@@ -3371,7 +3369,7 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>585</v>
+        <v>658</v>
       </c>
     </row>
     <row r="39">
@@ -3381,16 +3379,16 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>129</v>
+        <v>115</v>
       </c>
       <c r="C39" t="n">
-        <v>16</v>
+        <v>49</v>
       </c>
       <c r="D39" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F39" t="n">
         <v>1</v>
@@ -3405,7 +3403,7 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>150</v>
+        <v>170</v>
       </c>
     </row>
     <row r="40">
@@ -3415,10 +3413,10 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>712</v>
+        <v>805</v>
       </c>
       <c r="C40" t="n">
-        <v>13</v>
+        <v>48</v>
       </c>
       <c r="D40" t="n">
         <v>0</v>
@@ -3439,7 +3437,7 @@
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>729</v>
+        <v>857</v>
       </c>
     </row>
     <row r="41">
@@ -3449,17 +3447,17 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>340</v>
+        <v>406</v>
       </c>
       <c r="C41" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D41" t="n">
+        <v>3</v>
+      </c>
+      <c r="E41" t="n">
         <v>4</v>
       </c>
-      <c r="E41" t="n">
-        <v>3</v>
-      </c>
       <c r="F41" t="n">
         <v>1</v>
       </c>
@@ -3473,7 +3471,7 @@
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>355</v>
+        <v>425</v>
       </c>
     </row>
     <row r="42">
@@ -3483,19 +3481,19 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>353</v>
+        <v>502</v>
       </c>
       <c r="C42" t="n">
         <v>36</v>
       </c>
       <c r="D42" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E42" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G42" t="n">
         <v>0</v>
@@ -3507,7 +3505,7 @@
         <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>393</v>
+        <v>544</v>
       </c>
     </row>
     <row r="43">
@@ -3517,16 +3515,16 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>1283</v>
+        <v>1162</v>
       </c>
       <c r="C43" t="n">
-        <v>34</v>
+        <v>272</v>
       </c>
       <c r="D43" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E43" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F43" t="n">
         <v>1</v>
@@ -3541,7 +3539,7 @@
         <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>1324</v>
+        <v>1445</v>
       </c>
     </row>
     <row r="44">
@@ -3551,16 +3549,16 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>369</v>
+        <v>352</v>
       </c>
       <c r="C44" t="n">
-        <v>36</v>
+        <v>110</v>
       </c>
       <c r="D44" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F44" t="n">
         <v>0</v>
@@ -3575,7 +3573,7 @@
         <v>1</v>
       </c>
       <c r="J44" t="n">
-        <v>415</v>
+        <v>472</v>
       </c>
     </row>
     <row r="45">
@@ -3585,16 +3583,16 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>224</v>
+        <v>256</v>
       </c>
       <c r="C45" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D45" t="n">
         <v>2</v>
       </c>
       <c r="E45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F45" t="n">
         <v>1</v>
@@ -3609,7 +3607,7 @@
         <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>235</v>
+        <v>269</v>
       </c>
     </row>
     <row r="46">
@@ -3619,31 +3617,31 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>1061</v>
+        <v>698</v>
       </c>
       <c r="C46" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D46" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E46" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F46" t="n">
         <v>6</v>
       </c>
       <c r="G46" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I46" t="n">
         <v>0</v>
       </c>
       <c r="J46" t="n">
-        <v>1091</v>
+        <v>729</v>
       </c>
     </row>
     <row r="47">
@@ -3653,10 +3651,10 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="C47" t="n">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="D47" t="n">
         <v>3</v>
@@ -3677,7 +3675,7 @@
         <v>0</v>
       </c>
       <c r="J47" t="n">
-        <v>160</v>
+        <v>180</v>
       </c>
     </row>
     <row r="48">
@@ -3687,19 +3685,19 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>667</v>
+        <v>855</v>
       </c>
       <c r="C48" t="n">
-        <v>12</v>
+        <v>45</v>
       </c>
       <c r="D48" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E48" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F48" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G48" t="n">
         <v>1</v>
@@ -3711,7 +3709,7 @@
         <v>0</v>
       </c>
       <c r="J48" t="n">
-        <v>698</v>
+        <v>922</v>
       </c>
     </row>
     <row r="49">
@@ -3721,13 +3719,13 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>256</v>
+        <v>216</v>
       </c>
       <c r="C49" t="n">
-        <v>45</v>
+        <v>121</v>
       </c>
       <c r="D49" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E49" t="n">
         <v>1</v>
@@ -3745,7 +3743,7 @@
         <v>0</v>
       </c>
       <c r="J49" t="n">
-        <v>303</v>
+        <v>338</v>
       </c>
     </row>
     <row r="50">
@@ -3755,13 +3753,13 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>217</v>
+        <v>235</v>
       </c>
       <c r="C50" t="n">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="D50" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E50" t="n">
         <v>0</v>
@@ -3779,7 +3777,7 @@
         <v>0</v>
       </c>
       <c r="J50" t="n">
-        <v>244</v>
+        <v>290</v>
       </c>
     </row>
     <row r="51">
@@ -3789,10 +3787,10 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>369</v>
+        <v>562</v>
       </c>
       <c r="C51" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D51" t="n">
         <v>1</v>
@@ -3813,7 +3811,7 @@
         <v>0</v>
       </c>
       <c r="J51" t="n">
-        <v>390</v>
+        <v>584</v>
       </c>
     </row>
     <row r="52">
@@ -3823,22 +3821,22 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>5748</v>
+        <v>1951</v>
       </c>
       <c r="C52" t="n">
-        <v>2522</v>
+        <v>1167</v>
       </c>
       <c r="D52" t="n">
-        <v>179</v>
+        <v>128</v>
       </c>
       <c r="E52" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F52" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H52" t="n">
         <v>2</v>
@@ -3847,7 +3845,7 @@
         <v>0</v>
       </c>
       <c r="J52" t="n">
-        <v>8467</v>
+        <v>3262</v>
       </c>
     </row>
     <row r="53">
@@ -3857,16 +3855,16 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>868</v>
+        <v>670</v>
       </c>
       <c r="C53" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D53" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E53" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F53" t="n">
         <v>0</v>
@@ -3881,7 +3879,7 @@
         <v>0</v>
       </c>
       <c r="J53" t="n">
-        <v>884</v>
+        <v>689</v>
       </c>
     </row>
     <row r="54">
@@ -3891,13 +3889,13 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="C54" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="D54" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E54" t="n">
         <v>0</v>
@@ -3915,7 +3913,7 @@
         <v>0</v>
       </c>
       <c r="J54" t="n">
-        <v>95</v>
+        <v>117</v>
       </c>
     </row>
     <row r="55">
@@ -3925,19 +3923,19 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>5324</v>
+        <v>3444</v>
       </c>
       <c r="C55" t="n">
-        <v>2661</v>
+        <v>3114</v>
       </c>
       <c r="D55" t="n">
-        <v>60</v>
+        <v>298</v>
       </c>
       <c r="E55" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F55" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G55" t="n">
         <v>2</v>
@@ -3949,7 +3947,7 @@
         <v>0</v>
       </c>
       <c r="J55" t="n">
-        <v>8056</v>
+        <v>6868</v>
       </c>
     </row>
     <row r="56">
@@ -3959,13 +3957,13 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>279</v>
+        <v>338</v>
       </c>
       <c r="C56" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D56" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E56" t="n">
         <v>1</v>
@@ -3983,7 +3981,7 @@
         <v>0</v>
       </c>
       <c r="J56" t="n">
-        <v>295</v>
+        <v>357</v>
       </c>
     </row>
     <row r="57">
@@ -3993,13 +3991,13 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>149</v>
+        <v>127</v>
       </c>
       <c r="C57" t="n">
-        <v>34</v>
+        <v>72</v>
       </c>
       <c r="D57" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E57" t="n">
         <v>1</v>
@@ -4017,7 +4015,7 @@
         <v>0</v>
       </c>
       <c r="J57" t="n">
-        <v>191</v>
+        <v>211</v>
       </c>
     </row>
     <row r="58">
@@ -4027,17 +4025,17 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C58" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D58" t="n">
+        <v>3</v>
+      </c>
+      <c r="E58" t="n">
         <v>4</v>
       </c>
-      <c r="E58" t="n">
-        <v>3</v>
-      </c>
       <c r="F58" t="n">
         <v>0</v>
       </c>
@@ -4051,7 +4049,7 @@
         <v>0</v>
       </c>
       <c r="J58" t="n">
-        <v>75</v>
+        <v>85</v>
       </c>
     </row>
     <row r="59">
@@ -4061,10 +4059,10 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="C59" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="D59" t="n">
         <v>1</v>
@@ -4085,7 +4083,7 @@
         <v>0</v>
       </c>
       <c r="J59" t="n">
-        <v>74</v>
+        <v>79</v>
       </c>
     </row>
     <row r="60">
@@ -4095,16 +4093,16 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>488</v>
+        <v>657</v>
       </c>
       <c r="C60" t="n">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="D60" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E60" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F60" t="n">
         <v>0</v>
@@ -4119,7 +4117,7 @@
         <v>0</v>
       </c>
       <c r="J60" t="n">
-        <v>519</v>
+        <v>699</v>
       </c>
     </row>
     <row r="61">
@@ -4129,19 +4127,19 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>1549</v>
+        <v>1606</v>
       </c>
       <c r="C61" t="n">
-        <v>73</v>
+        <v>181</v>
       </c>
       <c r="D61" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E61" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F61" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G61" t="n">
         <v>1</v>
@@ -4153,7 +4151,7 @@
         <v>0</v>
       </c>
       <c r="J61" t="n">
-        <v>1638</v>
+        <v>1803</v>
       </c>
     </row>
     <row r="62">
@@ -4163,13 +4161,13 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>953</v>
+        <v>856</v>
       </c>
       <c r="C62" t="n">
-        <v>38</v>
+        <v>221</v>
       </c>
       <c r="D62" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E62" t="n">
         <v>0</v>
@@ -4187,7 +4185,7 @@
         <v>0</v>
       </c>
       <c r="J62" t="n">
-        <v>1001</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="63">
@@ -4197,16 +4195,16 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>1784</v>
+        <v>2594</v>
       </c>
       <c r="C63" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="D63" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E63" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F63" t="n">
         <v>7</v>
@@ -4221,7 +4219,7 @@
         <v>0</v>
       </c>
       <c r="J63" t="n">
-        <v>1849</v>
+        <v>2672</v>
       </c>
     </row>
     <row r="64">
@@ -4231,16 +4229,16 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>1798</v>
+        <v>1057</v>
       </c>
       <c r="C64" t="n">
-        <v>241</v>
+        <v>39</v>
       </c>
       <c r="D64" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E64" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F64" t="n">
         <v>3</v>
@@ -4255,7 +4253,7 @@
         <v>0</v>
       </c>
       <c r="J64" t="n">
-        <v>2061</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="65">
@@ -4265,31 +4263,31 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>73757</v>
+        <v>60816</v>
       </c>
       <c r="C65" t="n">
-        <v>17270</v>
+        <v>21293</v>
       </c>
       <c r="D65" t="n">
-        <v>818</v>
+        <v>1504</v>
       </c>
       <c r="E65" t="n">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="F65" t="n">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="G65" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H65" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I65" t="n">
         <v>2</v>
       </c>
       <c r="J65" t="n">
-        <v>92253</v>
+        <v>84018</v>
       </c>
     </row>
   </sheetData>
@@ -4365,16 +4363,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>10877</v>
+        <v>8310</v>
       </c>
       <c r="C2" t="n">
-        <v>4956</v>
+        <v>7027</v>
       </c>
       <c r="D2" t="n">
-        <v>101</v>
+        <v>306</v>
       </c>
       <c r="E2" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F2" t="n">
         <v>8</v>
@@ -4389,7 +4387,7 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>15957</v>
+        <v>15663</v>
       </c>
     </row>
     <row r="3">
@@ -4399,19 +4397,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4092</v>
+        <v>978</v>
       </c>
       <c r="C3" t="n">
-        <v>1982</v>
+        <v>366</v>
       </c>
       <c r="D3" t="n">
-        <v>39</v>
+        <v>76</v>
       </c>
       <c r="E3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F3" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G3" t="n">
         <v>2</v>
@@ -4423,7 +4421,7 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>6136</v>
+        <v>1441</v>
       </c>
     </row>
     <row r="4">
@@ -4433,19 +4431,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1425</v>
+        <v>2144</v>
       </c>
       <c r="C4" t="n">
-        <v>219</v>
+        <v>268</v>
       </c>
       <c r="D4" t="n">
-        <v>115</v>
+        <v>162</v>
       </c>
       <c r="E4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G4" t="n">
         <v>3</v>
@@ -4457,7 +4455,7 @@
         <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>1786</v>
+        <v>2598</v>
       </c>
     </row>
     <row r="5">
@@ -4467,19 +4465,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>669</v>
+        <v>753</v>
       </c>
       <c r="C5" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="D5" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -4491,7 +4489,7 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>705</v>
+        <v>801</v>
       </c>
     </row>
     <row r="6">
@@ -4501,19 +4499,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>634</v>
+        <v>821</v>
       </c>
       <c r="C6" t="n">
-        <v>11</v>
+        <v>45</v>
       </c>
       <c r="D6" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -4525,7 +4523,7 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>663</v>
+        <v>886</v>
       </c>
     </row>
     <row r="7">
@@ -4535,13 +4533,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1064</v>
+        <v>1343</v>
       </c>
       <c r="C7" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D7" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>
@@ -4559,7 +4557,7 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>1088</v>
+        <v>1373</v>
       </c>
     </row>
     <row r="8">
@@ -4569,16 +4567,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2252</v>
+        <v>461</v>
       </c>
       <c r="C8" t="n">
-        <v>72</v>
+        <v>35</v>
       </c>
       <c r="D8" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="E8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
@@ -4593,7 +4591,7 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>2357</v>
+        <v>506</v>
       </c>
     </row>
     <row r="9">
@@ -4603,16 +4601,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1284</v>
+        <v>1166</v>
       </c>
       <c r="C9" t="n">
-        <v>22</v>
+        <v>261</v>
       </c>
       <c r="D9" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
         <v>1</v>
@@ -4627,7 +4625,7 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>1313</v>
+        <v>1438</v>
       </c>
     </row>
     <row r="10">
@@ -4637,13 +4635,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>934</v>
+        <v>822</v>
       </c>
       <c r="C10" t="n">
-        <v>38</v>
+        <v>221</v>
       </c>
       <c r="D10" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -4661,7 +4659,7 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>981</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="11">
@@ -4671,19 +4669,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2329</v>
+        <v>3430</v>
       </c>
       <c r="C11" t="n">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="D11" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E11" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G11" t="n">
         <v>2</v>
@@ -4695,7 +4693,7 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>2414</v>
+        <v>3529</v>
       </c>
     </row>
     <row r="12">
@@ -4705,13 +4703,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="C12" t="n">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="D12" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
@@ -4729,7 +4727,7 @@
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>97</v>
+        <v>105</v>
       </c>
     </row>
     <row r="13">
@@ -4739,19 +4737,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>76</v>
+        <v>14</v>
       </c>
       <c r="C13" t="n">
-        <v>76</v>
+        <v>61</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
@@ -4763,7 +4761,7 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>153</v>
+        <v>80</v>
       </c>
     </row>
     <row r="14">
@@ -4773,13 +4771,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
@@ -4797,7 +4795,7 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>21</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15">
@@ -4807,13 +4805,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>52</v>
+        <v>4</v>
       </c>
       <c r="C15" t="n">
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
         <v>1</v>
@@ -4831,7 +4829,7 @@
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>136</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16">
@@ -4841,10 +4839,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>57</v>
+        <v>5</v>
       </c>
       <c r="C16" t="n">
-        <v>57</v>
+        <v>0</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
@@ -4865,7 +4863,7 @@
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>117</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17">
@@ -4875,10 +4873,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>88</v>
+        <v>9</v>
       </c>
       <c r="C17" t="n">
-        <v>65</v>
+        <v>4</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
@@ -4899,7 +4897,7 @@
         <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>154</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18">
@@ -4909,13 +4907,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C18" t="n">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="D18" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E18" t="n">
         <v>1</v>
@@ -4933,7 +4931,7 @@
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
     </row>
     <row r="19">
@@ -4943,16 +4941,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>58</v>
+        <v>1</v>
       </c>
       <c r="C19" t="n">
-        <v>66</v>
+        <v>2</v>
       </c>
       <c r="D19" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F19" t="n">
         <v>1</v>
@@ -4967,7 +4965,7 @@
         <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>140</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20">
@@ -4977,10 +4975,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="C20" t="n">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="D20" t="n">
         <v>1</v>
@@ -5001,7 +4999,7 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="21">
@@ -5011,10 +5009,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>113</v>
+        <v>16</v>
       </c>
       <c r="C21" t="n">
-        <v>79</v>
+        <v>17</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
@@ -5035,7 +5033,7 @@
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>192</v>
+        <v>33</v>
       </c>
     </row>
     <row r="22">
@@ -5045,13 +5043,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>76</v>
+        <v>45</v>
       </c>
       <c r="C22" t="n">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="D22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
@@ -5069,7 +5067,7 @@
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>134</v>
+        <v>139</v>
       </c>
     </row>
     <row r="23">
@@ -5079,13 +5077,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="C23" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -5103,7 +5101,7 @@
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>34</v>
+        <v>47</v>
       </c>
     </row>
     <row r="24">
@@ -5113,13 +5111,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>139</v>
+        <v>199</v>
       </c>
       <c r="C24" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="D24" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -5137,7 +5135,7 @@
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>191</v>
+        <v>256</v>
       </c>
     </row>
     <row r="25">
@@ -5150,7 +5148,7 @@
         <v>53</v>
       </c>
       <c r="C25" t="n">
-        <v>37</v>
+        <v>60</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
@@ -5171,7 +5169,7 @@
         <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>91</v>
+        <v>114</v>
       </c>
     </row>
     <row r="26">
@@ -5181,13 +5179,13 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1309</v>
+        <v>1081</v>
       </c>
       <c r="C26" t="n">
-        <v>53</v>
+        <v>549</v>
       </c>
       <c r="D26" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E26" t="n">
         <v>5</v>
@@ -5205,7 +5203,7 @@
         <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>1383</v>
+        <v>1657</v>
       </c>
     </row>
     <row r="27">
@@ -5215,16 +5213,16 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2021</v>
+        <v>2249</v>
       </c>
       <c r="C27" t="n">
-        <v>37</v>
+        <v>123</v>
       </c>
       <c r="D27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E27" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F27" t="n">
         <v>1</v>
@@ -5239,7 +5237,7 @@
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>2070</v>
+        <v>2384</v>
       </c>
     </row>
     <row r="28">
@@ -5249,31 +5247,31 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>6327</v>
+        <v>4031</v>
       </c>
       <c r="C28" t="n">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="D28" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E28" t="n">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="F28" t="n">
         <v>19</v>
       </c>
       <c r="G28" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I28" t="n">
         <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>6485</v>
+        <v>4215</v>
       </c>
     </row>
     <row r="29">
@@ -5283,19 +5281,19 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>600</v>
+        <v>542</v>
       </c>
       <c r="C29" t="n">
-        <v>41</v>
+        <v>146</v>
       </c>
       <c r="D29" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F29" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G29" t="n">
         <v>2</v>
@@ -5307,7 +5305,7 @@
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>674</v>
+        <v>723</v>
       </c>
     </row>
     <row r="30">
@@ -5317,19 +5315,19 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>546</v>
+        <v>725</v>
       </c>
       <c r="C30" t="n">
+        <v>37</v>
+      </c>
+      <c r="D30" t="n">
         <v>7</v>
       </c>
-      <c r="D30" t="n">
-        <v>5</v>
-      </c>
       <c r="E30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G30" t="n">
         <v>0</v>
@@ -5341,7 +5339,7 @@
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>564</v>
+        <v>775</v>
       </c>
     </row>
     <row r="31">
@@ -5351,16 +5349,16 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>3763</v>
+        <v>3963</v>
       </c>
       <c r="C31" t="n">
-        <v>66</v>
+        <v>126</v>
       </c>
       <c r="D31" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="E31" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F31" t="n">
         <v>0</v>
@@ -5375,7 +5373,7 @@
         <v>1</v>
       </c>
       <c r="J31" t="n">
-        <v>3882</v>
+        <v>4147</v>
       </c>
     </row>
     <row r="32">
@@ -5385,16 +5383,16 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>3934</v>
+        <v>3648</v>
       </c>
       <c r="C32" t="n">
-        <v>469</v>
+        <v>1344</v>
       </c>
       <c r="D32" t="n">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="E32" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F32" t="n">
         <v>7</v>
@@ -5409,7 +5407,7 @@
         <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>4444</v>
+        <v>5050</v>
       </c>
     </row>
     <row r="33">
@@ -5419,22 +5417,22 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>2516</v>
+        <v>4486</v>
       </c>
       <c r="C33" t="n">
-        <v>17</v>
+        <v>68</v>
       </c>
       <c r="D33" t="n">
+        <v>14</v>
+      </c>
+      <c r="E33" t="n">
         <v>12</v>
-      </c>
-      <c r="E33" t="n">
-        <v>11</v>
       </c>
       <c r="F33" t="n">
         <v>3</v>
       </c>
       <c r="G33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H33" t="n">
         <v>2</v>
@@ -5443,7 +5441,7 @@
         <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>2562</v>
+        <v>4585</v>
       </c>
     </row>
     <row r="34">
@@ -5453,13 +5451,13 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>2380</v>
+        <v>2521</v>
       </c>
       <c r="C34" t="n">
-        <v>63</v>
+        <v>248</v>
       </c>
       <c r="D34" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E34" t="n">
         <v>8</v>
@@ -5477,7 +5475,7 @@
         <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>2464</v>
+        <v>2792</v>
       </c>
     </row>
     <row r="35">
@@ -5487,13 +5485,13 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>570</v>
+        <v>671</v>
       </c>
       <c r="C35" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="D35" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E35" t="n">
         <v>5</v>
@@ -5511,7 +5509,7 @@
         <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>588</v>
+        <v>696</v>
       </c>
     </row>
     <row r="36">
@@ -5521,19 +5519,19 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1228</v>
+        <v>1763</v>
       </c>
       <c r="C36" t="n">
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="D36" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E36" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G36" t="n">
         <v>0</v>
@@ -5545,7 +5543,7 @@
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>1260</v>
+        <v>1814</v>
       </c>
     </row>
     <row r="37">
@@ -5555,19 +5553,19 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1620</v>
+        <v>1711</v>
       </c>
       <c r="C37" t="n">
-        <v>71</v>
+        <v>179</v>
       </c>
       <c r="D37" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E37" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G37" t="n">
         <v>1</v>
@@ -5579,7 +5577,7 @@
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>1705</v>
+        <v>1905</v>
       </c>
     </row>
     <row r="38">
@@ -5589,19 +5587,19 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>8217</v>
+        <v>6081</v>
       </c>
       <c r="C38" t="n">
-        <v>3320</v>
+        <v>4706</v>
       </c>
       <c r="D38" t="n">
-        <v>91</v>
+        <v>225</v>
       </c>
       <c r="E38" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F38" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G38" t="n">
         <v>5</v>
@@ -5613,7 +5611,7 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>11658</v>
+        <v>11041</v>
       </c>
     </row>
     <row r="39">
@@ -5623,13 +5621,13 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1584</v>
+        <v>1257</v>
       </c>
       <c r="C39" t="n">
-        <v>39</v>
+        <v>654</v>
       </c>
       <c r="D39" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E39" t="n">
         <v>1</v>
@@ -5647,7 +5645,7 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>1631</v>
+        <v>1923</v>
       </c>
     </row>
     <row r="40">
@@ -5657,22 +5655,22 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>4871</v>
+        <v>1706</v>
       </c>
       <c r="C40" t="n">
-        <v>2173</v>
+        <v>1097</v>
       </c>
       <c r="D40" t="n">
-        <v>130</v>
+        <v>98</v>
       </c>
       <c r="E40" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F40" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H40" t="n">
         <v>2</v>
@@ -5681,7 +5679,7 @@
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>7190</v>
+        <v>2915</v>
       </c>
     </row>
     <row r="41">
@@ -5691,19 +5689,19 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>5834</v>
+        <v>3675</v>
       </c>
       <c r="C41" t="n">
-        <v>2780</v>
+        <v>3129</v>
       </c>
       <c r="D41" t="n">
-        <v>53</v>
+        <v>307</v>
       </c>
       <c r="E41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F41" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G41" t="n">
         <v>2</v>
@@ -5715,7 +5713,7 @@
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>8677</v>
+        <v>7121</v>
       </c>
     </row>
     <row r="42">
@@ -5725,31 +5723,31 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>73757</v>
+        <v>60816</v>
       </c>
       <c r="C42" t="n">
-        <v>17270</v>
+        <v>21293</v>
       </c>
       <c r="D42" t="n">
-        <v>818</v>
+        <v>1504</v>
       </c>
       <c r="E42" t="n">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="F42" t="n">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="G42" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H42" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I42" t="n">
         <v>2</v>
       </c>
       <c r="J42" t="n">
-        <v>92253</v>
+        <v>84018</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): manual update 16/06/2026 05:17
</commit_message>
<xml_diff>
--- a/BaoCao_TonKho.xlsx
+++ b/BaoCao_TonKho.xlsx
@@ -443,7 +443,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>15/06/2026 21:26:31</t>
+          <t>16/06/2026 05:16:31</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -567,25 +567,25 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>14849</v>
+        <v>11381</v>
       </c>
       <c r="C7" t="n">
-        <v>933</v>
+        <v>1087</v>
       </c>
       <c r="D7" t="n">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="E7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -594,7 +594,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>15994</v>
+        <v>12687</v>
       </c>
     </row>
     <row r="8">
@@ -604,16 +604,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1912</v>
+        <v>547</v>
       </c>
       <c r="C8" t="n">
-        <v>184</v>
+        <v>66</v>
       </c>
       <c r="D8" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
@@ -621,7 +621,7 @@
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="n">
-        <v>2118</v>
+        <v>634</v>
       </c>
     </row>
     <row r="9">
@@ -631,20 +631,18 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2129</v>
+        <v>2193</v>
       </c>
       <c r="C9" t="n">
-        <v>150</v>
+        <v>214</v>
       </c>
       <c r="D9" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E9" t="n">
         <v>3</v>
       </c>
-      <c r="F9" t="n">
-        <v>1</v>
-      </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
         <v>2</v>
       </c>
@@ -654,7 +652,7 @@
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="n">
-        <v>2318</v>
+        <v>2446</v>
       </c>
     </row>
     <row r="10">
@@ -664,13 +662,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3848</v>
+        <v>1256</v>
       </c>
       <c r="C10" t="n">
-        <v>374</v>
+        <v>439</v>
       </c>
       <c r="D10" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
@@ -679,7 +677,7 @@
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="n">
-        <v>4254</v>
+        <v>1726</v>
       </c>
     </row>
     <row r="11">
@@ -689,13 +687,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>923</v>
+        <v>961</v>
       </c>
       <c r="C11" t="n">
-        <v>60</v>
+        <v>82</v>
       </c>
       <c r="D11" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E11" t="n">
         <v>1</v>
@@ -708,7 +706,7 @@
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="n">
-        <v>997</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="12">
@@ -718,13 +716,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>552</v>
+        <v>547</v>
       </c>
       <c r="C12" t="n">
-        <v>55</v>
+        <v>103</v>
       </c>
       <c r="D12" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
@@ -733,7 +731,7 @@
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="n">
-        <v>622</v>
+        <v>674</v>
       </c>
     </row>
     <row r="13">
@@ -743,13 +741,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>5485</v>
+        <v>5877</v>
       </c>
       <c r="C13" t="n">
-        <v>110</v>
+        <v>183</v>
       </c>
       <c r="D13" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E13" t="n">
         <v>8</v>
@@ -758,15 +756,15 @@
         <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="n">
-        <v>5685</v>
+        <v>6149</v>
       </c>
     </row>
     <row r="14">
@@ -776,13 +774,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1185</v>
+        <v>947</v>
       </c>
       <c r="C14" t="n">
-        <v>895</v>
+        <v>785</v>
       </c>
       <c r="D14" t="n">
-        <v>99</v>
+        <v>58</v>
       </c>
       <c r="E14" t="n">
         <v>1</v>
@@ -803,7 +801,7 @@
         <v>1</v>
       </c>
       <c r="K14" t="n">
-        <v>2190</v>
+        <v>1801</v>
       </c>
     </row>
     <row r="15">
@@ -816,7 +814,7 @@
         <v>24</v>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D15" t="n">
         <v>1</v>
@@ -830,7 +828,7 @@
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="16">
@@ -840,13 +838,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="C16" t="n">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="n">
@@ -857,7 +855,7 @@
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="n">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="17">
@@ -867,10 +865,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="C17" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D17" t="n">
         <v>1</v>
@@ -886,7 +884,7 @@
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
     </row>
     <row r="18">
@@ -896,13 +894,11 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>58</v>
-      </c>
-      <c r="C18" t="n">
-        <v>80</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="C18" t="inlineStr"/>
       <c r="D18" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
@@ -913,7 +909,7 @@
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="n">
-        <v>178</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19">
@@ -923,7 +919,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C19" t="n">
         <v>13</v>
@@ -938,7 +934,7 @@
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="20">
@@ -948,10 +944,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>76</v>
+        <v>65</v>
       </c>
       <c r="C20" t="n">
-        <v>43</v>
+        <v>57</v>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr"/>
@@ -961,7 +957,7 @@
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="n">
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
     <row r="21">
@@ -971,13 +967,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>68</v>
+        <v>9</v>
       </c>
       <c r="C21" t="n">
-        <v>83</v>
+        <v>7</v>
       </c>
       <c r="D21" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
@@ -986,7 +982,7 @@
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="n">
-        <v>158</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22">
@@ -998,7 +994,9 @@
       <c r="B22" t="n">
         <v>5</v>
       </c>
-      <c r="C22" t="inlineStr"/>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
       <c r="D22" t="n">
         <v>2</v>
       </c>
@@ -1011,7 +1009,7 @@
         <v>1</v>
       </c>
       <c r="K22" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23">
@@ -1021,13 +1019,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>56</v>
+        <v>13</v>
       </c>
       <c r="C23" t="n">
-        <v>74</v>
+        <v>3</v>
       </c>
       <c r="D23" t="n">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
@@ -1036,7 +1034,7 @@
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="n">
-        <v>157</v>
+        <v>18</v>
       </c>
     </row>
     <row r="24">
@@ -1046,11 +1044,9 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>29</v>
-      </c>
-      <c r="C24" t="n">
-        <v>1</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="C24" t="inlineStr"/>
       <c r="D24" t="n">
         <v>1</v>
       </c>
@@ -1061,7 +1057,7 @@
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="n">
-        <v>31</v>
+        <v>36</v>
       </c>
     </row>
     <row r="25">
@@ -1071,13 +1067,13 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="C25" t="n">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="D25" t="n">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
@@ -1088,7 +1084,7 @@
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="n">
-        <v>175</v>
+        <v>180</v>
       </c>
     </row>
     <row r="26">
@@ -1098,13 +1094,13 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>221</v>
+        <v>193</v>
       </c>
       <c r="C26" t="n">
-        <v>216</v>
+        <v>253</v>
       </c>
       <c r="D26" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
@@ -1117,7 +1113,7 @@
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="n">
-        <v>443</v>
+        <v>454</v>
       </c>
     </row>
     <row r="27">
@@ -1127,13 +1123,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>386</v>
+        <v>375</v>
       </c>
       <c r="C27" t="n">
-        <v>91</v>
+        <v>137</v>
       </c>
       <c r="D27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="n">
@@ -1146,7 +1142,7 @@
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="n">
-        <v>481</v>
+        <v>515</v>
       </c>
     </row>
     <row r="28">
@@ -1156,13 +1152,13 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="C28" t="n">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="D28" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
@@ -1171,7 +1167,7 @@
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="n">
-        <v>128</v>
+        <v>132</v>
       </c>
     </row>
     <row r="29">
@@ -1181,10 +1177,10 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>944</v>
+        <v>1012</v>
       </c>
       <c r="C29" t="n">
-        <v>46</v>
+        <v>79</v>
       </c>
       <c r="D29" t="n">
         <v>21</v>
@@ -1208,7 +1204,7 @@
         <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>1016</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="30">
@@ -1218,10 +1214,10 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>944</v>
+        <v>1012</v>
       </c>
       <c r="C30" t="n">
-        <v>46</v>
+        <v>79</v>
       </c>
       <c r="D30" t="n">
         <v>21</v>
@@ -1239,7 +1235,7 @@
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="n">
-        <v>1016</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="31">
@@ -1249,25 +1245,25 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>34719</v>
+        <v>27349</v>
       </c>
       <c r="C31" t="n">
-        <v>3512</v>
+        <v>5576</v>
       </c>
       <c r="D31" t="n">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="E31" t="n">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F31" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="G31" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H31" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I31" t="n">
         <v>0</v>
@@ -1276,7 +1272,7 @@
         <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>38976</v>
+        <v>33669</v>
       </c>
     </row>
     <row r="32">
@@ -1286,10 +1282,10 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>822</v>
+        <v>406</v>
       </c>
       <c r="C32" t="n">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="D32" t="n">
         <v>12</v>
@@ -1297,13 +1293,15 @@
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="n">
-        <v>5</v>
-      </c>
-      <c r="H32" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="H32" t="n">
+        <v>1</v>
+      </c>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="n">
-        <v>868</v>
+        <v>440</v>
       </c>
     </row>
     <row r="33">
@@ -1313,13 +1311,13 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1894</v>
+        <v>1948</v>
       </c>
       <c r="C33" t="n">
-        <v>257</v>
+        <v>374</v>
       </c>
       <c r="D33" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="E33" t="n">
         <v>1</v>
@@ -1330,7 +1328,7 @@
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="n">
-        <v>2190</v>
+        <v>2365</v>
       </c>
     </row>
     <row r="34">
@@ -1340,22 +1338,22 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>8937</v>
+        <v>5565</v>
       </c>
       <c r="C34" t="n">
-        <v>379</v>
+        <v>415</v>
       </c>
       <c r="D34" t="n">
-        <v>132</v>
+        <v>116</v>
       </c>
       <c r="E34" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F34" t="n">
         <v>4</v>
       </c>
       <c r="G34" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H34" t="n">
         <v>5</v>
@@ -1363,7 +1361,7 @@
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="n">
-        <v>9479</v>
+        <v>6129</v>
       </c>
     </row>
     <row r="35">
@@ -1373,10 +1371,10 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1400</v>
+        <v>1084</v>
       </c>
       <c r="C35" t="n">
-        <v>715</v>
+        <v>1104</v>
       </c>
       <c r="D35" t="n">
         <v>37</v>
@@ -1392,7 +1390,7 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="n">
-        <v>2155</v>
+        <v>2228</v>
       </c>
     </row>
     <row r="36">
@@ -1402,16 +1400,16 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>500</v>
+        <v>644</v>
       </c>
       <c r="C36" t="n">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D36" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr"/>
@@ -1421,7 +1419,7 @@
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="n">
-        <v>583</v>
+        <v>731</v>
       </c>
     </row>
     <row r="37">
@@ -1431,10 +1429,10 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>3859</v>
+        <v>4197</v>
       </c>
       <c r="C37" t="n">
-        <v>238</v>
+        <v>596</v>
       </c>
       <c r="D37" t="n">
         <v>116</v>
@@ -1442,9 +1440,7 @@
       <c r="E37" t="n">
         <v>22</v>
       </c>
-      <c r="F37" t="n">
-        <v>1</v>
-      </c>
+      <c r="F37" t="inlineStr"/>
       <c r="G37" t="n">
         <v>2</v>
       </c>
@@ -1452,7 +1448,7 @@
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="n">
-        <v>4238</v>
+        <v>4933</v>
       </c>
     </row>
     <row r="38">
@@ -1462,16 +1458,16 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>3088</v>
+        <v>2941</v>
       </c>
       <c r="C38" t="n">
-        <v>210</v>
+        <v>734</v>
       </c>
       <c r="D38" t="n">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="E38" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F38" t="n">
         <v>3</v>
@@ -1481,7 +1477,7 @@
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="n">
-        <v>3370</v>
+        <v>3744</v>
       </c>
     </row>
     <row r="39">
@@ -1491,22 +1487,20 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>5649</v>
+        <v>3658</v>
       </c>
       <c r="C39" t="n">
-        <v>149</v>
+        <v>339</v>
       </c>
       <c r="D39" t="n">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E39" t="n">
         <v>10</v>
       </c>
-      <c r="F39" t="n">
-        <v>1</v>
-      </c>
+      <c r="F39" t="inlineStr"/>
       <c r="G39" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H39" t="n">
         <v>2</v>
@@ -1514,7 +1508,7 @@
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="n">
-        <v>5994</v>
+        <v>4194</v>
       </c>
     </row>
     <row r="40">
@@ -1524,13 +1518,13 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1950</v>
+        <v>1825</v>
       </c>
       <c r="C40" t="n">
-        <v>649</v>
+        <v>942</v>
       </c>
       <c r="D40" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E40" t="n">
         <v>1</v>
@@ -1541,7 +1535,7 @@
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="n">
-        <v>2618</v>
+        <v>2788</v>
       </c>
     </row>
     <row r="41">
@@ -1551,13 +1545,13 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1275</v>
+        <v>1325</v>
       </c>
       <c r="C41" t="n">
-        <v>52</v>
+        <v>65</v>
       </c>
       <c r="D41" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr"/>
@@ -1568,7 +1562,7 @@
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="n">
-        <v>1338</v>
+        <v>1399</v>
       </c>
     </row>
     <row r="42">
@@ -1578,13 +1572,13 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>2264</v>
+        <v>736</v>
       </c>
       <c r="C42" t="n">
-        <v>345</v>
+        <v>306</v>
       </c>
       <c r="D42" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr"/>
@@ -1597,7 +1591,7 @@
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="n">
-        <v>2626</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="43">
@@ -1607,19 +1601,19 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>3081</v>
+        <v>3020</v>
       </c>
       <c r="C43" t="n">
-        <v>417</v>
+        <v>608</v>
       </c>
       <c r="D43" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E43" t="n">
         <v>2</v>
       </c>
       <c r="F43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="n">
@@ -1628,7 +1622,7 @@
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="n">
-        <v>3517</v>
+        <v>3656</v>
       </c>
     </row>
     <row r="44">
@@ -1638,16 +1632,16 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>3120</v>
+        <v>3412</v>
       </c>
       <c r="C44" t="n">
-        <v>585</v>
+        <v>721</v>
       </c>
       <c r="D44" t="n">
-        <v>380</v>
+        <v>348</v>
       </c>
       <c r="E44" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F44" t="n">
         <v>3</v>
@@ -1665,7 +1659,7 @@
         <v>0</v>
       </c>
       <c r="K44" t="n">
-        <v>4105</v>
+        <v>4503</v>
       </c>
     </row>
     <row r="45">
@@ -1675,16 +1669,16 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>3120</v>
+        <v>3412</v>
       </c>
       <c r="C45" t="n">
-        <v>585</v>
+        <v>721</v>
       </c>
       <c r="D45" t="n">
-        <v>380</v>
+        <v>348</v>
       </c>
       <c r="E45" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F45" t="n">
         <v>3</v>
@@ -1698,7 +1692,7 @@
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr"/>
       <c r="K45" t="n">
-        <v>4105</v>
+        <v>4503</v>
       </c>
     </row>
     <row r="46">
@@ -1708,22 +1702,22 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>25938</v>
+        <v>16366</v>
       </c>
       <c r="C46" t="n">
-        <v>10815</v>
+        <v>4212</v>
       </c>
       <c r="D46" t="n">
-        <v>743</v>
+        <v>416</v>
       </c>
       <c r="E46" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F46" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G46" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H46" t="n">
         <v>26</v>
@@ -1735,7 +1729,7 @@
         <v>1</v>
       </c>
       <c r="K46" t="n">
-        <v>37567</v>
+        <v>21064</v>
       </c>
     </row>
     <row r="47">
@@ -1745,13 +1739,13 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>11660</v>
+        <v>6142</v>
       </c>
       <c r="C47" t="n">
-        <v>5359</v>
+        <v>1796</v>
       </c>
       <c r="D47" t="n">
-        <v>340</v>
+        <v>133</v>
       </c>
       <c r="E47" t="n">
         <v>3</v>
@@ -1768,7 +1762,7 @@
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="n">
-        <v>17380</v>
+        <v>8092</v>
       </c>
     </row>
     <row r="48">
@@ -1778,10 +1772,10 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1079</v>
+        <v>1413</v>
       </c>
       <c r="C48" t="n">
-        <v>54</v>
+        <v>81</v>
       </c>
       <c r="D48" t="n">
         <v>80</v>
@@ -1789,11 +1783,9 @@
       <c r="E48" t="n">
         <v>2</v>
       </c>
-      <c r="F48" t="n">
-        <v>1</v>
-      </c>
+      <c r="F48" t="inlineStr"/>
       <c r="G48" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H48" t="n">
         <v>3</v>
@@ -1801,7 +1793,7 @@
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="n">
-        <v>1223</v>
+        <v>1584</v>
       </c>
     </row>
     <row r="49">
@@ -1811,13 +1803,13 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>7890</v>
+        <v>4918</v>
       </c>
       <c r="C49" t="n">
-        <v>3443</v>
+        <v>1824</v>
       </c>
       <c r="D49" t="n">
-        <v>142</v>
+        <v>88</v>
       </c>
       <c r="E49" t="n">
         <v>8</v>
@@ -1834,7 +1826,7 @@
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="n">
-        <v>11494</v>
+        <v>6849</v>
       </c>
     </row>
     <row r="50">
@@ -1844,18 +1836,20 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>1920</v>
+        <v>1788</v>
       </c>
       <c r="C50" t="n">
-        <v>429</v>
+        <v>89</v>
       </c>
       <c r="D50" t="n">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="E50" t="n">
-        <v>3</v>
-      </c>
-      <c r="F50" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="F50" t="n">
+        <v>1</v>
+      </c>
       <c r="G50" t="n">
         <v>3</v>
       </c>
@@ -1865,7 +1859,7 @@
       <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr"/>
       <c r="K50" t="n">
-        <v>2406</v>
+        <v>1930</v>
       </c>
     </row>
     <row r="51">
@@ -1875,20 +1869,18 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>3389</v>
+        <v>2105</v>
       </c>
       <c r="C51" t="n">
-        <v>1530</v>
+        <v>422</v>
       </c>
       <c r="D51" t="n">
-        <v>139</v>
+        <v>77</v>
       </c>
       <c r="E51" t="n">
         <v>1</v>
       </c>
-      <c r="F51" t="n">
-        <v>1</v>
-      </c>
+      <c r="F51" t="inlineStr"/>
       <c r="G51" t="n">
         <v>2</v>
       </c>
@@ -1900,7 +1892,7 @@
         <v>1</v>
       </c>
       <c r="K51" t="n">
-        <v>5064</v>
+        <v>2609</v>
       </c>
     </row>
     <row r="52">
@@ -1910,10 +1902,10 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>1490</v>
+        <v>1067</v>
       </c>
       <c r="C52" t="n">
-        <v>283</v>
+        <v>791</v>
       </c>
       <c r="D52" t="n">
         <v>4</v>
@@ -1937,7 +1929,7 @@
         <v>0</v>
       </c>
       <c r="K52" t="n">
-        <v>1777</v>
+        <v>1862</v>
       </c>
     </row>
     <row r="53">
@@ -1947,10 +1939,10 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>1490</v>
+        <v>1067</v>
       </c>
       <c r="C53" t="n">
-        <v>283</v>
+        <v>791</v>
       </c>
       <c r="D53" t="n">
         <v>4</v>
@@ -1962,7 +1954,7 @@
       <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr"/>
       <c r="K53" t="n">
-        <v>1777</v>
+        <v>1862</v>
       </c>
     </row>
     <row r="54">
@@ -1972,25 +1964,25 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>82245</v>
+        <v>61534</v>
       </c>
       <c r="C54" t="n">
-        <v>17069</v>
+        <v>13251</v>
       </c>
       <c r="D54" t="n">
-        <v>2072</v>
+        <v>1676</v>
       </c>
       <c r="E54" t="n">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="F54" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="G54" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="H54" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="I54" t="n">
         <v>0</v>
@@ -1999,7 +1991,7 @@
         <v>2</v>
       </c>
       <c r="K54" t="n">
-        <v>101625</v>
+        <v>76703</v>
       </c>
     </row>
   </sheetData>
@@ -2075,13 +2067,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2472</v>
+        <v>1696</v>
       </c>
       <c r="C2" t="n">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="D2" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -2099,7 +2091,7 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>2574</v>
+        <v>1805</v>
       </c>
     </row>
     <row r="3">
@@ -2109,10 +2101,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1396</v>
+        <v>1425</v>
       </c>
       <c r="C3" t="n">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="D3" t="n">
         <v>14</v>
@@ -2133,7 +2125,7 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>1444</v>
+        <v>1488</v>
       </c>
     </row>
     <row r="4">
@@ -2143,13 +2135,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>11725</v>
+        <v>6358</v>
       </c>
       <c r="C4" t="n">
-        <v>5701</v>
+        <v>2267</v>
       </c>
       <c r="D4" t="n">
-        <v>346</v>
+        <v>172</v>
       </c>
       <c r="E4" t="n">
         <v>2</v>
@@ -2167,7 +2159,7 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>17798</v>
+        <v>8823</v>
       </c>
     </row>
     <row r="5">
@@ -2177,19 +2169,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2385</v>
+        <v>2452</v>
       </c>
       <c r="C5" t="n">
-        <v>153</v>
+        <v>217</v>
       </c>
       <c r="D5" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E5" t="n">
         <v>7</v>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
         <v>2</v>
@@ -2201,7 +2193,7 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>2588</v>
+        <v>2719</v>
       </c>
     </row>
     <row r="6">
@@ -2211,13 +2203,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3897</v>
+        <v>1339</v>
       </c>
       <c r="C6" t="n">
-        <v>360</v>
+        <v>428</v>
       </c>
       <c r="D6" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
@@ -2235,7 +2227,7 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>4289</v>
+        <v>1798</v>
       </c>
     </row>
     <row r="7">
@@ -2245,13 +2237,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1171</v>
+        <v>1200</v>
       </c>
       <c r="C7" t="n">
-        <v>163</v>
+        <v>245</v>
       </c>
       <c r="D7" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E7" t="n">
         <v>1</v>
@@ -2269,7 +2261,7 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>1372</v>
+        <v>1481</v>
       </c>
     </row>
     <row r="8">
@@ -2279,10 +2271,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1169</v>
+        <v>975</v>
       </c>
       <c r="C8" t="n">
-        <v>64</v>
+        <v>107</v>
       </c>
       <c r="D8" t="n">
         <v>13</v>
@@ -2303,7 +2295,7 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>1248</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="9">
@@ -2313,10 +2305,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="C9" t="n">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="D9" t="n">
         <v>2</v>
@@ -2337,7 +2329,7 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>259</v>
+        <v>285</v>
       </c>
     </row>
     <row r="10">
@@ -2347,10 +2339,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C10" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D10" t="n">
         <v>1</v>
@@ -2371,7 +2363,7 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>43</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11">
@@ -2384,7 +2376,7 @@
         <v>446</v>
       </c>
       <c r="C11" t="n">
-        <v>89</v>
+        <v>140</v>
       </c>
       <c r="D11" t="n">
         <v>10</v>
@@ -2405,7 +2397,7 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>548</v>
+        <v>599</v>
       </c>
     </row>
     <row r="12">
@@ -2415,10 +2407,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1118</v>
+        <v>1433</v>
       </c>
       <c r="C12" t="n">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="D12" t="n">
         <v>86</v>
@@ -2427,10 +2419,10 @@
         <v>7</v>
       </c>
       <c r="F12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H12" t="n">
         <v>3</v>
@@ -2439,7 +2431,7 @@
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>1298</v>
+        <v>1641</v>
       </c>
     </row>
     <row r="13">
@@ -2452,10 +2444,10 @@
         <v>44</v>
       </c>
       <c r="C13" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
@@ -2473,7 +2465,7 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="14">
@@ -2483,13 +2475,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1103</v>
+        <v>881</v>
       </c>
       <c r="C14" t="n">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="D14" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
@@ -2507,7 +2499,7 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>1140</v>
+        <v>939</v>
       </c>
     </row>
     <row r="15">
@@ -2517,13 +2509,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>577</v>
+        <v>435</v>
       </c>
       <c r="C15" t="n">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="D15" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -2541,7 +2533,7 @@
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>653</v>
+        <v>517</v>
       </c>
     </row>
     <row r="16">
@@ -2551,16 +2543,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>374</v>
+        <v>483</v>
       </c>
       <c r="C16" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="D16" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
@@ -2575,7 +2567,7 @@
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>444</v>
+        <v>556</v>
       </c>
     </row>
     <row r="17">
@@ -2585,10 +2577,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C17" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
@@ -2619,10 +2611,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="C18" t="n">
-        <v>9</v>
+        <v>40</v>
       </c>
       <c r="D18" t="n">
         <v>1</v>
@@ -2643,7 +2635,7 @@
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>145</v>
+        <v>164</v>
       </c>
     </row>
     <row r="19">
@@ -2653,13 +2645,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>3183</v>
+        <v>2918</v>
       </c>
       <c r="C19" t="n">
-        <v>735</v>
+        <v>1314</v>
       </c>
       <c r="D19" t="n">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E19" t="n">
         <v>11</v>
@@ -2677,7 +2669,7 @@
         <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>4020</v>
+        <v>4331</v>
       </c>
     </row>
     <row r="20">
@@ -2687,10 +2679,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>406</v>
+        <v>249</v>
       </c>
       <c r="C20" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D20" t="n">
         <v>4</v>
@@ -2711,7 +2703,7 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>420</v>
+        <v>260</v>
       </c>
     </row>
     <row r="21">
@@ -2721,10 +2713,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="C21" t="n">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="D21" t="n">
         <v>7</v>
@@ -2745,7 +2737,7 @@
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>173</v>
+        <v>195</v>
       </c>
     </row>
     <row r="22">
@@ -2755,13 +2747,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>280</v>
+        <v>253</v>
       </c>
       <c r="C22" t="n">
-        <v>24</v>
+        <v>85</v>
       </c>
       <c r="D22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E22" t="n">
         <v>2</v>
@@ -2779,7 +2771,7 @@
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>310</v>
+        <v>343</v>
       </c>
     </row>
     <row r="23">
@@ -2789,13 +2781,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>293</v>
+        <v>264</v>
       </c>
       <c r="C23" t="n">
-        <v>19</v>
+        <v>79</v>
       </c>
       <c r="D23" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -2813,7 +2805,7 @@
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>319</v>
+        <v>348</v>
       </c>
     </row>
     <row r="24">
@@ -2823,13 +2815,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>391</v>
+        <v>362</v>
       </c>
       <c r="C24" t="n">
-        <v>39</v>
+        <v>87</v>
       </c>
       <c r="D24" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -2847,7 +2839,7 @@
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>445</v>
+        <v>461</v>
       </c>
     </row>
     <row r="25">
@@ -2857,14 +2849,14 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>273</v>
+        <v>210</v>
       </c>
       <c r="C25" t="n">
+        <v>22</v>
+      </c>
+      <c r="D25" t="n">
         <v>12</v>
       </c>
-      <c r="D25" t="n">
-        <v>13</v>
-      </c>
       <c r="E25" t="n">
         <v>1</v>
       </c>
@@ -2881,7 +2873,7 @@
         <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>299</v>
+        <v>245</v>
       </c>
     </row>
     <row r="26">
@@ -2891,16 +2883,16 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>6617</v>
+        <v>5661</v>
       </c>
       <c r="C26" t="n">
-        <v>837</v>
+        <v>1020</v>
       </c>
       <c r="D26" t="n">
-        <v>463</v>
+        <v>412</v>
       </c>
       <c r="E26" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F26" t="n">
         <v>4</v>
@@ -2915,7 +2907,7 @@
         <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>7943</v>
+        <v>7121</v>
       </c>
     </row>
     <row r="27">
@@ -2925,13 +2917,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1411</v>
+        <v>1350</v>
       </c>
       <c r="C27" t="n">
-        <v>432</v>
+        <v>608</v>
       </c>
       <c r="D27" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
@@ -2949,7 +2941,7 @@
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>1857</v>
+        <v>1974</v>
       </c>
     </row>
     <row r="28">
@@ -2959,13 +2951,13 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>2730</v>
+        <v>2027</v>
       </c>
       <c r="C28" t="n">
-        <v>321</v>
+        <v>877</v>
       </c>
       <c r="D28" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E28" t="n">
         <v>9</v>
@@ -2983,7 +2975,7 @@
         <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>3096</v>
+        <v>2947</v>
       </c>
     </row>
     <row r="29">
@@ -2993,10 +2985,10 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>124</v>
+        <v>172</v>
       </c>
       <c r="C29" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D29" t="n">
         <v>2</v>
@@ -3017,7 +3009,7 @@
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>144</v>
+        <v>191</v>
       </c>
     </row>
     <row r="30">
@@ -3027,10 +3019,10 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C30" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D30" t="n">
         <v>4</v>
@@ -3051,7 +3043,7 @@
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="31">
@@ -3061,13 +3053,13 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>7784</v>
+        <v>4753</v>
       </c>
       <c r="C31" t="n">
-        <v>3542</v>
+        <v>1882</v>
       </c>
       <c r="D31" t="n">
-        <v>156</v>
+        <v>101</v>
       </c>
       <c r="E31" t="n">
         <v>10</v>
@@ -3085,7 +3077,7 @@
         <v>0</v>
       </c>
       <c r="J31" t="n">
-        <v>11503</v>
+        <v>6757</v>
       </c>
     </row>
     <row r="32">
@@ -3095,10 +3087,10 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="C32" t="n">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="D32" t="n">
         <v>5</v>
@@ -3119,7 +3111,7 @@
         <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>147</v>
+        <v>161</v>
       </c>
     </row>
     <row r="33">
@@ -3129,10 +3121,10 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>343</v>
+        <v>293</v>
       </c>
       <c r="C33" t="n">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="D33" t="n">
         <v>14</v>
@@ -3153,7 +3145,7 @@
         <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>384</v>
+        <v>356</v>
       </c>
     </row>
     <row r="34">
@@ -3163,10 +3155,10 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C34" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="D34" t="n">
         <v>2</v>
@@ -3187,7 +3179,7 @@
         <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="35">
@@ -3197,10 +3189,10 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>250</v>
+        <v>211</v>
       </c>
       <c r="C35" t="n">
-        <v>13</v>
+        <v>79</v>
       </c>
       <c r="D35" t="n">
         <v>7</v>
@@ -3221,7 +3213,7 @@
         <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>270</v>
+        <v>297</v>
       </c>
     </row>
     <row r="36">
@@ -3231,31 +3223,31 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>857</v>
+        <v>458</v>
       </c>
       <c r="C36" t="n">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="D36" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E36" t="n">
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G36" t="n">
         <v>4</v>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>905</v>
+        <v>493</v>
       </c>
     </row>
     <row r="37">
@@ -3265,10 +3257,10 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C37" t="n">
-        <v>12</v>
+        <v>42</v>
       </c>
       <c r="D37" t="n">
         <v>3</v>
@@ -3289,7 +3281,7 @@
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>137</v>
+        <v>155</v>
       </c>
     </row>
     <row r="38">
@@ -3299,10 +3291,10 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>572</v>
+        <v>490</v>
       </c>
       <c r="C38" t="n">
-        <v>231</v>
+        <v>344</v>
       </c>
       <c r="D38" t="n">
         <v>4</v>
@@ -3323,7 +3315,7 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>808</v>
+        <v>839</v>
       </c>
     </row>
     <row r="39">
@@ -3333,10 +3325,10 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>205</v>
+        <v>192</v>
       </c>
       <c r="C39" t="n">
-        <v>19</v>
+        <v>48</v>
       </c>
       <c r="D39" t="n">
         <v>7</v>
@@ -3357,7 +3349,7 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>231</v>
+        <v>247</v>
       </c>
     </row>
     <row r="40">
@@ -3367,13 +3359,13 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>682</v>
+        <v>708</v>
       </c>
       <c r="C40" t="n">
-        <v>93</v>
+        <v>127</v>
       </c>
       <c r="D40" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E40" t="n">
         <v>0</v>
@@ -3391,7 +3383,7 @@
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>782</v>
+        <v>845</v>
       </c>
     </row>
     <row r="41">
@@ -3401,10 +3393,10 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>769</v>
+        <v>793</v>
       </c>
       <c r="C41" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="D41" t="n">
         <v>4</v>
@@ -3425,7 +3417,7 @@
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>804</v>
+        <v>835</v>
       </c>
     </row>
     <row r="42">
@@ -3435,10 +3427,10 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>661</v>
+        <v>222</v>
       </c>
       <c r="C42" t="n">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="D42" t="n">
         <v>3</v>
@@ -3459,7 +3451,7 @@
         <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>773</v>
+        <v>315</v>
       </c>
     </row>
     <row r="43">
@@ -3469,13 +3461,13 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>925</v>
+        <v>962</v>
       </c>
       <c r="C43" t="n">
-        <v>68</v>
+        <v>85</v>
       </c>
       <c r="D43" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E43" t="n">
         <v>1</v>
@@ -3493,7 +3485,7 @@
         <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>1008</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="44">
@@ -3503,10 +3495,10 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C44" t="n">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="D44" t="n">
         <v>10</v>
@@ -3527,7 +3519,7 @@
         <v>0</v>
       </c>
       <c r="J44" t="n">
-        <v>298</v>
+        <v>316</v>
       </c>
     </row>
     <row r="45">
@@ -3537,13 +3529,13 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>498</v>
+        <v>522</v>
       </c>
       <c r="C45" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D45" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E45" t="n">
         <v>0</v>
@@ -3561,7 +3553,7 @@
         <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>531</v>
+        <v>554</v>
       </c>
     </row>
     <row r="46">
@@ -3571,22 +3563,22 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>1611</v>
+        <v>924</v>
       </c>
       <c r="C46" t="n">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="D46" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E46" t="n">
         <v>3</v>
       </c>
       <c r="F46" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G46" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H46" t="n">
         <v>0</v>
@@ -3595,7 +3587,7 @@
         <v>0</v>
       </c>
       <c r="J46" t="n">
-        <v>1705</v>
+        <v>991</v>
       </c>
     </row>
     <row r="47">
@@ -3605,10 +3597,10 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="C47" t="n">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="D47" t="n">
         <v>4</v>
@@ -3629,7 +3621,7 @@
         <v>0</v>
       </c>
       <c r="J47" t="n">
-        <v>197</v>
+        <v>217</v>
       </c>
     </row>
     <row r="48">
@@ -3639,16 +3631,16 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1965</v>
+        <v>600</v>
       </c>
       <c r="C48" t="n">
-        <v>184</v>
+        <v>66</v>
       </c>
       <c r="D48" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F48" t="n">
         <v>0</v>
@@ -3663,7 +3655,7 @@
         <v>0</v>
       </c>
       <c r="J48" t="n">
-        <v>2174</v>
+        <v>690</v>
       </c>
     </row>
     <row r="49">
@@ -3673,16 +3665,16 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>237</v>
+        <v>195</v>
       </c>
       <c r="C49" t="n">
-        <v>23</v>
+        <v>92</v>
       </c>
       <c r="D49" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F49" t="n">
         <v>0</v>
@@ -3697,7 +3689,7 @@
         <v>0</v>
       </c>
       <c r="J49" t="n">
-        <v>267</v>
+        <v>290</v>
       </c>
     </row>
     <row r="50">
@@ -3707,13 +3699,13 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="C50" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D50" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E50" t="n">
         <v>0</v>
@@ -3731,7 +3723,7 @@
         <v>0</v>
       </c>
       <c r="J50" t="n">
-        <v>162</v>
+        <v>173</v>
       </c>
     </row>
     <row r="51">
@@ -3741,13 +3733,13 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>640</v>
+        <v>206</v>
       </c>
       <c r="C51" t="n">
-        <v>131</v>
+        <v>113</v>
       </c>
       <c r="D51" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E51" t="n">
         <v>1</v>
@@ -3765,7 +3757,7 @@
         <v>0</v>
       </c>
       <c r="J51" t="n">
-        <v>779</v>
+        <v>329</v>
       </c>
     </row>
     <row r="52">
@@ -3775,19 +3767,19 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>2388</v>
+        <v>2160</v>
       </c>
       <c r="C52" t="n">
-        <v>594</v>
+        <v>252</v>
       </c>
       <c r="D52" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="E52" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G52" t="n">
         <v>2</v>
@@ -3799,7 +3791,7 @@
         <v>0</v>
       </c>
       <c r="J52" t="n">
-        <v>3066</v>
+        <v>2466</v>
       </c>
     </row>
     <row r="53">
@@ -3809,16 +3801,16 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>1260</v>
+        <v>792</v>
       </c>
       <c r="C53" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D53" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="E53" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F53" t="n">
         <v>0</v>
@@ -3833,7 +3825,7 @@
         <v>0</v>
       </c>
       <c r="J53" t="n">
-        <v>1324</v>
+        <v>857</v>
       </c>
     </row>
     <row r="54">
@@ -3843,13 +3835,13 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C54" t="n">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="D54" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E54" t="n">
         <v>0</v>
@@ -3867,7 +3859,7 @@
         <v>0</v>
       </c>
       <c r="J54" t="n">
-        <v>98</v>
+        <v>108</v>
       </c>
     </row>
     <row r="55">
@@ -3877,19 +3869,19 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>3297</v>
+        <v>1987</v>
       </c>
       <c r="C55" t="n">
-        <v>1549</v>
+        <v>441</v>
       </c>
       <c r="D55" t="n">
-        <v>140</v>
+        <v>79</v>
       </c>
       <c r="E55" t="n">
         <v>1</v>
       </c>
       <c r="F55" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G55" t="n">
         <v>2</v>
@@ -3901,7 +3893,7 @@
         <v>2</v>
       </c>
       <c r="J55" t="n">
-        <v>4993</v>
+        <v>2513</v>
       </c>
     </row>
     <row r="56">
@@ -3911,13 +3903,13 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>357</v>
+        <v>271</v>
       </c>
       <c r="C56" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D56" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E56" t="n">
         <v>0</v>
@@ -3935,7 +3927,7 @@
         <v>0</v>
       </c>
       <c r="J56" t="n">
-        <v>403</v>
+        <v>320</v>
       </c>
     </row>
     <row r="57">
@@ -3948,10 +3940,10 @@
         <v>146</v>
       </c>
       <c r="C57" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="D57" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E57" t="n">
         <v>0</v>
@@ -3969,7 +3961,7 @@
         <v>0</v>
       </c>
       <c r="J57" t="n">
-        <v>161</v>
+        <v>174</v>
       </c>
     </row>
     <row r="58">
@@ -3979,13 +3971,13 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C58" t="n">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="D58" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E58" t="n">
         <v>0</v>
@@ -4003,7 +3995,7 @@
         <v>0</v>
       </c>
       <c r="J58" t="n">
-        <v>160</v>
+        <v>168</v>
       </c>
     </row>
     <row r="59">
@@ -4013,10 +4005,10 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>84</v>
+        <v>109</v>
       </c>
       <c r="C59" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D59" t="n">
         <v>6</v>
@@ -4037,7 +4029,7 @@
         <v>0</v>
       </c>
       <c r="J59" t="n">
-        <v>104</v>
+        <v>136</v>
       </c>
     </row>
     <row r="60">
@@ -4047,10 +4039,10 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>934</v>
+        <v>317</v>
       </c>
       <c r="C60" t="n">
-        <v>136</v>
+        <v>115</v>
       </c>
       <c r="D60" t="n">
         <v>7</v>
@@ -4071,7 +4063,7 @@
         <v>0</v>
       </c>
       <c r="J60" t="n">
-        <v>1078</v>
+        <v>440</v>
       </c>
     </row>
     <row r="61">
@@ -4081,19 +4073,19 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>2996</v>
+        <v>2941</v>
       </c>
       <c r="C61" t="n">
-        <v>398</v>
+        <v>581</v>
       </c>
       <c r="D61" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="E61" t="n">
         <v>2</v>
       </c>
       <c r="F61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G61" t="n">
         <v>0</v>
@@ -4105,7 +4097,7 @@
         <v>0</v>
       </c>
       <c r="J61" t="n">
-        <v>3413</v>
+        <v>3548</v>
       </c>
     </row>
     <row r="62">
@@ -4115,13 +4107,13 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>613</v>
+        <v>601</v>
       </c>
       <c r="C62" t="n">
-        <v>76</v>
+        <v>132</v>
       </c>
       <c r="D62" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="E62" t="n">
         <v>0</v>
@@ -4139,7 +4131,7 @@
         <v>0</v>
       </c>
       <c r="J62" t="n">
-        <v>707</v>
+        <v>759</v>
       </c>
     </row>
     <row r="63">
@@ -4149,13 +4141,13 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>4408</v>
+        <v>4714</v>
       </c>
       <c r="C63" t="n">
-        <v>85</v>
+        <v>147</v>
       </c>
       <c r="D63" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E63" t="n">
         <v>6</v>
@@ -4164,16 +4156,16 @@
         <v>1</v>
       </c>
       <c r="G63" t="n">
+        <v>1</v>
+      </c>
+      <c r="H63" t="n">
         <v>3</v>
       </c>
-      <c r="H63" t="n">
-        <v>1</v>
-      </c>
       <c r="I63" t="n">
         <v>0</v>
       </c>
       <c r="J63" t="n">
-        <v>4565</v>
+        <v>4932</v>
       </c>
     </row>
     <row r="64">
@@ -4183,16 +4175,16 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>2352</v>
+        <v>1512</v>
       </c>
       <c r="C64" t="n">
         <v>78</v>
       </c>
       <c r="D64" t="n">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="E64" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F64" t="n">
         <v>0</v>
@@ -4207,7 +4199,7 @@
         <v>0</v>
       </c>
       <c r="J64" t="n">
-        <v>2485</v>
+        <v>1641</v>
       </c>
     </row>
     <row r="65">
@@ -4217,31 +4209,31 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>82245</v>
+        <v>61534</v>
       </c>
       <c r="C65" t="n">
-        <v>17069</v>
+        <v>13251</v>
       </c>
       <c r="D65" t="n">
-        <v>2072</v>
+        <v>1676</v>
       </c>
       <c r="E65" t="n">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="F65" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="G65" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="H65" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="I65" t="n">
         <v>2</v>
       </c>
       <c r="J65" t="n">
-        <v>101625</v>
+        <v>76703</v>
       </c>
     </row>
   </sheetData>
@@ -4317,13 +4309,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>11660</v>
+        <v>6142</v>
       </c>
       <c r="C2" t="n">
-        <v>5359</v>
+        <v>1796</v>
       </c>
       <c r="D2" t="n">
-        <v>340</v>
+        <v>133</v>
       </c>
       <c r="E2" t="n">
         <v>3</v>
@@ -4341,7 +4333,7 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>17380</v>
+        <v>8092</v>
       </c>
     </row>
     <row r="3">
@@ -4351,10 +4343,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1079</v>
+        <v>1413</v>
       </c>
       <c r="C3" t="n">
-        <v>54</v>
+        <v>81</v>
       </c>
       <c r="D3" t="n">
         <v>80</v>
@@ -4363,10 +4355,10 @@
         <v>2</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H3" t="n">
         <v>3</v>
@@ -4375,7 +4367,7 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>1223</v>
+        <v>1584</v>
       </c>
     </row>
     <row r="4">
@@ -4385,16 +4377,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3120</v>
+        <v>3412</v>
       </c>
       <c r="C4" t="n">
-        <v>585</v>
+        <v>721</v>
       </c>
       <c r="D4" t="n">
-        <v>380</v>
+        <v>348</v>
       </c>
       <c r="E4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F4" t="n">
         <v>3</v>
@@ -4409,7 +4401,7 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>4105</v>
+        <v>4503</v>
       </c>
     </row>
     <row r="5">
@@ -4419,10 +4411,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>944</v>
+        <v>1012</v>
       </c>
       <c r="C5" t="n">
-        <v>46</v>
+        <v>79</v>
       </c>
       <c r="D5" t="n">
         <v>21</v>
@@ -4443,7 +4435,7 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>1016</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="6">
@@ -4453,16 +4445,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1912</v>
+        <v>547</v>
       </c>
       <c r="C6" t="n">
-        <v>184</v>
+        <v>66</v>
       </c>
       <c r="D6" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
@@ -4477,7 +4469,7 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>2118</v>
+        <v>634</v>
       </c>
     </row>
     <row r="7">
@@ -4487,19 +4479,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2129</v>
+        <v>2193</v>
       </c>
       <c r="C7" t="n">
-        <v>150</v>
+        <v>214</v>
       </c>
       <c r="D7" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>
       </c>
       <c r="F7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
         <v>2</v>
@@ -4511,7 +4503,7 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>2318</v>
+        <v>2446</v>
       </c>
     </row>
     <row r="8">
@@ -4521,13 +4513,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3848</v>
+        <v>1256</v>
       </c>
       <c r="C8" t="n">
-        <v>374</v>
+        <v>439</v>
       </c>
       <c r="D8" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
@@ -4545,7 +4537,7 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>4254</v>
+        <v>1726</v>
       </c>
     </row>
     <row r="9">
@@ -4555,13 +4547,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>923</v>
+        <v>961</v>
       </c>
       <c r="C9" t="n">
-        <v>60</v>
+        <v>82</v>
       </c>
       <c r="D9" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E9" t="n">
         <v>1</v>
@@ -4579,7 +4571,7 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>997</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="10">
@@ -4589,13 +4581,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>552</v>
+        <v>547</v>
       </c>
       <c r="C10" t="n">
-        <v>55</v>
+        <v>103</v>
       </c>
       <c r="D10" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -4613,7 +4605,7 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>622</v>
+        <v>674</v>
       </c>
     </row>
     <row r="11">
@@ -4623,13 +4615,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>5485</v>
+        <v>5877</v>
       </c>
       <c r="C11" t="n">
-        <v>110</v>
+        <v>183</v>
       </c>
       <c r="D11" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E11" t="n">
         <v>8</v>
@@ -4638,16 +4630,16 @@
         <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>5685</v>
+        <v>6149</v>
       </c>
     </row>
     <row r="12">
@@ -4660,7 +4652,7 @@
         <v>24</v>
       </c>
       <c r="C12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D12" t="n">
         <v>1</v>
@@ -4681,7 +4673,7 @@
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13">
@@ -4691,13 +4683,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="C13" t="n">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
@@ -4715,7 +4707,7 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="14">
@@ -4725,10 +4717,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="C14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D14" t="n">
         <v>1</v>
@@ -4749,7 +4741,7 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
     </row>
     <row r="15">
@@ -4759,13 +4751,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>58</v>
+        <v>3</v>
       </c>
       <c r="C15" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -4783,7 +4775,7 @@
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>178</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16">
@@ -4793,7 +4785,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C16" t="n">
         <v>13</v>
@@ -4817,7 +4809,7 @@
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="17">
@@ -4827,10 +4819,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>76</v>
+        <v>65</v>
       </c>
       <c r="C17" t="n">
-        <v>43</v>
+        <v>57</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
@@ -4851,7 +4843,7 @@
         <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
     <row r="18">
@@ -4861,13 +4853,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>68</v>
+        <v>9</v>
       </c>
       <c r="C18" t="n">
-        <v>83</v>
+        <v>7</v>
       </c>
       <c r="D18" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
@@ -4885,7 +4877,7 @@
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>158</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19">
@@ -4898,7 +4890,7 @@
         <v>5</v>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D19" t="n">
         <v>2</v>
@@ -4919,7 +4911,7 @@
         <v>1</v>
       </c>
       <c r="J19" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20">
@@ -4929,13 +4921,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>56</v>
+        <v>13</v>
       </c>
       <c r="C20" t="n">
-        <v>74</v>
+        <v>3</v>
       </c>
       <c r="D20" t="n">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
@@ -4953,7 +4945,7 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>157</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21">
@@ -4963,10 +4955,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D21" t="n">
         <v>1</v>
@@ -4987,7 +4979,7 @@
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>31</v>
+        <v>36</v>
       </c>
     </row>
     <row r="22">
@@ -4997,13 +4989,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="C22" t="n">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="D22" t="n">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
@@ -5021,7 +5013,7 @@
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>175</v>
+        <v>180</v>
       </c>
     </row>
     <row r="23">
@@ -5031,13 +5023,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>221</v>
+        <v>193</v>
       </c>
       <c r="C23" t="n">
-        <v>216</v>
+        <v>253</v>
       </c>
       <c r="D23" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -5055,7 +5047,7 @@
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>443</v>
+        <v>454</v>
       </c>
     </row>
     <row r="24">
@@ -5065,13 +5057,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>386</v>
+        <v>375</v>
       </c>
       <c r="C24" t="n">
-        <v>91</v>
+        <v>137</v>
       </c>
       <c r="D24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -5089,7 +5081,7 @@
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>481</v>
+        <v>515</v>
       </c>
     </row>
     <row r="25">
@@ -5099,13 +5091,13 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="C25" t="n">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="D25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
@@ -5123,7 +5115,7 @@
         <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>128</v>
+        <v>132</v>
       </c>
     </row>
     <row r="26">
@@ -5133,10 +5125,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>822</v>
+        <v>406</v>
       </c>
       <c r="C26" t="n">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="D26" t="n">
         <v>12</v>
@@ -5148,16 +5140,16 @@
         <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I26" t="n">
         <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>868</v>
+        <v>440</v>
       </c>
     </row>
     <row r="27">
@@ -5167,13 +5159,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1894</v>
+        <v>1948</v>
       </c>
       <c r="C27" t="n">
-        <v>257</v>
+        <v>374</v>
       </c>
       <c r="D27" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="E27" t="n">
         <v>1</v>
@@ -5191,7 +5183,7 @@
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>2190</v>
+        <v>2365</v>
       </c>
     </row>
     <row r="28">
@@ -5201,22 +5193,22 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>8937</v>
+        <v>5565</v>
       </c>
       <c r="C28" t="n">
-        <v>379</v>
+        <v>415</v>
       </c>
       <c r="D28" t="n">
-        <v>132</v>
+        <v>116</v>
       </c>
       <c r="E28" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F28" t="n">
         <v>4</v>
       </c>
       <c r="G28" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H28" t="n">
         <v>5</v>
@@ -5225,7 +5217,7 @@
         <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>9479</v>
+        <v>6129</v>
       </c>
     </row>
     <row r="29">
@@ -5235,10 +5227,10 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1400</v>
+        <v>1084</v>
       </c>
       <c r="C29" t="n">
-        <v>715</v>
+        <v>1104</v>
       </c>
       <c r="D29" t="n">
         <v>37</v>
@@ -5259,7 +5251,7 @@
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>2155</v>
+        <v>2228</v>
       </c>
     </row>
     <row r="30">
@@ -5269,16 +5261,16 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>500</v>
+        <v>644</v>
       </c>
       <c r="C30" t="n">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D30" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F30" t="n">
         <v>0</v>
@@ -5293,7 +5285,7 @@
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>583</v>
+        <v>731</v>
       </c>
     </row>
     <row r="31">
@@ -5303,10 +5295,10 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>3859</v>
+        <v>4197</v>
       </c>
       <c r="C31" t="n">
-        <v>238</v>
+        <v>596</v>
       </c>
       <c r="D31" t="n">
         <v>116</v>
@@ -5315,7 +5307,7 @@
         <v>22</v>
       </c>
       <c r="F31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G31" t="n">
         <v>2</v>
@@ -5327,7 +5319,7 @@
         <v>0</v>
       </c>
       <c r="J31" t="n">
-        <v>4238</v>
+        <v>4933</v>
       </c>
     </row>
     <row r="32">
@@ -5337,16 +5329,16 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>3088</v>
+        <v>2941</v>
       </c>
       <c r="C32" t="n">
-        <v>210</v>
+        <v>734</v>
       </c>
       <c r="D32" t="n">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="E32" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F32" t="n">
         <v>3</v>
@@ -5361,7 +5353,7 @@
         <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>3370</v>
+        <v>3744</v>
       </c>
     </row>
     <row r="33">
@@ -5371,22 +5363,22 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>5649</v>
+        <v>3658</v>
       </c>
       <c r="C33" t="n">
-        <v>149</v>
+        <v>339</v>
       </c>
       <c r="D33" t="n">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E33" t="n">
         <v>10</v>
       </c>
       <c r="F33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G33" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H33" t="n">
         <v>2</v>
@@ -5395,7 +5387,7 @@
         <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>5994</v>
+        <v>4194</v>
       </c>
     </row>
     <row r="34">
@@ -5405,13 +5397,13 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1950</v>
+        <v>1825</v>
       </c>
       <c r="C34" t="n">
-        <v>649</v>
+        <v>942</v>
       </c>
       <c r="D34" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E34" t="n">
         <v>1</v>
@@ -5429,7 +5421,7 @@
         <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>2618</v>
+        <v>2788</v>
       </c>
     </row>
     <row r="35">
@@ -5439,13 +5431,13 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1275</v>
+        <v>1325</v>
       </c>
       <c r="C35" t="n">
-        <v>52</v>
+        <v>65</v>
       </c>
       <c r="D35" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E35" t="n">
         <v>0</v>
@@ -5463,7 +5455,7 @@
         <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>1338</v>
+        <v>1399</v>
       </c>
     </row>
     <row r="36">
@@ -5473,13 +5465,13 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>2264</v>
+        <v>736</v>
       </c>
       <c r="C36" t="n">
-        <v>345</v>
+        <v>306</v>
       </c>
       <c r="D36" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E36" t="n">
         <v>0</v>
@@ -5497,7 +5489,7 @@
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>2626</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="37">
@@ -5507,19 +5499,19 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>3081</v>
+        <v>3020</v>
       </c>
       <c r="C37" t="n">
-        <v>417</v>
+        <v>608</v>
       </c>
       <c r="D37" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E37" t="n">
         <v>2</v>
       </c>
       <c r="F37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G37" t="n">
         <v>0</v>
@@ -5531,7 +5523,7 @@
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>3517</v>
+        <v>3656</v>
       </c>
     </row>
     <row r="38">
@@ -5541,13 +5533,13 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>7890</v>
+        <v>4918</v>
       </c>
       <c r="C38" t="n">
-        <v>3443</v>
+        <v>1824</v>
       </c>
       <c r="D38" t="n">
-        <v>142</v>
+        <v>88</v>
       </c>
       <c r="E38" t="n">
         <v>8</v>
@@ -5565,7 +5557,7 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>11494</v>
+        <v>6849</v>
       </c>
     </row>
     <row r="39">
@@ -5575,10 +5567,10 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1490</v>
+        <v>1067</v>
       </c>
       <c r="C39" t="n">
-        <v>283</v>
+        <v>791</v>
       </c>
       <c r="D39" t="n">
         <v>4</v>
@@ -5599,7 +5591,7 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>1777</v>
+        <v>1862</v>
       </c>
     </row>
     <row r="40">
@@ -5609,19 +5601,19 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1920</v>
+        <v>1788</v>
       </c>
       <c r="C40" t="n">
-        <v>429</v>
+        <v>89</v>
       </c>
       <c r="D40" t="n">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="E40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G40" t="n">
         <v>3</v>
@@ -5633,7 +5625,7 @@
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>2406</v>
+        <v>1930</v>
       </c>
     </row>
     <row r="41">
@@ -5643,19 +5635,19 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>3389</v>
+        <v>2105</v>
       </c>
       <c r="C41" t="n">
-        <v>1530</v>
+        <v>422</v>
       </c>
       <c r="D41" t="n">
-        <v>139</v>
+        <v>77</v>
       </c>
       <c r="E41" t="n">
         <v>1</v>
       </c>
       <c r="F41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G41" t="n">
         <v>2</v>
@@ -5667,7 +5659,7 @@
         <v>1</v>
       </c>
       <c r="J41" t="n">
-        <v>5064</v>
+        <v>2609</v>
       </c>
     </row>
     <row r="42">
@@ -5677,31 +5669,31 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>82245</v>
+        <v>61534</v>
       </c>
       <c r="C42" t="n">
-        <v>17069</v>
+        <v>13251</v>
       </c>
       <c r="D42" t="n">
-        <v>2072</v>
+        <v>1676</v>
       </c>
       <c r="E42" t="n">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="F42" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="G42" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="H42" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="I42" t="n">
         <v>2</v>
       </c>
       <c r="J42" t="n">
-        <v>101625</v>
+        <v>76703</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: capture and print subprocess output to debug export_tonkho_v2.py silent failure in cron
</commit_message>
<xml_diff>
--- a/BaoCao_TonKho.xlsx
+++ b/BaoCao_TonKho.xlsx
@@ -443,7 +443,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>16/06/2026 20:33:45</t>
+          <t>17/06/2026 03:40:32</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -567,13 +567,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>9380</v>
+        <v>9419</v>
       </c>
       <c r="C7" t="n">
-        <v>1126</v>
+        <v>1088</v>
       </c>
       <c r="D7" t="n">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E7" t="n">
         <v>94</v>
@@ -604,10 +604,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>993</v>
+        <v>1005</v>
       </c>
       <c r="C8" t="n">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="D8" t="n">
         <v>84</v>
@@ -633,10 +633,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1954</v>
+        <v>1955</v>
       </c>
       <c r="C9" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D9" t="n">
         <v>14</v>
@@ -666,10 +666,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1339</v>
+        <v>1350</v>
       </c>
       <c r="C10" t="n">
-        <v>163</v>
+        <v>152</v>
       </c>
       <c r="D10" t="n">
         <v>16</v>
@@ -695,10 +695,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1628</v>
+        <v>1639</v>
       </c>
       <c r="C11" t="n">
-        <v>506</v>
+        <v>495</v>
       </c>
       <c r="D11" t="n">
         <v>9</v>
@@ -726,10 +726,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>749</v>
+        <v>752</v>
       </c>
       <c r="C12" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D12" t="n">
         <v>5</v>
@@ -753,13 +753,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2717</v>
+        <v>2718</v>
       </c>
       <c r="C13" t="n">
         <v>283</v>
       </c>
       <c r="D13" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E13" t="n">
         <v>49</v>
@@ -786,10 +786,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1064</v>
+        <v>1075</v>
       </c>
       <c r="C14" t="n">
-        <v>1113</v>
+        <v>1102</v>
       </c>
       <c r="D14" t="n">
         <v>80</v>
@@ -823,10 +823,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C15" t="n">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D15" t="n">
         <v>1</v>
@@ -848,10 +848,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C16" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D16" t="n">
         <v>1</v>
@@ -929,10 +929,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C19" t="n">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D19" t="n">
         <v>7</v>
@@ -956,10 +956,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C20" t="n">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D20" t="n">
         <v>13</v>
@@ -1008,10 +1008,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C22" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D22" t="n">
         <v>7</v>
@@ -1066,10 +1066,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C24" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D24" t="n">
         <v>4</v>
@@ -1151,10 +1151,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C27" t="n">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D27" t="n">
         <v>12</v>
@@ -1273,16 +1273,16 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>27257</v>
+        <v>27300</v>
       </c>
       <c r="C31" t="n">
-        <v>2435</v>
+        <v>2402</v>
       </c>
       <c r="D31" t="n">
-        <v>1141</v>
+        <v>1132</v>
       </c>
       <c r="E31" t="n">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F31" t="n">
         <v>94</v>
@@ -1310,13 +1310,13 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1544</v>
+        <v>1547</v>
       </c>
       <c r="C32" t="n">
-        <v>356</v>
+        <v>362</v>
       </c>
       <c r="D32" t="n">
-        <v>347</v>
+        <v>338</v>
       </c>
       <c r="E32" t="n">
         <v>10</v>
@@ -1343,10 +1343,10 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>2701</v>
+        <v>2707</v>
       </c>
       <c r="C33" t="n">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="D33" t="n">
         <v>11</v>
@@ -1374,10 +1374,10 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>5050</v>
+        <v>5052</v>
       </c>
       <c r="C34" t="n">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D34" t="n">
         <v>87</v>
@@ -1407,10 +1407,10 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1536</v>
+        <v>1540</v>
       </c>
       <c r="C35" t="n">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="D35" t="n">
         <v>43</v>
@@ -1440,10 +1440,10 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>802</v>
+        <v>804</v>
       </c>
       <c r="C36" t="n">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D36" t="n">
         <v>12</v>
@@ -1475,10 +1475,10 @@
         <v>426</v>
       </c>
       <c r="D37" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E37" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F37" t="n">
         <v>5</v>
@@ -1502,10 +1502,10 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>2781</v>
+        <v>2782</v>
       </c>
       <c r="C38" t="n">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="D38" t="n">
         <v>123</v>
@@ -1533,10 +1533,10 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>3852</v>
+        <v>3854</v>
       </c>
       <c r="C39" t="n">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D39" t="n">
         <v>49</v>
@@ -1566,13 +1566,13 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>2038</v>
+        <v>2042</v>
       </c>
       <c r="C40" t="n">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="D40" t="n">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E40" t="n">
         <v>45</v>
@@ -1595,10 +1595,10 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="C41" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D41" t="n">
         <v>72</v>
@@ -1626,10 +1626,10 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1969</v>
+        <v>1980</v>
       </c>
       <c r="C42" t="n">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="D42" t="n">
         <v>50</v>
@@ -1657,10 +1657,10 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>1979</v>
+        <v>1986</v>
       </c>
       <c r="C43" t="n">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="D43" t="n">
         <v>42</v>
@@ -1688,13 +1688,13 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>1970</v>
+        <v>1980</v>
       </c>
       <c r="C44" t="n">
-        <v>856</v>
+        <v>847</v>
       </c>
       <c r="D44" t="n">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="E44" t="n">
         <v>44</v>
@@ -1725,13 +1725,13 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>1970</v>
+        <v>1980</v>
       </c>
       <c r="C45" t="n">
-        <v>856</v>
+        <v>847</v>
       </c>
       <c r="D45" t="n">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="E45" t="n">
         <v>44</v>
@@ -1756,13 +1756,13 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>30333</v>
+        <v>30526</v>
       </c>
       <c r="C46" t="n">
-        <v>14010</v>
+        <v>13869</v>
       </c>
       <c r="D46" t="n">
-        <v>851</v>
+        <v>799</v>
       </c>
       <c r="E46" t="n">
         <v>66</v>
@@ -1793,13 +1793,13 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>10336</v>
+        <v>10402</v>
       </c>
       <c r="C47" t="n">
-        <v>4802</v>
+        <v>4749</v>
       </c>
       <c r="D47" t="n">
-        <v>220</v>
+        <v>207</v>
       </c>
       <c r="E47" t="n">
         <v>23</v>
@@ -1826,13 +1826,13 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>3514</v>
+        <v>3534</v>
       </c>
       <c r="C48" t="n">
-        <v>1493</v>
+        <v>1483</v>
       </c>
       <c r="D48" t="n">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="E48" t="n">
         <v>6</v>
@@ -1861,13 +1861,13 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>6864</v>
+        <v>6913</v>
       </c>
       <c r="C49" t="n">
-        <v>3212</v>
+        <v>3168</v>
       </c>
       <c r="D49" t="n">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="E49" t="n">
         <v>10</v>
@@ -1894,13 +1894,13 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>4232</v>
+        <v>4257</v>
       </c>
       <c r="C50" t="n">
-        <v>1832</v>
+        <v>1813</v>
       </c>
       <c r="D50" t="n">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="E50" t="n">
         <v>19</v>
@@ -1927,13 +1927,13 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>5387</v>
+        <v>5420</v>
       </c>
       <c r="C51" t="n">
-        <v>2671</v>
+        <v>2656</v>
       </c>
       <c r="D51" t="n">
-        <v>150</v>
+        <v>132</v>
       </c>
       <c r="E51" t="n">
         <v>8</v>
@@ -1960,10 +1960,10 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>919</v>
+        <v>920</v>
       </c>
       <c r="C52" t="n">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D52" t="n">
         <v>9</v>
@@ -1997,10 +1997,10 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>919</v>
+        <v>920</v>
       </c>
       <c r="C53" t="n">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D53" t="n">
         <v>9</v>
@@ -2026,16 +2026,16 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>71723</v>
+        <v>72020</v>
       </c>
       <c r="C54" t="n">
-        <v>19779</v>
+        <v>19546</v>
       </c>
       <c r="D54" t="n">
-        <v>2956</v>
+        <v>2893</v>
       </c>
       <c r="E54" t="n">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="F54" t="n">
         <v>239</v>
@@ -2134,10 +2134,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1230</v>
+        <v>1232</v>
       </c>
       <c r="C2" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D2" t="n">
         <v>25</v>
@@ -2171,10 +2171,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>993</v>
+        <v>994</v>
       </c>
       <c r="C3" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D3" t="n">
         <v>21</v>
@@ -2208,13 +2208,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10326</v>
+        <v>10398</v>
       </c>
       <c r="C4" t="n">
-        <v>5139</v>
+        <v>5079</v>
       </c>
       <c r="D4" t="n">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="E4" t="n">
         <v>26</v>
@@ -2245,13 +2245,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2555</v>
+        <v>2557</v>
       </c>
       <c r="C5" t="n">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D5" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E5" t="n">
         <v>6</v>
@@ -2282,10 +2282,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1312</v>
+        <v>1322</v>
       </c>
       <c r="C6" t="n">
-        <v>163</v>
+        <v>153</v>
       </c>
       <c r="D6" t="n">
         <v>18</v>
@@ -2319,10 +2319,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1661</v>
+        <v>1664</v>
       </c>
       <c r="C7" t="n">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D7" t="n">
         <v>8</v>
@@ -2504,13 +2504,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3589</v>
+        <v>3611</v>
       </c>
       <c r="C12" t="n">
-        <v>1539</v>
+        <v>1527</v>
       </c>
       <c r="D12" t="n">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="E12" t="n">
         <v>9</v>
@@ -2652,10 +2652,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="C16" t="n">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D16" t="n">
         <v>18</v>
@@ -2763,10 +2763,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2140</v>
+        <v>2143</v>
       </c>
       <c r="C19" t="n">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="D19" t="n">
         <v>97</v>
@@ -2800,13 +2800,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="C20" t="n">
         <v>117</v>
       </c>
       <c r="D20" t="n">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E20" t="n">
         <v>1</v>
@@ -2874,10 +2874,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C22" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D22" t="n">
         <v>7</v>
@@ -3022,13 +3022,13 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>4188</v>
+        <v>4202</v>
       </c>
       <c r="C26" t="n">
-        <v>1182</v>
+        <v>1169</v>
       </c>
       <c r="D26" t="n">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="E26" t="n">
         <v>47</v>
@@ -3059,13 +3059,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1569</v>
+        <v>1573</v>
       </c>
       <c r="C27" t="n">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="D27" t="n">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E27" t="n">
         <v>32</v>
@@ -3096,10 +3096,10 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>2479</v>
+        <v>2480</v>
       </c>
       <c r="C28" t="n">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D28" t="n">
         <v>20</v>
@@ -3207,13 +3207,13 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>6247</v>
+        <v>6292</v>
       </c>
       <c r="C31" t="n">
-        <v>2997</v>
+        <v>2956</v>
       </c>
       <c r="D31" t="n">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="E31" t="n">
         <v>21</v>
@@ -3392,13 +3392,13 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1310</v>
+        <v>1312</v>
       </c>
       <c r="C36" t="n">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="D36" t="n">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="E36" t="n">
         <v>11</v>
@@ -3429,10 +3429,10 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C37" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D37" t="n">
         <v>8</v>
@@ -3466,10 +3466,10 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="C38" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D38" t="n">
         <v>27</v>
@@ -3540,10 +3540,10 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>985</v>
+        <v>987</v>
       </c>
       <c r="C40" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D40" t="n">
         <v>10</v>
@@ -3577,10 +3577,10 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C41" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D41" t="n">
         <v>35</v>
@@ -3614,10 +3614,10 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>545</v>
+        <v>548</v>
       </c>
       <c r="C42" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D42" t="n">
         <v>17</v>
@@ -3651,10 +3651,10 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>1656</v>
+        <v>1667</v>
       </c>
       <c r="C43" t="n">
-        <v>509</v>
+        <v>498</v>
       </c>
       <c r="D43" t="n">
         <v>9</v>
@@ -3836,10 +3836,10 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>994</v>
+        <v>1006</v>
       </c>
       <c r="C48" t="n">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="D48" t="n">
         <v>85</v>
@@ -3947,10 +3947,10 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>594</v>
+        <v>597</v>
       </c>
       <c r="C51" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D51" t="n">
         <v>13</v>
@@ -3984,13 +3984,13 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>5208</v>
+        <v>5238</v>
       </c>
       <c r="C52" t="n">
-        <v>2264</v>
+        <v>2238</v>
       </c>
       <c r="D52" t="n">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="E52" t="n">
         <v>45</v>
@@ -4095,13 +4095,13 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>4886</v>
+        <v>4918</v>
       </c>
       <c r="C55" t="n">
-        <v>2613</v>
+        <v>2599</v>
       </c>
       <c r="D55" t="n">
-        <v>141</v>
+        <v>123</v>
       </c>
       <c r="E55" t="n">
         <v>8</v>
@@ -4249,10 +4249,10 @@
         <v>20</v>
       </c>
       <c r="D59" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E59" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F59" t="n">
         <v>2</v>
@@ -4280,10 +4280,10 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>795</v>
+        <v>800</v>
       </c>
       <c r="C60" t="n">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D60" t="n">
         <v>26</v>
@@ -4317,10 +4317,10 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>1932</v>
+        <v>1938</v>
       </c>
       <c r="C61" t="n">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="D61" t="n">
         <v>44</v>
@@ -4354,10 +4354,10 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>803</v>
+        <v>807</v>
       </c>
       <c r="C62" t="n">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="D62" t="n">
         <v>5</v>
@@ -4394,10 +4394,10 @@
         <v>2081</v>
       </c>
       <c r="C63" t="n">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D63" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E63" t="n">
         <v>42</v>
@@ -4428,13 +4428,13 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>1480</v>
+        <v>1481</v>
       </c>
       <c r="C64" t="n">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="D64" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E64" t="n">
         <v>5</v>
@@ -4465,16 +4465,16 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>71723</v>
+        <v>72020</v>
       </c>
       <c r="C65" t="n">
-        <v>19779</v>
+        <v>19546</v>
       </c>
       <c r="D65" t="n">
-        <v>2956</v>
+        <v>2893</v>
       </c>
       <c r="E65" t="n">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="F65" t="n">
         <v>239</v>
@@ -4573,13 +4573,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>10336</v>
+        <v>10402</v>
       </c>
       <c r="C2" t="n">
-        <v>4802</v>
+        <v>4749</v>
       </c>
       <c r="D2" t="n">
-        <v>220</v>
+        <v>207</v>
       </c>
       <c r="E2" t="n">
         <v>23</v>
@@ -4610,13 +4610,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3514</v>
+        <v>3534</v>
       </c>
       <c r="C3" t="n">
-        <v>1493</v>
+        <v>1483</v>
       </c>
       <c r="D3" t="n">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="E3" t="n">
         <v>6</v>
@@ -4647,13 +4647,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1970</v>
+        <v>1980</v>
       </c>
       <c r="C4" t="n">
-        <v>856</v>
+        <v>847</v>
       </c>
       <c r="D4" t="n">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="E4" t="n">
         <v>44</v>
@@ -4721,10 +4721,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>993</v>
+        <v>1005</v>
       </c>
       <c r="C6" t="n">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="D6" t="n">
         <v>84</v>
@@ -4758,10 +4758,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1954</v>
+        <v>1955</v>
       </c>
       <c r="C7" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D7" t="n">
         <v>14</v>
@@ -4795,10 +4795,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1339</v>
+        <v>1350</v>
       </c>
       <c r="C8" t="n">
-        <v>163</v>
+        <v>152</v>
       </c>
       <c r="D8" t="n">
         <v>16</v>
@@ -4832,10 +4832,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1628</v>
+        <v>1639</v>
       </c>
       <c r="C9" t="n">
-        <v>506</v>
+        <v>495</v>
       </c>
       <c r="D9" t="n">
         <v>9</v>
@@ -4869,10 +4869,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>749</v>
+        <v>752</v>
       </c>
       <c r="C10" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D10" t="n">
         <v>5</v>
@@ -4906,13 +4906,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2717</v>
+        <v>2718</v>
       </c>
       <c r="C11" t="n">
         <v>283</v>
       </c>
       <c r="D11" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E11" t="n">
         <v>49</v>
@@ -4943,10 +4943,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C12" t="n">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D12" t="n">
         <v>1</v>
@@ -4980,10 +4980,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C13" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D13" t="n">
         <v>1</v>
@@ -5091,10 +5091,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C16" t="n">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D16" t="n">
         <v>7</v>
@@ -5128,10 +5128,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C17" t="n">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D17" t="n">
         <v>13</v>
@@ -5202,10 +5202,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C19" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D19" t="n">
         <v>7</v>
@@ -5276,10 +5276,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C21" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D21" t="n">
         <v>4</v>
@@ -5387,10 +5387,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C24" t="n">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D24" t="n">
         <v>12</v>
@@ -5461,13 +5461,13 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1544</v>
+        <v>1547</v>
       </c>
       <c r="C26" t="n">
-        <v>356</v>
+        <v>362</v>
       </c>
       <c r="D26" t="n">
-        <v>347</v>
+        <v>338</v>
       </c>
       <c r="E26" t="n">
         <v>10</v>
@@ -5498,10 +5498,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2701</v>
+        <v>2707</v>
       </c>
       <c r="C27" t="n">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="D27" t="n">
         <v>11</v>
@@ -5535,10 +5535,10 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>5050</v>
+        <v>5052</v>
       </c>
       <c r="C28" t="n">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D28" t="n">
         <v>87</v>
@@ -5572,10 +5572,10 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1536</v>
+        <v>1540</v>
       </c>
       <c r="C29" t="n">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="D29" t="n">
         <v>43</v>
@@ -5609,10 +5609,10 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>802</v>
+        <v>804</v>
       </c>
       <c r="C30" t="n">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D30" t="n">
         <v>12</v>
@@ -5652,10 +5652,10 @@
         <v>426</v>
       </c>
       <c r="D31" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E31" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F31" t="n">
         <v>5</v>
@@ -5683,10 +5683,10 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>2781</v>
+        <v>2782</v>
       </c>
       <c r="C32" t="n">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="D32" t="n">
         <v>123</v>
@@ -5720,10 +5720,10 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>3852</v>
+        <v>3854</v>
       </c>
       <c r="C33" t="n">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D33" t="n">
         <v>49</v>
@@ -5757,13 +5757,13 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>2038</v>
+        <v>2042</v>
       </c>
       <c r="C34" t="n">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="D34" t="n">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E34" t="n">
         <v>45</v>
@@ -5794,10 +5794,10 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="C35" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D35" t="n">
         <v>72</v>
@@ -5831,10 +5831,10 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1969</v>
+        <v>1980</v>
       </c>
       <c r="C36" t="n">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="D36" t="n">
         <v>50</v>
@@ -5868,10 +5868,10 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1979</v>
+        <v>1986</v>
       </c>
       <c r="C37" t="n">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="D37" t="n">
         <v>42</v>
@@ -5905,13 +5905,13 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>6864</v>
+        <v>6913</v>
       </c>
       <c r="C38" t="n">
-        <v>3212</v>
+        <v>3168</v>
       </c>
       <c r="D38" t="n">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="E38" t="n">
         <v>10</v>
@@ -5942,10 +5942,10 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>919</v>
+        <v>920</v>
       </c>
       <c r="C39" t="n">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D39" t="n">
         <v>9</v>
@@ -5979,13 +5979,13 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>4232</v>
+        <v>4257</v>
       </c>
       <c r="C40" t="n">
-        <v>1832</v>
+        <v>1813</v>
       </c>
       <c r="D40" t="n">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="E40" t="n">
         <v>19</v>
@@ -6016,13 +6016,13 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>5387</v>
+        <v>5420</v>
       </c>
       <c r="C41" t="n">
-        <v>2671</v>
+        <v>2656</v>
       </c>
       <c r="D41" t="n">
-        <v>150</v>
+        <v>132</v>
       </c>
       <c r="E41" t="n">
         <v>8</v>
@@ -6053,16 +6053,16 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>71723</v>
+        <v>72020</v>
       </c>
       <c r="C42" t="n">
-        <v>19779</v>
+        <v>19546</v>
       </c>
       <c r="D42" t="n">
-        <v>2956</v>
+        <v>2893</v>
       </c>
       <c r="E42" t="n">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="F42" t="n">
         <v>239</v>

</xml_diff>